<commit_message>
Update GEMM performance comparison workflow
</commit_message>
<xml_diff>
--- a/gemm_performance_comparison.xlsx
+++ b/gemm_performance_comparison.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="环境对比" sheetId="1" r:id="R87dc70e1d30f46a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="环境对比" sheetId="1" r:id="R4edfec29e10f4859"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -46,7 +46,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="15">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -76,6 +76,46 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFFDF2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDDEBF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF4472C4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFBF9000"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC65911"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF548235"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -115,7 +155,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="24">
+  <x:cellXfs count="53">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -162,6 +202,67 @@
     <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -173,7 +274,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -183,7 +284,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -410,11 +511,15 @@
     <x:col min="3" max="3" width="10" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="25" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="25" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="30" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="30" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="21" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="28" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="21" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="21" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="21" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="28" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -451,21 +556,33 @@
         <x:v>128, 256, 512, 1024, 2048</x:v>
       </x:c>
       <x:c r="G2" s="9" t="str">
-        <x:v>结果来源</x:v>
+        <x:v>CUTLASS来源</x:v>
       </x:c>
       <x:c r="H2" s="9" t="str">
-        <x:v>collect_gemm_results.py</x:v>
+        <x:v>脚本自动回填</x:v>
       </x:c>
       <x:c r="I2" s="9" t="str">
+        <x:v>HGEMM（自研）</x:v>
+      </x:c>
+      <x:c r="J2" s="10" t="str">
+        <x:v>人工筛选</x:v>
+      </x:c>
+      <x:c r="K2" t="str">
+        <x:v>HGEMM（CUDA）</x:v>
+      </x:c>
+      <x:c r="L2" t="str">
+        <x:v>人工筛选</x:v>
+      </x:c>
+      <x:c r="M2" t="str">
         <x:v>加速比</x:v>
       </x:c>
-      <x:c r="J2" s="10" t="str">
-        <x:v>自研 GFLOPS / 原生 GFLOPS</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="28" customHeight="1">
+      <x:c r="N2" t="str">
+        <x:v>HGEMM/CUTLASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="42" customHeight="1">
       <x:c r="A3" s="13" t="str">
-        <x:v>使用方法：原生与自研环境分别保存 run_gemm.sh 日志，再用 collect_gemm_results.py 增量合并到同一 CSV；将 CSV 数据粘贴到对应结果列。</x:v>
+        <x:v>使用方法：运行 run_gemm.sh 保存 CUTLASS 日志，再用 collect_gemm_results.py 自动生成/更新 CUTLASS 最佳配置和 GFLOPS；HGEMM（自研）和 HGEMM（CUDA）来自其他测试程序，请人工筛选最佳结果后填写黄色列。</x:v>
       </x:c>
       <x:c r="B3" s="13"/>
       <x:c r="C3" s="13"/>
@@ -476,6 +593,10 @@
       <x:c r="H3" s="13"/>
       <x:c r="I3" s="13"/>
       <x:c r="J3" s="13"/>
+      <x:c r="K3" s="52"/>
+      <x:c r="L3" s="52"/>
+      <x:c r="M3" s="52"/>
+      <x:c r="N3" s="52"/>
     </x:row>
     <x:row r="5" ht="20" customHeight="1">
       <x:c r="A5" s="18" t="str">
@@ -493,20 +614,32 @@
       <x:c r="E5" s="18" t="str">
         <x:v>K</x:v>
       </x:c>
-      <x:c r="F5" s="18" t="str">
-        <x:v>原生最佳配置</x:v>
-      </x:c>
-      <x:c r="G5" s="18" t="str">
-        <x:v>原生 GFLOPS</x:v>
-      </x:c>
-      <x:c r="H5" s="18" t="str">
-        <x:v>自研最佳配置</x:v>
-      </x:c>
-      <x:c r="I5" s="18" t="str">
-        <x:v>自研 GFLOPS</x:v>
-      </x:c>
-      <x:c r="J5" s="18" t="str">
-        <x:v>自研/原生加速比</x:v>
+      <x:c r="F5" s="31" t="str">
+        <x:v>CUTLASS最佳配置（脚本回填）</x:v>
+      </x:c>
+      <x:c r="G5" s="31" t="str">
+        <x:v>CUTLASS GFLOPS（脚本回填）</x:v>
+      </x:c>
+      <x:c r="H5" s="32" t="str">
+        <x:v>HGEMM（自研）最佳配置</x:v>
+      </x:c>
+      <x:c r="I5" s="32" t="str">
+        <x:v>HGEMM（自研）GFLOPS</x:v>
+      </x:c>
+      <x:c r="J5" s="33" t="str">
+        <x:v>HGEMM（CUDA）最佳配置</x:v>
+      </x:c>
+      <x:c r="K5" s="40" t="str">
+        <x:v>HGEMM（CUDA）GFLOPS</x:v>
+      </x:c>
+      <x:c r="L5" s="41" t="str">
+        <x:v>自研/CUTLASS 加速比</x:v>
+      </x:c>
+      <x:c r="M5" s="41" t="str">
+        <x:v>CUDA/CUTLASS 加速比</x:v>
+      </x:c>
+      <x:c r="N5" s="42" t="str">
+        <x:v>人工筛选备注</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20" customHeight="1">
@@ -525,13 +658,19 @@
       <x:c r="E6" s="19" t="n">
         <x:v>3584</x:v>
       </x:c>
-      <x:c r="F6" s="22" t="str"/>
-      <x:c r="G6" s="23"/>
-      <x:c r="H6" s="22" t="str"/>
-      <x:c r="I6" s="23"/>
-      <x:c r="J6" s="21" t="str">
+      <x:c r="F6" s="43" t="str"/>
+      <x:c r="G6" s="44"/>
+      <x:c r="H6" s="45" t="str"/>
+      <x:c r="I6" s="46"/>
+      <x:c r="J6" s="47"/>
+      <x:c r="K6" s="50"/>
+      <x:c r="L6" s="51" t="str">
         <x:f>IFERROR(I6/G6,"")</x:f>
       </x:c>
+      <x:c r="M6" s="51" t="str">
+        <x:f>IFERROR(K6/G6,"")</x:f>
+      </x:c>
+      <x:c r="N6" s="45"/>
     </x:row>
     <x:row r="7" ht="20" customHeight="1">
       <x:c r="A7" s="19" t="n">
@@ -549,13 +688,19 @@
       <x:c r="E7" s="19" t="n">
         <x:v>3584</x:v>
       </x:c>
-      <x:c r="F7" s="22" t="str"/>
-      <x:c r="G7" s="23"/>
-      <x:c r="H7" s="22" t="str"/>
-      <x:c r="I7" s="23"/>
-      <x:c r="J7" s="21" t="str">
+      <x:c r="F7" s="43" t="str"/>
+      <x:c r="G7" s="44"/>
+      <x:c r="H7" s="45" t="str"/>
+      <x:c r="I7" s="46"/>
+      <x:c r="J7" s="47"/>
+      <x:c r="K7" s="50"/>
+      <x:c r="L7" s="51" t="str">
         <x:f>IFERROR(I7/G7,"")</x:f>
       </x:c>
+      <x:c r="M7" s="51" t="str">
+        <x:f>IFERROR(K7/G7,"")</x:f>
+      </x:c>
+      <x:c r="N7" s="45"/>
     </x:row>
     <x:row r="8" ht="20" customHeight="1">
       <x:c r="A8" s="19" t="n">
@@ -573,13 +718,19 @@
       <x:c r="E8" s="19" t="n">
         <x:v>3584</x:v>
       </x:c>
-      <x:c r="F8" s="22" t="str"/>
-      <x:c r="G8" s="23"/>
-      <x:c r="H8" s="22" t="str"/>
-      <x:c r="I8" s="23"/>
-      <x:c r="J8" s="21" t="str">
+      <x:c r="F8" s="43" t="str"/>
+      <x:c r="G8" s="44"/>
+      <x:c r="H8" s="45" t="str"/>
+      <x:c r="I8" s="46"/>
+      <x:c r="J8" s="47"/>
+      <x:c r="K8" s="50"/>
+      <x:c r="L8" s="51" t="str">
         <x:f>IFERROR(I8/G8,"")</x:f>
       </x:c>
+      <x:c r="M8" s="51" t="str">
+        <x:f>IFERROR(K8/G8,"")</x:f>
+      </x:c>
+      <x:c r="N8" s="45"/>
     </x:row>
     <x:row r="9" ht="20" customHeight="1">
       <x:c r="A9" s="19" t="n">
@@ -597,13 +748,19 @@
       <x:c r="E9" s="19" t="n">
         <x:v>128</x:v>
       </x:c>
-      <x:c r="F9" s="22" t="str"/>
-      <x:c r="G9" s="23"/>
-      <x:c r="H9" s="22" t="str"/>
-      <x:c r="I9" s="23"/>
-      <x:c r="J9" s="21" t="str">
+      <x:c r="F9" s="43" t="str"/>
+      <x:c r="G9" s="44"/>
+      <x:c r="H9" s="45" t="str"/>
+      <x:c r="I9" s="46"/>
+      <x:c r="J9" s="47"/>
+      <x:c r="K9" s="50"/>
+      <x:c r="L9" s="51" t="str">
         <x:f>IFERROR(I9/G9,"")</x:f>
       </x:c>
+      <x:c r="M9" s="51" t="str">
+        <x:f>IFERROR(K9/G9,"")</x:f>
+      </x:c>
+      <x:c r="N9" s="45"/>
     </x:row>
     <x:row r="10" ht="20" customHeight="1">
       <x:c r="A10" s="19" t="n">
@@ -621,13 +778,19 @@
       <x:c r="E10" s="19" t="n">
         <x:v>128</x:v>
       </x:c>
-      <x:c r="F10" s="22" t="str"/>
-      <x:c r="G10" s="23"/>
-      <x:c r="H10" s="22" t="str"/>
-      <x:c r="I10" s="23"/>
-      <x:c r="J10" s="21" t="str">
+      <x:c r="F10" s="43" t="str"/>
+      <x:c r="G10" s="44"/>
+      <x:c r="H10" s="45" t="str"/>
+      <x:c r="I10" s="46"/>
+      <x:c r="J10" s="47"/>
+      <x:c r="K10" s="50"/>
+      <x:c r="L10" s="51" t="str">
         <x:f>IFERROR(I10/G10,"")</x:f>
       </x:c>
+      <x:c r="M10" s="51" t="str">
+        <x:f>IFERROR(K10/G10,"")</x:f>
+      </x:c>
+      <x:c r="N10" s="45"/>
     </x:row>
     <x:row r="11" ht="20" customHeight="1">
       <x:c r="A11" s="19" t="n">
@@ -645,13 +808,19 @@
       <x:c r="E11" s="19" t="n">
         <x:v>3584</x:v>
       </x:c>
-      <x:c r="F11" s="22" t="str"/>
-      <x:c r="G11" s="23"/>
-      <x:c r="H11" s="22" t="str"/>
-      <x:c r="I11" s="23"/>
-      <x:c r="J11" s="21" t="str">
+      <x:c r="F11" s="43" t="str"/>
+      <x:c r="G11" s="44"/>
+      <x:c r="H11" s="45" t="str"/>
+      <x:c r="I11" s="46"/>
+      <x:c r="J11" s="47"/>
+      <x:c r="K11" s="50"/>
+      <x:c r="L11" s="51" t="str">
         <x:f>IFERROR(I11/G11,"")</x:f>
       </x:c>
+      <x:c r="M11" s="51" t="str">
+        <x:f>IFERROR(K11/G11,"")</x:f>
+      </x:c>
+      <x:c r="N11" s="45"/>
     </x:row>
     <x:row r="12" ht="20" customHeight="1">
       <x:c r="A12" s="19" t="n">
@@ -669,13 +838,19 @@
       <x:c r="E12" s="19" t="n">
         <x:v>3584</x:v>
       </x:c>
-      <x:c r="F12" s="22" t="str"/>
-      <x:c r="G12" s="23"/>
-      <x:c r="H12" s="22" t="str"/>
-      <x:c r="I12" s="23"/>
-      <x:c r="J12" s="21" t="str">
+      <x:c r="F12" s="43" t="str"/>
+      <x:c r="G12" s="44"/>
+      <x:c r="H12" s="45" t="str"/>
+      <x:c r="I12" s="46"/>
+      <x:c r="J12" s="47"/>
+      <x:c r="K12" s="50"/>
+      <x:c r="L12" s="51" t="str">
         <x:f>IFERROR(I12/G12,"")</x:f>
       </x:c>
+      <x:c r="M12" s="51" t="str">
+        <x:f>IFERROR(K12/G12,"")</x:f>
+      </x:c>
+      <x:c r="N12" s="45"/>
     </x:row>
     <x:row r="13" ht="20" customHeight="1">
       <x:c r="A13" s="19" t="n">
@@ -693,13 +868,19 @@
       <x:c r="E13" s="19" t="n">
         <x:v>18944</x:v>
       </x:c>
-      <x:c r="F13" s="22" t="str"/>
-      <x:c r="G13" s="23"/>
-      <x:c r="H13" s="22" t="str"/>
-      <x:c r="I13" s="23"/>
-      <x:c r="J13" s="21" t="str">
+      <x:c r="F13" s="43" t="str"/>
+      <x:c r="G13" s="44"/>
+      <x:c r="H13" s="45" t="str"/>
+      <x:c r="I13" s="46"/>
+      <x:c r="J13" s="47"/>
+      <x:c r="K13" s="50"/>
+      <x:c r="L13" s="51" t="str">
         <x:f>IFERROR(I13/G13,"")</x:f>
       </x:c>
+      <x:c r="M13" s="51" t="str">
+        <x:f>IFERROR(K13/G13,"")</x:f>
+      </x:c>
+      <x:c r="N13" s="45"/>
     </x:row>
     <x:row r="14" ht="20" customHeight="1">
       <x:c r="A14" s="19" t="n">
@@ -717,13 +898,19 @@
       <x:c r="E14" s="19" t="n">
         <x:v>3584</x:v>
       </x:c>
-      <x:c r="F14" s="22" t="str"/>
-      <x:c r="G14" s="23"/>
-      <x:c r="H14" s="22" t="str"/>
-      <x:c r="I14" s="23"/>
-      <x:c r="J14" s="21" t="str">
+      <x:c r="F14" s="43" t="str"/>
+      <x:c r="G14" s="44"/>
+      <x:c r="H14" s="45" t="str"/>
+      <x:c r="I14" s="46"/>
+      <x:c r="J14" s="47"/>
+      <x:c r="K14" s="50"/>
+      <x:c r="L14" s="51" t="str">
         <x:f>IFERROR(I14/G14,"")</x:f>
       </x:c>
+      <x:c r="M14" s="51" t="str">
+        <x:f>IFERROR(K14/G14,"")</x:f>
+      </x:c>
+      <x:c r="N14" s="45"/>
     </x:row>
     <x:row r="15" ht="20" customHeight="1">
       <x:c r="A15" s="19" t="n">
@@ -741,13 +928,19 @@
       <x:c r="E15" s="19" t="n">
         <x:v>3584</x:v>
       </x:c>
-      <x:c r="F15" s="22" t="str"/>
-      <x:c r="G15" s="23"/>
-      <x:c r="H15" s="22" t="str"/>
-      <x:c r="I15" s="23"/>
-      <x:c r="J15" s="21" t="str">
+      <x:c r="F15" s="43" t="str"/>
+      <x:c r="G15" s="44"/>
+      <x:c r="H15" s="45" t="str"/>
+      <x:c r="I15" s="46"/>
+      <x:c r="J15" s="47"/>
+      <x:c r="K15" s="50"/>
+      <x:c r="L15" s="51" t="str">
         <x:f>IFERROR(I15/G15,"")</x:f>
       </x:c>
+      <x:c r="M15" s="51" t="str">
+        <x:f>IFERROR(K15/G15,"")</x:f>
+      </x:c>
+      <x:c r="N15" s="45"/>
     </x:row>
     <x:row r="16" ht="20" customHeight="1">
       <x:c r="A16" s="19" t="n">
@@ -765,13 +958,19 @@
       <x:c r="E16" s="19" t="n">
         <x:v>3584</x:v>
       </x:c>
-      <x:c r="F16" s="22" t="str"/>
-      <x:c r="G16" s="23"/>
-      <x:c r="H16" s="22" t="str"/>
-      <x:c r="I16" s="23"/>
-      <x:c r="J16" s="21" t="str">
+      <x:c r="F16" s="43" t="str"/>
+      <x:c r="G16" s="44"/>
+      <x:c r="H16" s="45" t="str"/>
+      <x:c r="I16" s="46"/>
+      <x:c r="J16" s="47"/>
+      <x:c r="K16" s="50"/>
+      <x:c r="L16" s="51" t="str">
         <x:f>IFERROR(I16/G16,"")</x:f>
       </x:c>
+      <x:c r="M16" s="51" t="str">
+        <x:f>IFERROR(K16/G16,"")</x:f>
+      </x:c>
+      <x:c r="N16" s="45"/>
     </x:row>
     <x:row r="17" ht="20" customHeight="1">
       <x:c r="A17" s="19" t="n">
@@ -789,13 +988,19 @@
       <x:c r="E17" s="19" t="n">
         <x:v>3584</x:v>
       </x:c>
-      <x:c r="F17" s="22" t="str"/>
-      <x:c r="G17" s="23"/>
-      <x:c r="H17" s="22" t="str"/>
-      <x:c r="I17" s="23"/>
-      <x:c r="J17" s="21" t="str">
+      <x:c r="F17" s="43" t="str"/>
+      <x:c r="G17" s="44"/>
+      <x:c r="H17" s="45" t="str"/>
+      <x:c r="I17" s="46"/>
+      <x:c r="J17" s="47"/>
+      <x:c r="K17" s="50"/>
+      <x:c r="L17" s="51" t="str">
         <x:f>IFERROR(I17/G17,"")</x:f>
       </x:c>
+      <x:c r="M17" s="51" t="str">
+        <x:f>IFERROR(K17/G17,"")</x:f>
+      </x:c>
+      <x:c r="N17" s="45"/>
     </x:row>
     <x:row r="18" ht="20" customHeight="1">
       <x:c r="A18" s="19" t="n">
@@ -813,13 +1018,19 @@
       <x:c r="E18" s="19" t="n">
         <x:v>128</x:v>
       </x:c>
-      <x:c r="F18" s="22" t="str"/>
-      <x:c r="G18" s="23"/>
-      <x:c r="H18" s="22" t="str"/>
-      <x:c r="I18" s="23"/>
-      <x:c r="J18" s="21" t="str">
+      <x:c r="F18" s="43" t="str"/>
+      <x:c r="G18" s="44"/>
+      <x:c r="H18" s="45" t="str"/>
+      <x:c r="I18" s="46"/>
+      <x:c r="J18" s="47"/>
+      <x:c r="K18" s="50"/>
+      <x:c r="L18" s="51" t="str">
         <x:f>IFERROR(I18/G18,"")</x:f>
       </x:c>
+      <x:c r="M18" s="51" t="str">
+        <x:f>IFERROR(K18/G18,"")</x:f>
+      </x:c>
+      <x:c r="N18" s="45"/>
     </x:row>
     <x:row r="19" ht="20" customHeight="1">
       <x:c r="A19" s="19" t="n">
@@ -837,13 +1048,19 @@
       <x:c r="E19" s="19" t="n">
         <x:v>256</x:v>
       </x:c>
-      <x:c r="F19" s="22" t="str"/>
-      <x:c r="G19" s="23"/>
-      <x:c r="H19" s="22" t="str"/>
-      <x:c r="I19" s="23"/>
-      <x:c r="J19" s="21" t="str">
+      <x:c r="F19" s="43" t="str"/>
+      <x:c r="G19" s="44"/>
+      <x:c r="H19" s="45" t="str"/>
+      <x:c r="I19" s="46"/>
+      <x:c r="J19" s="47"/>
+      <x:c r="K19" s="50"/>
+      <x:c r="L19" s="51" t="str">
         <x:f>IFERROR(I19/G19,"")</x:f>
       </x:c>
+      <x:c r="M19" s="51" t="str">
+        <x:f>IFERROR(K19/G19,"")</x:f>
+      </x:c>
+      <x:c r="N19" s="45"/>
     </x:row>
     <x:row r="20" ht="20" customHeight="1">
       <x:c r="A20" s="19" t="n">
@@ -861,13 +1078,19 @@
       <x:c r="E20" s="19" t="n">
         <x:v>3584</x:v>
       </x:c>
-      <x:c r="F20" s="22" t="str"/>
-      <x:c r="G20" s="23"/>
-      <x:c r="H20" s="22" t="str"/>
-      <x:c r="I20" s="23"/>
-      <x:c r="J20" s="21" t="str">
+      <x:c r="F20" s="43" t="str"/>
+      <x:c r="G20" s="44"/>
+      <x:c r="H20" s="45" t="str"/>
+      <x:c r="I20" s="46"/>
+      <x:c r="J20" s="47"/>
+      <x:c r="K20" s="50"/>
+      <x:c r="L20" s="51" t="str">
         <x:f>IFERROR(I20/G20,"")</x:f>
       </x:c>
+      <x:c r="M20" s="51" t="str">
+        <x:f>IFERROR(K20/G20,"")</x:f>
+      </x:c>
+      <x:c r="N20" s="45"/>
     </x:row>
     <x:row r="21" ht="20" customHeight="1">
       <x:c r="A21" s="19" t="n">
@@ -885,13 +1108,19 @@
       <x:c r="E21" s="19" t="n">
         <x:v>3584</x:v>
       </x:c>
-      <x:c r="F21" s="22" t="str"/>
-      <x:c r="G21" s="23"/>
-      <x:c r="H21" s="22" t="str"/>
-      <x:c r="I21" s="23"/>
-      <x:c r="J21" s="21" t="str">
+      <x:c r="F21" s="43" t="str"/>
+      <x:c r="G21" s="44"/>
+      <x:c r="H21" s="45" t="str"/>
+      <x:c r="I21" s="46"/>
+      <x:c r="J21" s="47"/>
+      <x:c r="K21" s="50"/>
+      <x:c r="L21" s="51" t="str">
         <x:f>IFERROR(I21/G21,"")</x:f>
       </x:c>
+      <x:c r="M21" s="51" t="str">
+        <x:f>IFERROR(K21/G21,"")</x:f>
+      </x:c>
+      <x:c r="N21" s="45"/>
     </x:row>
     <x:row r="22" ht="20" customHeight="1">
       <x:c r="A22" s="19" t="n">
@@ -909,13 +1138,19 @@
       <x:c r="E22" s="19" t="n">
         <x:v>18944</x:v>
       </x:c>
-      <x:c r="F22" s="22" t="str"/>
-      <x:c r="G22" s="23"/>
-      <x:c r="H22" s="22" t="str"/>
-      <x:c r="I22" s="23"/>
-      <x:c r="J22" s="21" t="str">
+      <x:c r="F22" s="43" t="str"/>
+      <x:c r="G22" s="44"/>
+      <x:c r="H22" s="45" t="str"/>
+      <x:c r="I22" s="46"/>
+      <x:c r="J22" s="47"/>
+      <x:c r="K22" s="50"/>
+      <x:c r="L22" s="51" t="str">
         <x:f>IFERROR(I22/G22,"")</x:f>
       </x:c>
+      <x:c r="M22" s="51" t="str">
+        <x:f>IFERROR(K22/G22,"")</x:f>
+      </x:c>
+      <x:c r="N22" s="45"/>
     </x:row>
     <x:row r="23" ht="20" customHeight="1">
       <x:c r="A23" s="19" t="n">
@@ -933,13 +1168,19 @@
       <x:c r="E23" s="19" t="n">
         <x:v>3584</x:v>
       </x:c>
-      <x:c r="F23" s="22" t="str"/>
-      <x:c r="G23" s="23"/>
-      <x:c r="H23" s="22" t="str"/>
-      <x:c r="I23" s="23"/>
-      <x:c r="J23" s="21" t="str">
+      <x:c r="F23" s="43" t="str"/>
+      <x:c r="G23" s="44"/>
+      <x:c r="H23" s="45" t="str"/>
+      <x:c r="I23" s="46"/>
+      <x:c r="J23" s="47"/>
+      <x:c r="K23" s="50"/>
+      <x:c r="L23" s="51" t="str">
         <x:f>IFERROR(I23/G23,"")</x:f>
       </x:c>
+      <x:c r="M23" s="51" t="str">
+        <x:f>IFERROR(K23/G23,"")</x:f>
+      </x:c>
+      <x:c r="N23" s="45"/>
     </x:row>
     <x:row r="24" ht="20" customHeight="1">
       <x:c r="A24" s="19" t="n">
@@ -957,13 +1198,19 @@
       <x:c r="E24" s="19" t="n">
         <x:v>3584</x:v>
       </x:c>
-      <x:c r="F24" s="22" t="str"/>
-      <x:c r="G24" s="23"/>
-      <x:c r="H24" s="22" t="str"/>
-      <x:c r="I24" s="23"/>
-      <x:c r="J24" s="21" t="str">
+      <x:c r="F24" s="43" t="str"/>
+      <x:c r="G24" s="44"/>
+      <x:c r="H24" s="45" t="str"/>
+      <x:c r="I24" s="46"/>
+      <x:c r="J24" s="47"/>
+      <x:c r="K24" s="50"/>
+      <x:c r="L24" s="51" t="str">
         <x:f>IFERROR(I24/G24,"")</x:f>
       </x:c>
+      <x:c r="M24" s="51" t="str">
+        <x:f>IFERROR(K24/G24,"")</x:f>
+      </x:c>
+      <x:c r="N24" s="45"/>
     </x:row>
     <x:row r="25" ht="20" customHeight="1">
       <x:c r="A25" s="19" t="n">
@@ -981,13 +1228,19 @@
       <x:c r="E25" s="19" t="n">
         <x:v>3584</x:v>
       </x:c>
-      <x:c r="F25" s="22" t="str"/>
-      <x:c r="G25" s="23"/>
-      <x:c r="H25" s="22" t="str"/>
-      <x:c r="I25" s="23"/>
-      <x:c r="J25" s="21" t="str">
+      <x:c r="F25" s="43" t="str"/>
+      <x:c r="G25" s="44"/>
+      <x:c r="H25" s="45" t="str"/>
+      <x:c r="I25" s="46"/>
+      <x:c r="J25" s="47"/>
+      <x:c r="K25" s="50"/>
+      <x:c r="L25" s="51" t="str">
         <x:f>IFERROR(I25/G25,"")</x:f>
       </x:c>
+      <x:c r="M25" s="51" t="str">
+        <x:f>IFERROR(K25/G25,"")</x:f>
+      </x:c>
+      <x:c r="N25" s="45"/>
     </x:row>
     <x:row r="26" ht="20" customHeight="1">
       <x:c r="A26" s="19" t="n">
@@ -1005,13 +1258,19 @@
       <x:c r="E26" s="19" t="n">
         <x:v>3584</x:v>
       </x:c>
-      <x:c r="F26" s="22" t="str"/>
-      <x:c r="G26" s="23"/>
-      <x:c r="H26" s="22" t="str"/>
-      <x:c r="I26" s="23"/>
-      <x:c r="J26" s="21" t="str">
+      <x:c r="F26" s="43" t="str"/>
+      <x:c r="G26" s="44"/>
+      <x:c r="H26" s="45" t="str"/>
+      <x:c r="I26" s="46"/>
+      <x:c r="J26" s="47"/>
+      <x:c r="K26" s="50"/>
+      <x:c r="L26" s="51" t="str">
         <x:f>IFERROR(I26/G26,"")</x:f>
       </x:c>
+      <x:c r="M26" s="51" t="str">
+        <x:f>IFERROR(K26/G26,"")</x:f>
+      </x:c>
+      <x:c r="N26" s="45"/>
     </x:row>
     <x:row r="27" ht="20" customHeight="1">
       <x:c r="A27" s="19" t="n">
@@ -1029,13 +1288,19 @@
       <x:c r="E27" s="19" t="n">
         <x:v>128</x:v>
       </x:c>
-      <x:c r="F27" s="22" t="str"/>
-      <x:c r="G27" s="23"/>
-      <x:c r="H27" s="22" t="str"/>
-      <x:c r="I27" s="23"/>
-      <x:c r="J27" s="21" t="str">
+      <x:c r="F27" s="43" t="str"/>
+      <x:c r="G27" s="44"/>
+      <x:c r="H27" s="45" t="str"/>
+      <x:c r="I27" s="46"/>
+      <x:c r="J27" s="47"/>
+      <x:c r="K27" s="50"/>
+      <x:c r="L27" s="51" t="str">
         <x:f>IFERROR(I27/G27,"")</x:f>
       </x:c>
+      <x:c r="M27" s="51" t="str">
+        <x:f>IFERROR(K27/G27,"")</x:f>
+      </x:c>
+      <x:c r="N27" s="45"/>
     </x:row>
     <x:row r="28" ht="20" customHeight="1">
       <x:c r="A28" s="19" t="n">
@@ -1053,13 +1318,19 @@
       <x:c r="E28" s="19" t="n">
         <x:v>512</x:v>
       </x:c>
-      <x:c r="F28" s="22" t="str"/>
-      <x:c r="G28" s="23"/>
-      <x:c r="H28" s="22" t="str"/>
-      <x:c r="I28" s="23"/>
-      <x:c r="J28" s="21" t="str">
+      <x:c r="F28" s="43" t="str"/>
+      <x:c r="G28" s="44"/>
+      <x:c r="H28" s="45" t="str"/>
+      <x:c r="I28" s="46"/>
+      <x:c r="J28" s="47"/>
+      <x:c r="K28" s="50"/>
+      <x:c r="L28" s="51" t="str">
         <x:f>IFERROR(I28/G28,"")</x:f>
       </x:c>
+      <x:c r="M28" s="51" t="str">
+        <x:f>IFERROR(K28/G28,"")</x:f>
+      </x:c>
+      <x:c r="N28" s="45"/>
     </x:row>
     <x:row r="29" ht="20" customHeight="1">
       <x:c r="A29" s="19" t="n">
@@ -1077,13 +1348,19 @@
       <x:c r="E29" s="19" t="n">
         <x:v>3584</x:v>
       </x:c>
-      <x:c r="F29" s="22" t="str"/>
-      <x:c r="G29" s="23"/>
-      <x:c r="H29" s="22" t="str"/>
-      <x:c r="I29" s="23"/>
-      <x:c r="J29" s="21" t="str">
+      <x:c r="F29" s="43" t="str"/>
+      <x:c r="G29" s="44"/>
+      <x:c r="H29" s="45" t="str"/>
+      <x:c r="I29" s="46"/>
+      <x:c r="J29" s="47"/>
+      <x:c r="K29" s="50"/>
+      <x:c r="L29" s="51" t="str">
         <x:f>IFERROR(I29/G29,"")</x:f>
       </x:c>
+      <x:c r="M29" s="51" t="str">
+        <x:f>IFERROR(K29/G29,"")</x:f>
+      </x:c>
+      <x:c r="N29" s="45"/>
     </x:row>
     <x:row r="30" ht="20" customHeight="1">
       <x:c r="A30" s="19" t="n">
@@ -1101,13 +1378,19 @@
       <x:c r="E30" s="19" t="n">
         <x:v>3584</x:v>
       </x:c>
-      <x:c r="F30" s="22" t="str"/>
-      <x:c r="G30" s="23"/>
-      <x:c r="H30" s="22" t="str"/>
-      <x:c r="I30" s="23"/>
-      <x:c r="J30" s="21" t="str">
+      <x:c r="F30" s="43" t="str"/>
+      <x:c r="G30" s="44"/>
+      <x:c r="H30" s="45" t="str"/>
+      <x:c r="I30" s="46"/>
+      <x:c r="J30" s="47"/>
+      <x:c r="K30" s="50"/>
+      <x:c r="L30" s="51" t="str">
         <x:f>IFERROR(I30/G30,"")</x:f>
       </x:c>
+      <x:c r="M30" s="51" t="str">
+        <x:f>IFERROR(K30/G30,"")</x:f>
+      </x:c>
+      <x:c r="N30" s="45"/>
     </x:row>
     <x:row r="31" ht="20" customHeight="1">
       <x:c r="A31" s="19" t="n">
@@ -1125,13 +1408,19 @@
       <x:c r="E31" s="19" t="n">
         <x:v>18944</x:v>
       </x:c>
-      <x:c r="F31" s="22" t="str"/>
-      <x:c r="G31" s="23"/>
-      <x:c r="H31" s="22" t="str"/>
-      <x:c r="I31" s="23"/>
-      <x:c r="J31" s="21" t="str">
+      <x:c r="F31" s="43" t="str"/>
+      <x:c r="G31" s="44"/>
+      <x:c r="H31" s="45" t="str"/>
+      <x:c r="I31" s="46"/>
+      <x:c r="J31" s="47"/>
+      <x:c r="K31" s="50"/>
+      <x:c r="L31" s="51" t="str">
         <x:f>IFERROR(I31/G31,"")</x:f>
       </x:c>
+      <x:c r="M31" s="51" t="str">
+        <x:f>IFERROR(K31/G31,"")</x:f>
+      </x:c>
+      <x:c r="N31" s="45"/>
     </x:row>
     <x:row r="32" ht="20" customHeight="1">
       <x:c r="A32" s="19" t="n">
@@ -1149,13 +1438,19 @@
       <x:c r="E32" s="19" t="n">
         <x:v>3584</x:v>
       </x:c>
-      <x:c r="F32" s="22" t="str"/>
-      <x:c r="G32" s="23"/>
-      <x:c r="H32" s="22" t="str"/>
-      <x:c r="I32" s="23"/>
-      <x:c r="J32" s="21" t="str">
+      <x:c r="F32" s="43" t="str"/>
+      <x:c r="G32" s="44"/>
+      <x:c r="H32" s="45" t="str"/>
+      <x:c r="I32" s="46"/>
+      <x:c r="J32" s="47"/>
+      <x:c r="K32" s="50"/>
+      <x:c r="L32" s="51" t="str">
         <x:f>IFERROR(I32/G32,"")</x:f>
       </x:c>
+      <x:c r="M32" s="51" t="str">
+        <x:f>IFERROR(K32/G32,"")</x:f>
+      </x:c>
+      <x:c r="N32" s="45"/>
     </x:row>
     <x:row r="33" ht="20" customHeight="1">
       <x:c r="A33" s="19" t="n">
@@ -1173,13 +1468,19 @@
       <x:c r="E33" s="19" t="n">
         <x:v>3584</x:v>
       </x:c>
-      <x:c r="F33" s="22" t="str"/>
-      <x:c r="G33" s="23"/>
-      <x:c r="H33" s="22" t="str"/>
-      <x:c r="I33" s="23"/>
-      <x:c r="J33" s="21" t="str">
+      <x:c r="F33" s="43" t="str"/>
+      <x:c r="G33" s="44"/>
+      <x:c r="H33" s="45" t="str"/>
+      <x:c r="I33" s="46"/>
+      <x:c r="J33" s="47"/>
+      <x:c r="K33" s="50"/>
+      <x:c r="L33" s="51" t="str">
         <x:f>IFERROR(I33/G33,"")</x:f>
       </x:c>
+      <x:c r="M33" s="51" t="str">
+        <x:f>IFERROR(K33/G33,"")</x:f>
+      </x:c>
+      <x:c r="N33" s="45"/>
     </x:row>
     <x:row r="34" ht="20" customHeight="1">
       <x:c r="A34" s="19" t="n">
@@ -1197,13 +1498,19 @@
       <x:c r="E34" s="19" t="n">
         <x:v>3584</x:v>
       </x:c>
-      <x:c r="F34" s="22" t="str"/>
-      <x:c r="G34" s="23"/>
-      <x:c r="H34" s="22" t="str"/>
-      <x:c r="I34" s="23"/>
-      <x:c r="J34" s="21" t="str">
+      <x:c r="F34" s="43" t="str"/>
+      <x:c r="G34" s="44"/>
+      <x:c r="H34" s="45" t="str"/>
+      <x:c r="I34" s="46"/>
+      <x:c r="J34" s="47"/>
+      <x:c r="K34" s="50"/>
+      <x:c r="L34" s="51" t="str">
         <x:f>IFERROR(I34/G34,"")</x:f>
       </x:c>
+      <x:c r="M34" s="51" t="str">
+        <x:f>IFERROR(K34/G34,"")</x:f>
+      </x:c>
+      <x:c r="N34" s="45"/>
     </x:row>
     <x:row r="35" ht="20" customHeight="1">
       <x:c r="A35" s="19" t="n">
@@ -1221,13 +1528,19 @@
       <x:c r="E35" s="19" t="n">
         <x:v>3584</x:v>
       </x:c>
-      <x:c r="F35" s="22" t="str"/>
-      <x:c r="G35" s="23"/>
-      <x:c r="H35" s="22" t="str"/>
-      <x:c r="I35" s="23"/>
-      <x:c r="J35" s="21" t="str">
+      <x:c r="F35" s="43" t="str"/>
+      <x:c r="G35" s="44"/>
+      <x:c r="H35" s="45" t="str"/>
+      <x:c r="I35" s="46"/>
+      <x:c r="J35" s="47"/>
+      <x:c r="K35" s="50"/>
+      <x:c r="L35" s="51" t="str">
         <x:f>IFERROR(I35/G35,"")</x:f>
       </x:c>
+      <x:c r="M35" s="51" t="str">
+        <x:f>IFERROR(K35/G35,"")</x:f>
+      </x:c>
+      <x:c r="N35" s="45"/>
     </x:row>
     <x:row r="36" ht="20" customHeight="1">
       <x:c r="A36" s="19" t="n">
@@ -1245,13 +1558,19 @@
       <x:c r="E36" s="19" t="n">
         <x:v>128</x:v>
       </x:c>
-      <x:c r="F36" s="22" t="str"/>
-      <x:c r="G36" s="23"/>
-      <x:c r="H36" s="22" t="str"/>
-      <x:c r="I36" s="23"/>
-      <x:c r="J36" s="21" t="str">
+      <x:c r="F36" s="43" t="str"/>
+      <x:c r="G36" s="44"/>
+      <x:c r="H36" s="45" t="str"/>
+      <x:c r="I36" s="46"/>
+      <x:c r="J36" s="47"/>
+      <x:c r="K36" s="50"/>
+      <x:c r="L36" s="51" t="str">
         <x:f>IFERROR(I36/G36,"")</x:f>
       </x:c>
+      <x:c r="M36" s="51" t="str">
+        <x:f>IFERROR(K36/G36,"")</x:f>
+      </x:c>
+      <x:c r="N36" s="45"/>
     </x:row>
     <x:row r="37" ht="20" customHeight="1">
       <x:c r="A37" s="19" t="n">
@@ -1269,13 +1588,19 @@
       <x:c r="E37" s="19" t="n">
         <x:v>1024</x:v>
       </x:c>
-      <x:c r="F37" s="22" t="str"/>
-      <x:c r="G37" s="23"/>
-      <x:c r="H37" s="22" t="str"/>
-      <x:c r="I37" s="23"/>
-      <x:c r="J37" s="21" t="str">
+      <x:c r="F37" s="43" t="str"/>
+      <x:c r="G37" s="44"/>
+      <x:c r="H37" s="45" t="str"/>
+      <x:c r="I37" s="46"/>
+      <x:c r="J37" s="47"/>
+      <x:c r="K37" s="50"/>
+      <x:c r="L37" s="51" t="str">
         <x:f>IFERROR(I37/G37,"")</x:f>
       </x:c>
+      <x:c r="M37" s="51" t="str">
+        <x:f>IFERROR(K37/G37,"")</x:f>
+      </x:c>
+      <x:c r="N37" s="45"/>
     </x:row>
     <x:row r="38" ht="20" customHeight="1">
       <x:c r="A38" s="19" t="n">
@@ -1293,13 +1618,19 @@
       <x:c r="E38" s="19" t="n">
         <x:v>3584</x:v>
       </x:c>
-      <x:c r="F38" s="22" t="str"/>
-      <x:c r="G38" s="23"/>
-      <x:c r="H38" s="22" t="str"/>
-      <x:c r="I38" s="23"/>
-      <x:c r="J38" s="21" t="str">
+      <x:c r="F38" s="43" t="str"/>
+      <x:c r="G38" s="44"/>
+      <x:c r="H38" s="45" t="str"/>
+      <x:c r="I38" s="46"/>
+      <x:c r="J38" s="47"/>
+      <x:c r="K38" s="50"/>
+      <x:c r="L38" s="51" t="str">
         <x:f>IFERROR(I38/G38,"")</x:f>
       </x:c>
+      <x:c r="M38" s="51" t="str">
+        <x:f>IFERROR(K38/G38,"")</x:f>
+      </x:c>
+      <x:c r="N38" s="45"/>
     </x:row>
     <x:row r="39" ht="20" customHeight="1">
       <x:c r="A39" s="19" t="n">
@@ -1317,13 +1648,19 @@
       <x:c r="E39" s="19" t="n">
         <x:v>3584</x:v>
       </x:c>
-      <x:c r="F39" s="22" t="str"/>
-      <x:c r="G39" s="23"/>
-      <x:c r="H39" s="22" t="str"/>
-      <x:c r="I39" s="23"/>
-      <x:c r="J39" s="21" t="str">
+      <x:c r="F39" s="43" t="str"/>
+      <x:c r="G39" s="44"/>
+      <x:c r="H39" s="45" t="str"/>
+      <x:c r="I39" s="46"/>
+      <x:c r="J39" s="47"/>
+      <x:c r="K39" s="50"/>
+      <x:c r="L39" s="51" t="str">
         <x:f>IFERROR(I39/G39,"")</x:f>
       </x:c>
+      <x:c r="M39" s="51" t="str">
+        <x:f>IFERROR(K39/G39,"")</x:f>
+      </x:c>
+      <x:c r="N39" s="45"/>
     </x:row>
     <x:row r="40" ht="20" customHeight="1">
       <x:c r="A40" s="19" t="n">
@@ -1341,13 +1678,19 @@
       <x:c r="E40" s="19" t="n">
         <x:v>18944</x:v>
       </x:c>
-      <x:c r="F40" s="22" t="str"/>
-      <x:c r="G40" s="23"/>
-      <x:c r="H40" s="22" t="str"/>
-      <x:c r="I40" s="23"/>
-      <x:c r="J40" s="21" t="str">
+      <x:c r="F40" s="43" t="str"/>
+      <x:c r="G40" s="44"/>
+      <x:c r="H40" s="45" t="str"/>
+      <x:c r="I40" s="46"/>
+      <x:c r="J40" s="47"/>
+      <x:c r="K40" s="50"/>
+      <x:c r="L40" s="51" t="str">
         <x:f>IFERROR(I40/G40,"")</x:f>
       </x:c>
+      <x:c r="M40" s="51" t="str">
+        <x:f>IFERROR(K40/G40,"")</x:f>
+      </x:c>
+      <x:c r="N40" s="45"/>
     </x:row>
     <x:row r="41" ht="20" customHeight="1">
       <x:c r="A41" s="19" t="n">
@@ -1365,13 +1708,19 @@
       <x:c r="E41" s="19" t="n">
         <x:v>3584</x:v>
       </x:c>
-      <x:c r="F41" s="22" t="str"/>
-      <x:c r="G41" s="23"/>
-      <x:c r="H41" s="22" t="str"/>
-      <x:c r="I41" s="23"/>
-      <x:c r="J41" s="21" t="str">
+      <x:c r="F41" s="43" t="str"/>
+      <x:c r="G41" s="44"/>
+      <x:c r="H41" s="45" t="str"/>
+      <x:c r="I41" s="46"/>
+      <x:c r="J41" s="47"/>
+      <x:c r="K41" s="50"/>
+      <x:c r="L41" s="51" t="str">
         <x:f>IFERROR(I41/G41,"")</x:f>
       </x:c>
+      <x:c r="M41" s="51" t="str">
+        <x:f>IFERROR(K41/G41,"")</x:f>
+      </x:c>
+      <x:c r="N41" s="45"/>
     </x:row>
     <x:row r="42" ht="20" customHeight="1">
       <x:c r="A42" s="19" t="n">
@@ -1389,13 +1738,19 @@
       <x:c r="E42" s="19" t="n">
         <x:v>3584</x:v>
       </x:c>
-      <x:c r="F42" s="22" t="str"/>
-      <x:c r="G42" s="23"/>
-      <x:c r="H42" s="22" t="str"/>
-      <x:c r="I42" s="23"/>
-      <x:c r="J42" s="21" t="str">
+      <x:c r="F42" s="43" t="str"/>
+      <x:c r="G42" s="44"/>
+      <x:c r="H42" s="45" t="str"/>
+      <x:c r="I42" s="46"/>
+      <x:c r="J42" s="47"/>
+      <x:c r="K42" s="50"/>
+      <x:c r="L42" s="51" t="str">
         <x:f>IFERROR(I42/G42,"")</x:f>
       </x:c>
+      <x:c r="M42" s="51" t="str">
+        <x:f>IFERROR(K42/G42,"")</x:f>
+      </x:c>
+      <x:c r="N42" s="45"/>
     </x:row>
     <x:row r="43" ht="20" customHeight="1">
       <x:c r="A43" s="19" t="n">
@@ -1413,13 +1768,19 @@
       <x:c r="E43" s="19" t="n">
         <x:v>3584</x:v>
       </x:c>
-      <x:c r="F43" s="22" t="str"/>
-      <x:c r="G43" s="23"/>
-      <x:c r="H43" s="22" t="str"/>
-      <x:c r="I43" s="23"/>
-      <x:c r="J43" s="21" t="str">
+      <x:c r="F43" s="43" t="str"/>
+      <x:c r="G43" s="44"/>
+      <x:c r="H43" s="45" t="str"/>
+      <x:c r="I43" s="46"/>
+      <x:c r="J43" s="47"/>
+      <x:c r="K43" s="50"/>
+      <x:c r="L43" s="51" t="str">
         <x:f>IFERROR(I43/G43,"")</x:f>
       </x:c>
+      <x:c r="M43" s="51" t="str">
+        <x:f>IFERROR(K43/G43,"")</x:f>
+      </x:c>
+      <x:c r="N43" s="45"/>
     </x:row>
     <x:row r="44" ht="20" customHeight="1">
       <x:c r="A44" s="19" t="n">
@@ -1437,13 +1798,19 @@
       <x:c r="E44" s="19" t="n">
         <x:v>3584</x:v>
       </x:c>
-      <x:c r="F44" s="22" t="str"/>
-      <x:c r="G44" s="23"/>
-      <x:c r="H44" s="22" t="str"/>
-      <x:c r="I44" s="23"/>
-      <x:c r="J44" s="21" t="str">
+      <x:c r="F44" s="43" t="str"/>
+      <x:c r="G44" s="44"/>
+      <x:c r="H44" s="45" t="str"/>
+      <x:c r="I44" s="46"/>
+      <x:c r="J44" s="47"/>
+      <x:c r="K44" s="50"/>
+      <x:c r="L44" s="51" t="str">
         <x:f>IFERROR(I44/G44,"")</x:f>
       </x:c>
+      <x:c r="M44" s="51" t="str">
+        <x:f>IFERROR(K44/G44,"")</x:f>
+      </x:c>
+      <x:c r="N44" s="45"/>
     </x:row>
     <x:row r="45" ht="20" customHeight="1">
       <x:c r="A45" s="19" t="n">
@@ -1461,13 +1828,19 @@
       <x:c r="E45" s="19" t="n">
         <x:v>128</x:v>
       </x:c>
-      <x:c r="F45" s="22" t="str"/>
-      <x:c r="G45" s="23"/>
-      <x:c r="H45" s="22" t="str"/>
-      <x:c r="I45" s="23"/>
-      <x:c r="J45" s="21" t="str">
+      <x:c r="F45" s="43" t="str"/>
+      <x:c r="G45" s="44"/>
+      <x:c r="H45" s="45" t="str"/>
+      <x:c r="I45" s="46"/>
+      <x:c r="J45" s="47"/>
+      <x:c r="K45" s="50"/>
+      <x:c r="L45" s="51" t="str">
         <x:f>IFERROR(I45/G45,"")</x:f>
       </x:c>
+      <x:c r="M45" s="51" t="str">
+        <x:f>IFERROR(K45/G45,"")</x:f>
+      </x:c>
+      <x:c r="N45" s="45"/>
     </x:row>
     <x:row r="46" ht="20" customHeight="1">
       <x:c r="A46" s="19" t="n">
@@ -1485,13 +1858,19 @@
       <x:c r="E46" s="19" t="n">
         <x:v>2048</x:v>
       </x:c>
-      <x:c r="F46" s="22" t="str"/>
-      <x:c r="G46" s="23"/>
-      <x:c r="H46" s="22" t="str"/>
-      <x:c r="I46" s="23"/>
-      <x:c r="J46" s="21" t="str">
+      <x:c r="F46" s="43" t="str"/>
+      <x:c r="G46" s="44"/>
+      <x:c r="H46" s="45" t="str"/>
+      <x:c r="I46" s="46"/>
+      <x:c r="J46" s="47"/>
+      <x:c r="K46" s="50"/>
+      <x:c r="L46" s="51" t="str">
         <x:f>IFERROR(I46/G46,"")</x:f>
       </x:c>
+      <x:c r="M46" s="51" t="str">
+        <x:f>IFERROR(K46/G46,"")</x:f>
+      </x:c>
+      <x:c r="N46" s="45"/>
     </x:row>
     <x:row r="47" ht="20" customHeight="1">
       <x:c r="A47" s="19" t="n">
@@ -1509,13 +1888,19 @@
       <x:c r="E47" s="19" t="n">
         <x:v>3584</x:v>
       </x:c>
-      <x:c r="F47" s="22" t="str"/>
-      <x:c r="G47" s="23"/>
-      <x:c r="H47" s="22" t="str"/>
-      <x:c r="I47" s="23"/>
-      <x:c r="J47" s="21" t="str">
+      <x:c r="F47" s="43" t="str"/>
+      <x:c r="G47" s="44"/>
+      <x:c r="H47" s="45" t="str"/>
+      <x:c r="I47" s="46"/>
+      <x:c r="J47" s="47"/>
+      <x:c r="K47" s="50"/>
+      <x:c r="L47" s="51" t="str">
         <x:f>IFERROR(I47/G47,"")</x:f>
       </x:c>
+      <x:c r="M47" s="51" t="str">
+        <x:f>IFERROR(K47/G47,"")</x:f>
+      </x:c>
+      <x:c r="N47" s="45"/>
     </x:row>
     <x:row r="48" ht="20" customHeight="1">
       <x:c r="A48" s="19" t="n">
@@ -1533,13 +1918,19 @@
       <x:c r="E48" s="19" t="n">
         <x:v>3584</x:v>
       </x:c>
-      <x:c r="F48" s="22" t="str"/>
-      <x:c r="G48" s="23"/>
-      <x:c r="H48" s="22" t="str"/>
-      <x:c r="I48" s="23"/>
-      <x:c r="J48" s="21" t="str">
+      <x:c r="F48" s="43" t="str"/>
+      <x:c r="G48" s="44"/>
+      <x:c r="H48" s="45" t="str"/>
+      <x:c r="I48" s="46"/>
+      <x:c r="J48" s="47"/>
+      <x:c r="K48" s="50"/>
+      <x:c r="L48" s="51" t="str">
         <x:f>IFERROR(I48/G48,"")</x:f>
       </x:c>
+      <x:c r="M48" s="51" t="str">
+        <x:f>IFERROR(K48/G48,"")</x:f>
+      </x:c>
+      <x:c r="N48" s="45"/>
     </x:row>
     <x:row r="49" ht="20" customHeight="1">
       <x:c r="A49" s="19" t="n">
@@ -1557,13 +1948,19 @@
       <x:c r="E49" s="19" t="n">
         <x:v>18944</x:v>
       </x:c>
-      <x:c r="F49" s="22" t="str"/>
-      <x:c r="G49" s="23"/>
-      <x:c r="H49" s="22" t="str"/>
-      <x:c r="I49" s="23"/>
-      <x:c r="J49" s="21" t="str">
+      <x:c r="F49" s="43" t="str"/>
+      <x:c r="G49" s="44"/>
+      <x:c r="H49" s="45" t="str"/>
+      <x:c r="I49" s="46"/>
+      <x:c r="J49" s="47"/>
+      <x:c r="K49" s="50"/>
+      <x:c r="L49" s="51" t="str">
         <x:f>IFERROR(I49/G49,"")</x:f>
       </x:c>
+      <x:c r="M49" s="51" t="str">
+        <x:f>IFERROR(K49/G49,"")</x:f>
+      </x:c>
+      <x:c r="N49" s="45"/>
     </x:row>
     <x:row r="50" ht="20" customHeight="1">
       <x:c r="A50" s="19" t="n">
@@ -1581,18 +1978,24 @@
       <x:c r="E50" s="19" t="n">
         <x:v>3584</x:v>
       </x:c>
-      <x:c r="F50" s="22" t="str"/>
-      <x:c r="G50" s="23"/>
-      <x:c r="H50" s="22" t="str"/>
-      <x:c r="I50" s="23"/>
-      <x:c r="J50" s="21" t="str">
+      <x:c r="F50" s="43" t="str"/>
+      <x:c r="G50" s="44"/>
+      <x:c r="H50" s="45" t="str"/>
+      <x:c r="I50" s="46"/>
+      <x:c r="J50" s="47"/>
+      <x:c r="K50" s="50"/>
+      <x:c r="L50" s="51" t="str">
         <x:f>IFERROR(I50/G50,"")</x:f>
       </x:c>
+      <x:c r="M50" s="51" t="str">
+        <x:f>IFERROR(K50/G50,"")</x:f>
+      </x:c>
+      <x:c r="N50" s="45"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:J1"/>
-    <x:mergeCell ref="A3:J3"/>
+    <x:mergeCell ref="A1:N1"/>
+    <x:mergeCell ref="A3:N3"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="J6:J50">
     <x:cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
@@ -1604,7 +2007,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa81dc51d8874039"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02fb5cfa4e304eb9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add cuBLASLt-guided Qwen GEMM tuning
</commit_message>
<xml_diff>
--- a/gemm_performance_comparison.xlsx
+++ b/gemm_performance_comparison.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="环境对比" sheetId="1" r:id="Re0859d10a8a64bca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="环境对比" sheetId="1" r:id="Ra25625ebaeb74763"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -197,9 +197,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="GemmComparison" displayName="GemmComparison" ref="A5:L19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="GemmComparison" displayName="GemmComparison" ref="A5:L81" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
-    <x:tableColumn id="1" name="相关 L"/>
+    <x:tableColumn id="1" name="阶段/相关长度"/>
     <x:tableColumn id="2" name="来源算子"/>
     <x:tableColumn id="3" name="M"/>
     <x:tableColumn id="4" name="N"/>
@@ -411,7 +411,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="10" hidden="0" customWidth="1"/>
@@ -427,7 +427,7 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>Qwen2.5 Decode GEMM 性能对比</x:v>
+        <x:v>Qwen2.5 Decode + Prefill GEMM 性能对比</x:v>
       </x:c>
       <x:c r="B1" s="3"/>
       <x:c r="C1" s="3"/>
@@ -449,16 +449,16 @@
         <x:v>Qwen2.5-7B</x:v>
       </x:c>
       <x:c r="C2" s="7" t="str">
-        <x:v>Decode Batch</x:v>
+        <x:v>Batch</x:v>
       </x:c>
       <x:c r="D2" s="7" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E2" s="7" t="str">
-        <x:v>上下文长度</x:v>
+        <x:v>阶段</x:v>
       </x:c>
       <x:c r="F2" s="7" t="str">
-        <x:v>128, 256, 512, 1024, 2048</x:v>
+        <x:v>Decode + Prefill</x:v>
       </x:c>
       <x:c r="G2" s="7" t="str">
         <x:v>CUTLASS来源</x:v>
@@ -481,7 +481,7 @@
     </x:row>
     <x:row r="3" ht="42" customHeight="1">
       <x:c r="A3" s="35" t="str">
-        <x:v>使用方法：Decode GEMM 严格按 M/N/K 去重；“-”表示该 GEMM 与 L 无关。运行 run_gemm.sh 保存 CUTLASS 日志，再用 collect_gemm_results.py 回填；两类 HGEMM 请按相同 M/N/K 人工筛选。</x:v>
+        <x:v>使用方法：Decode 与 Prefill GEMM 严格按 M/N/K 去重；L/S=- 表示与长度无关。运行 run_gemm.sh 保存 CUTLASS 日志，再用 collect_gemm_results.py 回填；两类 HGEMM 请按相同 M/N/K 人工筛选。</x:v>
       </x:c>
       <x:c r="B3" s="35"/>
       <x:c r="C3" s="35"/>
@@ -498,7 +498,7 @@
     <x:row r="4" ht="8" customHeight="1"/>
     <x:row r="5">
       <x:c r="A5" s="22" t="str">
-        <x:v>相关 L</x:v>
+        <x:v>阶段/相关长度</x:v>
       </x:c>
       <x:c r="B5" s="22" t="str">
         <x:v>来源算子</x:v>
@@ -536,7 +536,7 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="22" t="str">
-        <x:v>-</x:v>
+        <x:v>Decode L=-</x:v>
       </x:c>
       <x:c r="B6" s="22" t="str">
         <x:v>Q / Attention Out</x:v>
@@ -564,7 +564,7 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="22" t="str">
-        <x:v>-</x:v>
+        <x:v>Decode L=-</x:v>
       </x:c>
       <x:c r="B7" s="22" t="str">
         <x:v>K / V</x:v>
@@ -592,7 +592,7 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="22" t="str">
-        <x:v>-</x:v>
+        <x:v>Decode L=-</x:v>
       </x:c>
       <x:c r="B8" s="22" t="str">
         <x:v>MLP Up/Gate</x:v>
@@ -620,7 +620,7 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="22" t="str">
-        <x:v>-</x:v>
+        <x:v>Decode L=-</x:v>
       </x:c>
       <x:c r="B9" s="22" t="str">
         <x:v>MLP Down</x:v>
@@ -648,7 +648,7 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="22" t="str">
-        <x:v>-</x:v>
+        <x:v>Decode L=-</x:v>
       </x:c>
       <x:c r="B10" s="22" t="str">
         <x:v>LM Head</x:v>
@@ -676,7 +676,7 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="22" t="str">
-        <x:v>128</x:v>
+        <x:v>Decode L=128</x:v>
       </x:c>
       <x:c r="B11" s="22" t="str">
         <x:v>Attention QK^T / Attention AV</x:v>
@@ -704,7 +704,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="22" t="str">
-        <x:v>256</x:v>
+        <x:v>Decode L=256</x:v>
       </x:c>
       <x:c r="B12" s="22" t="str">
         <x:v>Attention QK^T</x:v>
@@ -732,7 +732,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="22" t="str">
-        <x:v>256</x:v>
+        <x:v>Decode L=256</x:v>
       </x:c>
       <x:c r="B13" s="22" t="str">
         <x:v>Attention AV</x:v>
@@ -760,7 +760,7 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="22" t="str">
-        <x:v>512</x:v>
+        <x:v>Decode L=512</x:v>
       </x:c>
       <x:c r="B14" s="22" t="str">
         <x:v>Attention QK^T</x:v>
@@ -788,7 +788,7 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="22" t="str">
-        <x:v>512</x:v>
+        <x:v>Decode L=512</x:v>
       </x:c>
       <x:c r="B15" s="22" t="str">
         <x:v>Attention AV</x:v>
@@ -816,7 +816,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="22" t="str">
-        <x:v>1024</x:v>
+        <x:v>Decode L=1024</x:v>
       </x:c>
       <x:c r="B16" s="22" t="str">
         <x:v>Attention QK^T</x:v>
@@ -844,7 +844,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="22" t="str">
-        <x:v>1024</x:v>
+        <x:v>Decode L=1024</x:v>
       </x:c>
       <x:c r="B17" s="22" t="str">
         <x:v>Attention AV</x:v>
@@ -872,7 +872,7 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="22" t="str">
-        <x:v>2048</x:v>
+        <x:v>Decode L=2048</x:v>
       </x:c>
       <x:c r="B18" s="22" t="str">
         <x:v>Attention QK^T</x:v>
@@ -900,7 +900,7 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="22" t="str">
-        <x:v>2048</x:v>
+        <x:v>Decode L=2048</x:v>
       </x:c>
       <x:c r="B19" s="22" t="str">
         <x:v>Attention AV</x:v>
@@ -925,6 +925,1742 @@
         <x:f>IFERROR(I19/G19,"")</x:f>
       </x:c>
       <x:c r="L19" s="28"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="22" t="str">
+        <x:v>Prefill S=128</x:v>
+      </x:c>
+      <x:c r="B20" s="22" t="str">
+        <x:v>Q / Attention Out</x:v>
+      </x:c>
+      <x:c r="C20" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="D20" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="E20" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F20" s="27"/>
+      <x:c r="G20" s="31"/>
+      <x:c r="H20" s="32"/>
+      <x:c r="I20" s="33"/>
+      <x:c r="J20" s="34" t="str">
+        <x:f>IFERROR(H20/G20,"")</x:f>
+      </x:c>
+      <x:c r="K20" s="34" t="str">
+        <x:f>IFERROR(I20/G20,"")</x:f>
+      </x:c>
+      <x:c r="L20" s="28"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="22" t="str">
+        <x:v>Prefill S=128</x:v>
+      </x:c>
+      <x:c r="B21" s="22" t="str">
+        <x:v>K / V</x:v>
+      </x:c>
+      <x:c r="C21" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="D21" s="22" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="E21" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F21" s="27"/>
+      <x:c r="G21" s="31"/>
+      <x:c r="H21" s="32"/>
+      <x:c r="I21" s="33"/>
+      <x:c r="J21" s="34" t="str">
+        <x:f>IFERROR(H21/G21,"")</x:f>
+      </x:c>
+      <x:c r="K21" s="34" t="str">
+        <x:f>IFERROR(I21/G21,"")</x:f>
+      </x:c>
+      <x:c r="L21" s="28"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="22" t="str">
+        <x:v>Prefill S=128</x:v>
+      </x:c>
+      <x:c r="B22" s="22" t="str">
+        <x:v>MLP Up/Gate</x:v>
+      </x:c>
+      <x:c r="C22" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="D22" s="22" t="n">
+        <x:v>37888</x:v>
+      </x:c>
+      <x:c r="E22" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F22" s="27"/>
+      <x:c r="G22" s="31"/>
+      <x:c r="H22" s="32"/>
+      <x:c r="I22" s="33"/>
+      <x:c r="J22" s="34" t="str">
+        <x:f>IFERROR(H22/G22,"")</x:f>
+      </x:c>
+      <x:c r="K22" s="34" t="str">
+        <x:f>IFERROR(I22/G22,"")</x:f>
+      </x:c>
+      <x:c r="L22" s="28"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="22" t="str">
+        <x:v>Prefill S=128</x:v>
+      </x:c>
+      <x:c r="B23" s="22" t="str">
+        <x:v>MLP Down</x:v>
+      </x:c>
+      <x:c r="C23" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="D23" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="E23" s="22" t="n">
+        <x:v>18944</x:v>
+      </x:c>
+      <x:c r="F23" s="27"/>
+      <x:c r="G23" s="31"/>
+      <x:c r="H23" s="32"/>
+      <x:c r="I23" s="33"/>
+      <x:c r="J23" s="34" t="str">
+        <x:f>IFERROR(H23/G23,"")</x:f>
+      </x:c>
+      <x:c r="K23" s="34" t="str">
+        <x:f>IFERROR(I23/G23,"")</x:f>
+      </x:c>
+      <x:c r="L23" s="28"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="22" t="str">
+        <x:v>Prefill S=128</x:v>
+      </x:c>
+      <x:c r="B24" s="22" t="str">
+        <x:v>LM Head</x:v>
+      </x:c>
+      <x:c r="C24" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="D24" s="22" t="n">
+        <x:v>152064</x:v>
+      </x:c>
+      <x:c r="E24" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F24" s="27"/>
+      <x:c r="G24" s="31"/>
+      <x:c r="H24" s="32"/>
+      <x:c r="I24" s="33"/>
+      <x:c r="J24" s="34" t="str">
+        <x:f>IFERROR(H24/G24,"")</x:f>
+      </x:c>
+      <x:c r="K24" s="34" t="str">
+        <x:f>IFERROR(I24/G24,"")</x:f>
+      </x:c>
+      <x:c r="L24" s="28"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="22" t="str">
+        <x:v>Prefill S=128</x:v>
+      </x:c>
+      <x:c r="B25" s="22" t="str">
+        <x:v>Attention QK^T / Attention AV</x:v>
+      </x:c>
+      <x:c r="C25" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="D25" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="E25" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="F25" s="27"/>
+      <x:c r="G25" s="31"/>
+      <x:c r="H25" s="32"/>
+      <x:c r="I25" s="33"/>
+      <x:c r="J25" s="34" t="str">
+        <x:f>IFERROR(H25/G25,"")</x:f>
+      </x:c>
+      <x:c r="K25" s="34" t="str">
+        <x:f>IFERROR(I25/G25,"")</x:f>
+      </x:c>
+      <x:c r="L25" s="28"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="22" t="str">
+        <x:v>Prefill S=256</x:v>
+      </x:c>
+      <x:c r="B26" s="22" t="str">
+        <x:v>Q / Attention Out</x:v>
+      </x:c>
+      <x:c r="C26" s="22" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="D26" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="E26" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F26" s="27"/>
+      <x:c r="G26" s="31"/>
+      <x:c r="H26" s="32"/>
+      <x:c r="I26" s="33"/>
+      <x:c r="J26" s="34" t="str">
+        <x:f>IFERROR(H26/G26,"")</x:f>
+      </x:c>
+      <x:c r="K26" s="34" t="str">
+        <x:f>IFERROR(I26/G26,"")</x:f>
+      </x:c>
+      <x:c r="L26" s="28"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="22" t="str">
+        <x:v>Prefill S=256</x:v>
+      </x:c>
+      <x:c r="B27" s="22" t="str">
+        <x:v>K / V</x:v>
+      </x:c>
+      <x:c r="C27" s="22" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="D27" s="22" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="E27" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F27" s="27"/>
+      <x:c r="G27" s="31"/>
+      <x:c r="H27" s="32"/>
+      <x:c r="I27" s="33"/>
+      <x:c r="J27" s="34" t="str">
+        <x:f>IFERROR(H27/G27,"")</x:f>
+      </x:c>
+      <x:c r="K27" s="34" t="str">
+        <x:f>IFERROR(I27/G27,"")</x:f>
+      </x:c>
+      <x:c r="L27" s="28"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="22" t="str">
+        <x:v>Prefill S=256</x:v>
+      </x:c>
+      <x:c r="B28" s="22" t="str">
+        <x:v>MLP Up/Gate</x:v>
+      </x:c>
+      <x:c r="C28" s="22" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="D28" s="22" t="n">
+        <x:v>37888</x:v>
+      </x:c>
+      <x:c r="E28" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F28" s="27"/>
+      <x:c r="G28" s="31"/>
+      <x:c r="H28" s="32"/>
+      <x:c r="I28" s="33"/>
+      <x:c r="J28" s="34" t="str">
+        <x:f>IFERROR(H28/G28,"")</x:f>
+      </x:c>
+      <x:c r="K28" s="34" t="str">
+        <x:f>IFERROR(I28/G28,"")</x:f>
+      </x:c>
+      <x:c r="L28" s="28"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="22" t="str">
+        <x:v>Prefill S=256</x:v>
+      </x:c>
+      <x:c r="B29" s="22" t="str">
+        <x:v>MLP Down</x:v>
+      </x:c>
+      <x:c r="C29" s="22" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="D29" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="E29" s="22" t="n">
+        <x:v>18944</x:v>
+      </x:c>
+      <x:c r="F29" s="27"/>
+      <x:c r="G29" s="31"/>
+      <x:c r="H29" s="32"/>
+      <x:c r="I29" s="33"/>
+      <x:c r="J29" s="34" t="str">
+        <x:f>IFERROR(H29/G29,"")</x:f>
+      </x:c>
+      <x:c r="K29" s="34" t="str">
+        <x:f>IFERROR(I29/G29,"")</x:f>
+      </x:c>
+      <x:c r="L29" s="28"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="22" t="str">
+        <x:v>Prefill S=256</x:v>
+      </x:c>
+      <x:c r="B30" s="22" t="str">
+        <x:v>LM Head</x:v>
+      </x:c>
+      <x:c r="C30" s="22" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="D30" s="22" t="n">
+        <x:v>152064</x:v>
+      </x:c>
+      <x:c r="E30" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F30" s="27"/>
+      <x:c r="G30" s="31"/>
+      <x:c r="H30" s="32"/>
+      <x:c r="I30" s="33"/>
+      <x:c r="J30" s="34" t="str">
+        <x:f>IFERROR(H30/G30,"")</x:f>
+      </x:c>
+      <x:c r="K30" s="34" t="str">
+        <x:f>IFERROR(I30/G30,"")</x:f>
+      </x:c>
+      <x:c r="L30" s="28"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="22" t="str">
+        <x:v>Prefill S=256</x:v>
+      </x:c>
+      <x:c r="B31" s="22" t="str">
+        <x:v>Attention QK^T</x:v>
+      </x:c>
+      <x:c r="C31" s="22" t="n">
+        <x:v>7168</x:v>
+      </x:c>
+      <x:c r="D31" s="22" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="E31" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="F31" s="27"/>
+      <x:c r="G31" s="31"/>
+      <x:c r="H31" s="32"/>
+      <x:c r="I31" s="33"/>
+      <x:c r="J31" s="34" t="str">
+        <x:f>IFERROR(H31/G31,"")</x:f>
+      </x:c>
+      <x:c r="K31" s="34" t="str">
+        <x:f>IFERROR(I31/G31,"")</x:f>
+      </x:c>
+      <x:c r="L31" s="28"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="22" t="str">
+        <x:v>Prefill S=256</x:v>
+      </x:c>
+      <x:c r="B32" s="22" t="str">
+        <x:v>Attention AV</x:v>
+      </x:c>
+      <x:c r="C32" s="22" t="n">
+        <x:v>7168</x:v>
+      </x:c>
+      <x:c r="D32" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="E32" s="22" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="F32" s="27"/>
+      <x:c r="G32" s="31"/>
+      <x:c r="H32" s="32"/>
+      <x:c r="I32" s="33"/>
+      <x:c r="J32" s="34" t="str">
+        <x:f>IFERROR(H32/G32,"")</x:f>
+      </x:c>
+      <x:c r="K32" s="34" t="str">
+        <x:f>IFERROR(I32/G32,"")</x:f>
+      </x:c>
+      <x:c r="L32" s="28"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="22" t="str">
+        <x:v>Prefill S=512</x:v>
+      </x:c>
+      <x:c r="B33" s="22" t="str">
+        <x:v>Q / Attention Out</x:v>
+      </x:c>
+      <x:c r="C33" s="22" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="D33" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="E33" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F33" s="27"/>
+      <x:c r="G33" s="31"/>
+      <x:c r="H33" s="32"/>
+      <x:c r="I33" s="33"/>
+      <x:c r="J33" s="34" t="str">
+        <x:f>IFERROR(H33/G33,"")</x:f>
+      </x:c>
+      <x:c r="K33" s="34" t="str">
+        <x:f>IFERROR(I33/G33,"")</x:f>
+      </x:c>
+      <x:c r="L33" s="28"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="22" t="str">
+        <x:v>Prefill S=512</x:v>
+      </x:c>
+      <x:c r="B34" s="22" t="str">
+        <x:v>K / V</x:v>
+      </x:c>
+      <x:c r="C34" s="22" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="D34" s="22" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="E34" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F34" s="27"/>
+      <x:c r="G34" s="31"/>
+      <x:c r="H34" s="32"/>
+      <x:c r="I34" s="33"/>
+      <x:c r="J34" s="34" t="str">
+        <x:f>IFERROR(H34/G34,"")</x:f>
+      </x:c>
+      <x:c r="K34" s="34" t="str">
+        <x:f>IFERROR(I34/G34,"")</x:f>
+      </x:c>
+      <x:c r="L34" s="28"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="22" t="str">
+        <x:v>Prefill S=512</x:v>
+      </x:c>
+      <x:c r="B35" s="22" t="str">
+        <x:v>MLP Up/Gate</x:v>
+      </x:c>
+      <x:c r="C35" s="22" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="D35" s="22" t="n">
+        <x:v>37888</x:v>
+      </x:c>
+      <x:c r="E35" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F35" s="27"/>
+      <x:c r="G35" s="31"/>
+      <x:c r="H35" s="32"/>
+      <x:c r="I35" s="33"/>
+      <x:c r="J35" s="34" t="str">
+        <x:f>IFERROR(H35/G35,"")</x:f>
+      </x:c>
+      <x:c r="K35" s="34" t="str">
+        <x:f>IFERROR(I35/G35,"")</x:f>
+      </x:c>
+      <x:c r="L35" s="28"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="22" t="str">
+        <x:v>Prefill S=512</x:v>
+      </x:c>
+      <x:c r="B36" s="22" t="str">
+        <x:v>MLP Down</x:v>
+      </x:c>
+      <x:c r="C36" s="22" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="D36" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="E36" s="22" t="n">
+        <x:v>18944</x:v>
+      </x:c>
+      <x:c r="F36" s="27"/>
+      <x:c r="G36" s="31"/>
+      <x:c r="H36" s="32"/>
+      <x:c r="I36" s="33"/>
+      <x:c r="J36" s="34" t="str">
+        <x:f>IFERROR(H36/G36,"")</x:f>
+      </x:c>
+      <x:c r="K36" s="34" t="str">
+        <x:f>IFERROR(I36/G36,"")</x:f>
+      </x:c>
+      <x:c r="L36" s="28"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="22" t="str">
+        <x:v>Prefill S=512</x:v>
+      </x:c>
+      <x:c r="B37" s="22" t="str">
+        <x:v>LM Head</x:v>
+      </x:c>
+      <x:c r="C37" s="22" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="D37" s="22" t="n">
+        <x:v>152064</x:v>
+      </x:c>
+      <x:c r="E37" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F37" s="27"/>
+      <x:c r="G37" s="31"/>
+      <x:c r="H37" s="32"/>
+      <x:c r="I37" s="33"/>
+      <x:c r="J37" s="34" t="str">
+        <x:f>IFERROR(H37/G37,"")</x:f>
+      </x:c>
+      <x:c r="K37" s="34" t="str">
+        <x:f>IFERROR(I37/G37,"")</x:f>
+      </x:c>
+      <x:c r="L37" s="28"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="22" t="str">
+        <x:v>Prefill S=512</x:v>
+      </x:c>
+      <x:c r="B38" s="22" t="str">
+        <x:v>Attention QK^T</x:v>
+      </x:c>
+      <x:c r="C38" s="22" t="n">
+        <x:v>14336</x:v>
+      </x:c>
+      <x:c r="D38" s="22" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="E38" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="F38" s="27"/>
+      <x:c r="G38" s="31"/>
+      <x:c r="H38" s="32"/>
+      <x:c r="I38" s="33"/>
+      <x:c r="J38" s="34" t="str">
+        <x:f>IFERROR(H38/G38,"")</x:f>
+      </x:c>
+      <x:c r="K38" s="34" t="str">
+        <x:f>IFERROR(I38/G38,"")</x:f>
+      </x:c>
+      <x:c r="L38" s="28"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="22" t="str">
+        <x:v>Prefill S=512</x:v>
+      </x:c>
+      <x:c r="B39" s="22" t="str">
+        <x:v>Attention AV</x:v>
+      </x:c>
+      <x:c r="C39" s="22" t="n">
+        <x:v>14336</x:v>
+      </x:c>
+      <x:c r="D39" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="E39" s="22" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="F39" s="27"/>
+      <x:c r="G39" s="31"/>
+      <x:c r="H39" s="32"/>
+      <x:c r="I39" s="33"/>
+      <x:c r="J39" s="34" t="str">
+        <x:f>IFERROR(H39/G39,"")</x:f>
+      </x:c>
+      <x:c r="K39" s="34" t="str">
+        <x:f>IFERROR(I39/G39,"")</x:f>
+      </x:c>
+      <x:c r="L39" s="28"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="22" t="str">
+        <x:v>Prefill S=1024</x:v>
+      </x:c>
+      <x:c r="B40" s="22" t="str">
+        <x:v>Q / Attention Out</x:v>
+      </x:c>
+      <x:c r="C40" s="22" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="D40" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="E40" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F40" s="27"/>
+      <x:c r="G40" s="31"/>
+      <x:c r="H40" s="32"/>
+      <x:c r="I40" s="33"/>
+      <x:c r="J40" s="34" t="str">
+        <x:f>IFERROR(H40/G40,"")</x:f>
+      </x:c>
+      <x:c r="K40" s="34" t="str">
+        <x:f>IFERROR(I40/G40,"")</x:f>
+      </x:c>
+      <x:c r="L40" s="28"/>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="22" t="str">
+        <x:v>Prefill S=1024</x:v>
+      </x:c>
+      <x:c r="B41" s="22" t="str">
+        <x:v>K / V</x:v>
+      </x:c>
+      <x:c r="C41" s="22" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="D41" s="22" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="E41" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F41" s="27"/>
+      <x:c r="G41" s="31"/>
+      <x:c r="H41" s="32"/>
+      <x:c r="I41" s="33"/>
+      <x:c r="J41" s="34" t="str">
+        <x:f>IFERROR(H41/G41,"")</x:f>
+      </x:c>
+      <x:c r="K41" s="34" t="str">
+        <x:f>IFERROR(I41/G41,"")</x:f>
+      </x:c>
+      <x:c r="L41" s="28"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="22" t="str">
+        <x:v>Prefill S=1024</x:v>
+      </x:c>
+      <x:c r="B42" s="22" t="str">
+        <x:v>MLP Up/Gate</x:v>
+      </x:c>
+      <x:c r="C42" s="22" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="D42" s="22" t="n">
+        <x:v>37888</x:v>
+      </x:c>
+      <x:c r="E42" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F42" s="27"/>
+      <x:c r="G42" s="31"/>
+      <x:c r="H42" s="32"/>
+      <x:c r="I42" s="33"/>
+      <x:c r="J42" s="34" t="str">
+        <x:f>IFERROR(H42/G42,"")</x:f>
+      </x:c>
+      <x:c r="K42" s="34" t="str">
+        <x:f>IFERROR(I42/G42,"")</x:f>
+      </x:c>
+      <x:c r="L42" s="28"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="22" t="str">
+        <x:v>Prefill S=1024</x:v>
+      </x:c>
+      <x:c r="B43" s="22" t="str">
+        <x:v>MLP Down</x:v>
+      </x:c>
+      <x:c r="C43" s="22" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="D43" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="E43" s="22" t="n">
+        <x:v>18944</x:v>
+      </x:c>
+      <x:c r="F43" s="27"/>
+      <x:c r="G43" s="31"/>
+      <x:c r="H43" s="32"/>
+      <x:c r="I43" s="33"/>
+      <x:c r="J43" s="34" t="str">
+        <x:f>IFERROR(H43/G43,"")</x:f>
+      </x:c>
+      <x:c r="K43" s="34" t="str">
+        <x:f>IFERROR(I43/G43,"")</x:f>
+      </x:c>
+      <x:c r="L43" s="28"/>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="22" t="str">
+        <x:v>Prefill S=1024</x:v>
+      </x:c>
+      <x:c r="B44" s="22" t="str">
+        <x:v>LM Head</x:v>
+      </x:c>
+      <x:c r="C44" s="22" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="D44" s="22" t="n">
+        <x:v>152064</x:v>
+      </x:c>
+      <x:c r="E44" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F44" s="27"/>
+      <x:c r="G44" s="31"/>
+      <x:c r="H44" s="32"/>
+      <x:c r="I44" s="33"/>
+      <x:c r="J44" s="34" t="str">
+        <x:f>IFERROR(H44/G44,"")</x:f>
+      </x:c>
+      <x:c r="K44" s="34" t="str">
+        <x:f>IFERROR(I44/G44,"")</x:f>
+      </x:c>
+      <x:c r="L44" s="28"/>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="22" t="str">
+        <x:v>Prefill S=1024</x:v>
+      </x:c>
+      <x:c r="B45" s="22" t="str">
+        <x:v>Attention QK^T</x:v>
+      </x:c>
+      <x:c r="C45" s="22" t="n">
+        <x:v>28672</x:v>
+      </x:c>
+      <x:c r="D45" s="22" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="E45" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="F45" s="27"/>
+      <x:c r="G45" s="31"/>
+      <x:c r="H45" s="32"/>
+      <x:c r="I45" s="33"/>
+      <x:c r="J45" s="34" t="str">
+        <x:f>IFERROR(H45/G45,"")</x:f>
+      </x:c>
+      <x:c r="K45" s="34" t="str">
+        <x:f>IFERROR(I45/G45,"")</x:f>
+      </x:c>
+      <x:c r="L45" s="28"/>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="22" t="str">
+        <x:v>Prefill S=1024</x:v>
+      </x:c>
+      <x:c r="B46" s="22" t="str">
+        <x:v>Attention AV</x:v>
+      </x:c>
+      <x:c r="C46" s="22" t="n">
+        <x:v>28672</x:v>
+      </x:c>
+      <x:c r="D46" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="E46" s="22" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="F46" s="27"/>
+      <x:c r="G46" s="31"/>
+      <x:c r="H46" s="32"/>
+      <x:c r="I46" s="33"/>
+      <x:c r="J46" s="34" t="str">
+        <x:f>IFERROR(H46/G46,"")</x:f>
+      </x:c>
+      <x:c r="K46" s="34" t="str">
+        <x:f>IFERROR(I46/G46,"")</x:f>
+      </x:c>
+      <x:c r="L46" s="28"/>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="22" t="str">
+        <x:v>Prefill S=2048</x:v>
+      </x:c>
+      <x:c r="B47" s="22" t="str">
+        <x:v>Q / Attention Out</x:v>
+      </x:c>
+      <x:c r="C47" s="22" t="n">
+        <x:v>2048</x:v>
+      </x:c>
+      <x:c r="D47" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="E47" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F47" s="27"/>
+      <x:c r="G47" s="31"/>
+      <x:c r="H47" s="32"/>
+      <x:c r="I47" s="33"/>
+      <x:c r="J47" s="34" t="str">
+        <x:f>IFERROR(H47/G47,"")</x:f>
+      </x:c>
+      <x:c r="K47" s="34" t="str">
+        <x:f>IFERROR(I47/G47,"")</x:f>
+      </x:c>
+      <x:c r="L47" s="28"/>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="22" t="str">
+        <x:v>Prefill S=2048</x:v>
+      </x:c>
+      <x:c r="B48" s="22" t="str">
+        <x:v>K / V</x:v>
+      </x:c>
+      <x:c r="C48" s="22" t="n">
+        <x:v>2048</x:v>
+      </x:c>
+      <x:c r="D48" s="22" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="E48" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F48" s="27"/>
+      <x:c r="G48" s="31"/>
+      <x:c r="H48" s="32"/>
+      <x:c r="I48" s="33"/>
+      <x:c r="J48" s="34" t="str">
+        <x:f>IFERROR(H48/G48,"")</x:f>
+      </x:c>
+      <x:c r="K48" s="34" t="str">
+        <x:f>IFERROR(I48/G48,"")</x:f>
+      </x:c>
+      <x:c r="L48" s="28"/>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="22" t="str">
+        <x:v>Prefill S=2048</x:v>
+      </x:c>
+      <x:c r="B49" s="22" t="str">
+        <x:v>MLP Up/Gate</x:v>
+      </x:c>
+      <x:c r="C49" s="22" t="n">
+        <x:v>2048</x:v>
+      </x:c>
+      <x:c r="D49" s="22" t="n">
+        <x:v>37888</x:v>
+      </x:c>
+      <x:c r="E49" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F49" s="27"/>
+      <x:c r="G49" s="31"/>
+      <x:c r="H49" s="32"/>
+      <x:c r="I49" s="33"/>
+      <x:c r="J49" s="34" t="str">
+        <x:f>IFERROR(H49/G49,"")</x:f>
+      </x:c>
+      <x:c r="K49" s="34" t="str">
+        <x:f>IFERROR(I49/G49,"")</x:f>
+      </x:c>
+      <x:c r="L49" s="28"/>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="22" t="str">
+        <x:v>Prefill S=2048</x:v>
+      </x:c>
+      <x:c r="B50" s="22" t="str">
+        <x:v>MLP Down</x:v>
+      </x:c>
+      <x:c r="C50" s="22" t="n">
+        <x:v>2048</x:v>
+      </x:c>
+      <x:c r="D50" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="E50" s="22" t="n">
+        <x:v>18944</x:v>
+      </x:c>
+      <x:c r="F50" s="27"/>
+      <x:c r="G50" s="31"/>
+      <x:c r="H50" s="32"/>
+      <x:c r="I50" s="33"/>
+      <x:c r="J50" s="34" t="str">
+        <x:f>IFERROR(H50/G50,"")</x:f>
+      </x:c>
+      <x:c r="K50" s="34" t="str">
+        <x:f>IFERROR(I50/G50,"")</x:f>
+      </x:c>
+      <x:c r="L50" s="28"/>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="22" t="str">
+        <x:v>Prefill S=2048</x:v>
+      </x:c>
+      <x:c r="B51" s="22" t="str">
+        <x:v>LM Head</x:v>
+      </x:c>
+      <x:c r="C51" s="22" t="n">
+        <x:v>2048</x:v>
+      </x:c>
+      <x:c r="D51" s="22" t="n">
+        <x:v>152064</x:v>
+      </x:c>
+      <x:c r="E51" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F51" s="27"/>
+      <x:c r="G51" s="31"/>
+      <x:c r="H51" s="32"/>
+      <x:c r="I51" s="33"/>
+      <x:c r="J51" s="34" t="str">
+        <x:f>IFERROR(H51/G51,"")</x:f>
+      </x:c>
+      <x:c r="K51" s="34" t="str">
+        <x:f>IFERROR(I51/G51,"")</x:f>
+      </x:c>
+      <x:c r="L51" s="28"/>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="22" t="str">
+        <x:v>Prefill S=2048</x:v>
+      </x:c>
+      <x:c r="B52" s="22" t="str">
+        <x:v>Attention QK^T</x:v>
+      </x:c>
+      <x:c r="C52" s="22" t="n">
+        <x:v>57344</x:v>
+      </x:c>
+      <x:c r="D52" s="22" t="n">
+        <x:v>2048</x:v>
+      </x:c>
+      <x:c r="E52" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="F52" s="27"/>
+      <x:c r="G52" s="31"/>
+      <x:c r="H52" s="32"/>
+      <x:c r="I52" s="33"/>
+      <x:c r="J52" s="34" t="str">
+        <x:f>IFERROR(H52/G52,"")</x:f>
+      </x:c>
+      <x:c r="K52" s="34" t="str">
+        <x:f>IFERROR(I52/G52,"")</x:f>
+      </x:c>
+      <x:c r="L52" s="28"/>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="22" t="str">
+        <x:v>Prefill S=2048</x:v>
+      </x:c>
+      <x:c r="B53" s="22" t="str">
+        <x:v>Attention AV</x:v>
+      </x:c>
+      <x:c r="C53" s="22" t="n">
+        <x:v>57344</x:v>
+      </x:c>
+      <x:c r="D53" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="E53" s="22" t="n">
+        <x:v>2048</x:v>
+      </x:c>
+      <x:c r="F53" s="27"/>
+      <x:c r="G53" s="31"/>
+      <x:c r="H53" s="32"/>
+      <x:c r="I53" s="33"/>
+      <x:c r="J53" s="34" t="str">
+        <x:f>IFERROR(H53/G53,"")</x:f>
+      </x:c>
+      <x:c r="K53" s="34" t="str">
+        <x:f>IFERROR(I53/G53,"")</x:f>
+      </x:c>
+      <x:c r="L53" s="28"/>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="22" t="str">
+        <x:v>Prefill S=129</x:v>
+      </x:c>
+      <x:c r="B54" s="22" t="str">
+        <x:v>Q / Attention Out</x:v>
+      </x:c>
+      <x:c r="C54" s="22" t="n">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="D54" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="E54" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F54" s="27"/>
+      <x:c r="G54" s="31"/>
+      <x:c r="H54" s="32"/>
+      <x:c r="I54" s="33"/>
+      <x:c r="J54" s="34" t="str">
+        <x:f>IFERROR(H54/G54,"")</x:f>
+      </x:c>
+      <x:c r="K54" s="34" t="str">
+        <x:f>IFERROR(I54/G54,"")</x:f>
+      </x:c>
+      <x:c r="L54" s="28"/>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="22" t="str">
+        <x:v>Prefill S=129</x:v>
+      </x:c>
+      <x:c r="B55" s="22" t="str">
+        <x:v>K / V</x:v>
+      </x:c>
+      <x:c r="C55" s="22" t="n">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="D55" s="22" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="E55" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F55" s="27"/>
+      <x:c r="G55" s="31"/>
+      <x:c r="H55" s="32"/>
+      <x:c r="I55" s="33"/>
+      <x:c r="J55" s="34" t="str">
+        <x:f>IFERROR(H55/G55,"")</x:f>
+      </x:c>
+      <x:c r="K55" s="34" t="str">
+        <x:f>IFERROR(I55/G55,"")</x:f>
+      </x:c>
+      <x:c r="L55" s="28"/>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="22" t="str">
+        <x:v>Prefill S=129</x:v>
+      </x:c>
+      <x:c r="B56" s="22" t="str">
+        <x:v>MLP Up/Gate</x:v>
+      </x:c>
+      <x:c r="C56" s="22" t="n">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="D56" s="22" t="n">
+        <x:v>37888</x:v>
+      </x:c>
+      <x:c r="E56" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F56" s="27"/>
+      <x:c r="G56" s="31"/>
+      <x:c r="H56" s="32"/>
+      <x:c r="I56" s="33"/>
+      <x:c r="J56" s="34" t="str">
+        <x:f>IFERROR(H56/G56,"")</x:f>
+      </x:c>
+      <x:c r="K56" s="34" t="str">
+        <x:f>IFERROR(I56/G56,"")</x:f>
+      </x:c>
+      <x:c r="L56" s="28"/>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="22" t="str">
+        <x:v>Prefill S=129</x:v>
+      </x:c>
+      <x:c r="B57" s="22" t="str">
+        <x:v>MLP Down</x:v>
+      </x:c>
+      <x:c r="C57" s="22" t="n">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="D57" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="E57" s="22" t="n">
+        <x:v>18944</x:v>
+      </x:c>
+      <x:c r="F57" s="27"/>
+      <x:c r="G57" s="31"/>
+      <x:c r="H57" s="32"/>
+      <x:c r="I57" s="33"/>
+      <x:c r="J57" s="34" t="str">
+        <x:f>IFERROR(H57/G57,"")</x:f>
+      </x:c>
+      <x:c r="K57" s="34" t="str">
+        <x:f>IFERROR(I57/G57,"")</x:f>
+      </x:c>
+      <x:c r="L57" s="28"/>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="22" t="str">
+        <x:v>Prefill S=129</x:v>
+      </x:c>
+      <x:c r="B58" s="22" t="str">
+        <x:v>LM Head</x:v>
+      </x:c>
+      <x:c r="C58" s="22" t="n">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="D58" s="22" t="n">
+        <x:v>152064</x:v>
+      </x:c>
+      <x:c r="E58" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F58" s="27"/>
+      <x:c r="G58" s="31"/>
+      <x:c r="H58" s="32"/>
+      <x:c r="I58" s="33"/>
+      <x:c r="J58" s="34" t="str">
+        <x:f>IFERROR(H58/G58,"")</x:f>
+      </x:c>
+      <x:c r="K58" s="34" t="str">
+        <x:f>IFERROR(I58/G58,"")</x:f>
+      </x:c>
+      <x:c r="L58" s="28"/>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="22" t="str">
+        <x:v>Prefill S=129</x:v>
+      </x:c>
+      <x:c r="B59" s="22" t="str">
+        <x:v>Attention QK^T</x:v>
+      </x:c>
+      <x:c r="C59" s="22" t="n">
+        <x:v>3612</x:v>
+      </x:c>
+      <x:c r="D59" s="22" t="n">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="E59" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="F59" s="27"/>
+      <x:c r="G59" s="31"/>
+      <x:c r="H59" s="32"/>
+      <x:c r="I59" s="33"/>
+      <x:c r="J59" s="34" t="str">
+        <x:f>IFERROR(H59/G59,"")</x:f>
+      </x:c>
+      <x:c r="K59" s="34" t="str">
+        <x:f>IFERROR(I59/G59,"")</x:f>
+      </x:c>
+      <x:c r="L59" s="28"/>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="22" t="str">
+        <x:v>Prefill S=129</x:v>
+      </x:c>
+      <x:c r="B60" s="22" t="str">
+        <x:v>Attention AV</x:v>
+      </x:c>
+      <x:c r="C60" s="22" t="n">
+        <x:v>3612</x:v>
+      </x:c>
+      <x:c r="D60" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="E60" s="22" t="n">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="F60" s="27"/>
+      <x:c r="G60" s="31"/>
+      <x:c r="H60" s="32"/>
+      <x:c r="I60" s="33"/>
+      <x:c r="J60" s="34" t="str">
+        <x:f>IFERROR(H60/G60,"")</x:f>
+      </x:c>
+      <x:c r="K60" s="34" t="str">
+        <x:f>IFERROR(I60/G60,"")</x:f>
+      </x:c>
+      <x:c r="L60" s="28"/>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="22" t="str">
+        <x:v>Prefill S=130</x:v>
+      </x:c>
+      <x:c r="B61" s="22" t="str">
+        <x:v>Q / Attention Out</x:v>
+      </x:c>
+      <x:c r="C61" s="22" t="n">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="D61" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="E61" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F61" s="27"/>
+      <x:c r="G61" s="31"/>
+      <x:c r="H61" s="32"/>
+      <x:c r="I61" s="33"/>
+      <x:c r="J61" s="34" t="str">
+        <x:f>IFERROR(H61/G61,"")</x:f>
+      </x:c>
+      <x:c r="K61" s="34" t="str">
+        <x:f>IFERROR(I61/G61,"")</x:f>
+      </x:c>
+      <x:c r="L61" s="28"/>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="22" t="str">
+        <x:v>Prefill S=130</x:v>
+      </x:c>
+      <x:c r="B62" s="22" t="str">
+        <x:v>K / V</x:v>
+      </x:c>
+      <x:c r="C62" s="22" t="n">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="D62" s="22" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="E62" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F62" s="27"/>
+      <x:c r="G62" s="31"/>
+      <x:c r="H62" s="32"/>
+      <x:c r="I62" s="33"/>
+      <x:c r="J62" s="34" t="str">
+        <x:f>IFERROR(H62/G62,"")</x:f>
+      </x:c>
+      <x:c r="K62" s="34" t="str">
+        <x:f>IFERROR(I62/G62,"")</x:f>
+      </x:c>
+      <x:c r="L62" s="28"/>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="22" t="str">
+        <x:v>Prefill S=130</x:v>
+      </x:c>
+      <x:c r="B63" s="22" t="str">
+        <x:v>MLP Up/Gate</x:v>
+      </x:c>
+      <x:c r="C63" s="22" t="n">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="D63" s="22" t="n">
+        <x:v>37888</x:v>
+      </x:c>
+      <x:c r="E63" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F63" s="27"/>
+      <x:c r="G63" s="31"/>
+      <x:c r="H63" s="32"/>
+      <x:c r="I63" s="33"/>
+      <x:c r="J63" s="34" t="str">
+        <x:f>IFERROR(H63/G63,"")</x:f>
+      </x:c>
+      <x:c r="K63" s="34" t="str">
+        <x:f>IFERROR(I63/G63,"")</x:f>
+      </x:c>
+      <x:c r="L63" s="28"/>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="22" t="str">
+        <x:v>Prefill S=130</x:v>
+      </x:c>
+      <x:c r="B64" s="22" t="str">
+        <x:v>MLP Down</x:v>
+      </x:c>
+      <x:c r="C64" s="22" t="n">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="D64" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="E64" s="22" t="n">
+        <x:v>18944</x:v>
+      </x:c>
+      <x:c r="F64" s="27"/>
+      <x:c r="G64" s="31"/>
+      <x:c r="H64" s="32"/>
+      <x:c r="I64" s="33"/>
+      <x:c r="J64" s="34" t="str">
+        <x:f>IFERROR(H64/G64,"")</x:f>
+      </x:c>
+      <x:c r="K64" s="34" t="str">
+        <x:f>IFERROR(I64/G64,"")</x:f>
+      </x:c>
+      <x:c r="L64" s="28"/>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="22" t="str">
+        <x:v>Prefill S=130</x:v>
+      </x:c>
+      <x:c r="B65" s="22" t="str">
+        <x:v>LM Head</x:v>
+      </x:c>
+      <x:c r="C65" s="22" t="n">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="D65" s="22" t="n">
+        <x:v>152064</x:v>
+      </x:c>
+      <x:c r="E65" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F65" s="27"/>
+      <x:c r="G65" s="31"/>
+      <x:c r="H65" s="32"/>
+      <x:c r="I65" s="33"/>
+      <x:c r="J65" s="34" t="str">
+        <x:f>IFERROR(H65/G65,"")</x:f>
+      </x:c>
+      <x:c r="K65" s="34" t="str">
+        <x:f>IFERROR(I65/G65,"")</x:f>
+      </x:c>
+      <x:c r="L65" s="28"/>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="22" t="str">
+        <x:v>Prefill S=130</x:v>
+      </x:c>
+      <x:c r="B66" s="22" t="str">
+        <x:v>Attention QK^T</x:v>
+      </x:c>
+      <x:c r="C66" s="22" t="n">
+        <x:v>3640</x:v>
+      </x:c>
+      <x:c r="D66" s="22" t="n">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="E66" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="F66" s="27"/>
+      <x:c r="G66" s="31"/>
+      <x:c r="H66" s="32"/>
+      <x:c r="I66" s="33"/>
+      <x:c r="J66" s="34" t="str">
+        <x:f>IFERROR(H66/G66,"")</x:f>
+      </x:c>
+      <x:c r="K66" s="34" t="str">
+        <x:f>IFERROR(I66/G66,"")</x:f>
+      </x:c>
+      <x:c r="L66" s="28"/>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="22" t="str">
+        <x:v>Prefill S=130</x:v>
+      </x:c>
+      <x:c r="B67" s="22" t="str">
+        <x:v>Attention AV</x:v>
+      </x:c>
+      <x:c r="C67" s="22" t="n">
+        <x:v>3640</x:v>
+      </x:c>
+      <x:c r="D67" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="E67" s="22" t="n">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="F67" s="27"/>
+      <x:c r="G67" s="31"/>
+      <x:c r="H67" s="32"/>
+      <x:c r="I67" s="33"/>
+      <x:c r="J67" s="34" t="str">
+        <x:f>IFERROR(H67/G67,"")</x:f>
+      </x:c>
+      <x:c r="K67" s="34" t="str">
+        <x:f>IFERROR(I67/G67,"")</x:f>
+      </x:c>
+      <x:c r="L67" s="28"/>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" s="22" t="str">
+        <x:v>Prefill S=132</x:v>
+      </x:c>
+      <x:c r="B68" s="22" t="str">
+        <x:v>Q / Attention Out</x:v>
+      </x:c>
+      <x:c r="C68" s="22" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="D68" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="E68" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F68" s="27"/>
+      <x:c r="G68" s="31"/>
+      <x:c r="H68" s="32"/>
+      <x:c r="I68" s="33"/>
+      <x:c r="J68" s="34" t="str">
+        <x:f>IFERROR(H68/G68,"")</x:f>
+      </x:c>
+      <x:c r="K68" s="34" t="str">
+        <x:f>IFERROR(I68/G68,"")</x:f>
+      </x:c>
+      <x:c r="L68" s="28"/>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" s="22" t="str">
+        <x:v>Prefill S=132</x:v>
+      </x:c>
+      <x:c r="B69" s="22" t="str">
+        <x:v>K / V</x:v>
+      </x:c>
+      <x:c r="C69" s="22" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="D69" s="22" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="E69" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F69" s="27"/>
+      <x:c r="G69" s="31"/>
+      <x:c r="H69" s="32"/>
+      <x:c r="I69" s="33"/>
+      <x:c r="J69" s="34" t="str">
+        <x:f>IFERROR(H69/G69,"")</x:f>
+      </x:c>
+      <x:c r="K69" s="34" t="str">
+        <x:f>IFERROR(I69/G69,"")</x:f>
+      </x:c>
+      <x:c r="L69" s="28"/>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" s="22" t="str">
+        <x:v>Prefill S=132</x:v>
+      </x:c>
+      <x:c r="B70" s="22" t="str">
+        <x:v>MLP Up/Gate</x:v>
+      </x:c>
+      <x:c r="C70" s="22" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="D70" s="22" t="n">
+        <x:v>37888</x:v>
+      </x:c>
+      <x:c r="E70" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F70" s="27"/>
+      <x:c r="G70" s="31"/>
+      <x:c r="H70" s="32"/>
+      <x:c r="I70" s="33"/>
+      <x:c r="J70" s="34" t="str">
+        <x:f>IFERROR(H70/G70,"")</x:f>
+      </x:c>
+      <x:c r="K70" s="34" t="str">
+        <x:f>IFERROR(I70/G70,"")</x:f>
+      </x:c>
+      <x:c r="L70" s="28"/>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" s="22" t="str">
+        <x:v>Prefill S=132</x:v>
+      </x:c>
+      <x:c r="B71" s="22" t="str">
+        <x:v>MLP Down</x:v>
+      </x:c>
+      <x:c r="C71" s="22" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="D71" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="E71" s="22" t="n">
+        <x:v>18944</x:v>
+      </x:c>
+      <x:c r="F71" s="27"/>
+      <x:c r="G71" s="31"/>
+      <x:c r="H71" s="32"/>
+      <x:c r="I71" s="33"/>
+      <x:c r="J71" s="34" t="str">
+        <x:f>IFERROR(H71/G71,"")</x:f>
+      </x:c>
+      <x:c r="K71" s="34" t="str">
+        <x:f>IFERROR(I71/G71,"")</x:f>
+      </x:c>
+      <x:c r="L71" s="28"/>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" s="22" t="str">
+        <x:v>Prefill S=132</x:v>
+      </x:c>
+      <x:c r="B72" s="22" t="str">
+        <x:v>LM Head</x:v>
+      </x:c>
+      <x:c r="C72" s="22" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="D72" s="22" t="n">
+        <x:v>152064</x:v>
+      </x:c>
+      <x:c r="E72" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F72" s="27"/>
+      <x:c r="G72" s="31"/>
+      <x:c r="H72" s="32"/>
+      <x:c r="I72" s="33"/>
+      <x:c r="J72" s="34" t="str">
+        <x:f>IFERROR(H72/G72,"")</x:f>
+      </x:c>
+      <x:c r="K72" s="34" t="str">
+        <x:f>IFERROR(I72/G72,"")</x:f>
+      </x:c>
+      <x:c r="L72" s="28"/>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" s="22" t="str">
+        <x:v>Prefill S=132</x:v>
+      </x:c>
+      <x:c r="B73" s="22" t="str">
+        <x:v>Attention QK^T</x:v>
+      </x:c>
+      <x:c r="C73" s="22" t="n">
+        <x:v>3696</x:v>
+      </x:c>
+      <x:c r="D73" s="22" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="E73" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="F73" s="27"/>
+      <x:c r="G73" s="31"/>
+      <x:c r="H73" s="32"/>
+      <x:c r="I73" s="33"/>
+      <x:c r="J73" s="34" t="str">
+        <x:f>IFERROR(H73/G73,"")</x:f>
+      </x:c>
+      <x:c r="K73" s="34" t="str">
+        <x:f>IFERROR(I73/G73,"")</x:f>
+      </x:c>
+      <x:c r="L73" s="28"/>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" s="22" t="str">
+        <x:v>Prefill S=132</x:v>
+      </x:c>
+      <x:c r="B74" s="22" t="str">
+        <x:v>Attention AV</x:v>
+      </x:c>
+      <x:c r="C74" s="22" t="n">
+        <x:v>3696</x:v>
+      </x:c>
+      <x:c r="D74" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="E74" s="22" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="F74" s="27"/>
+      <x:c r="G74" s="31"/>
+      <x:c r="H74" s="32"/>
+      <x:c r="I74" s="33"/>
+      <x:c r="J74" s="34" t="str">
+        <x:f>IFERROR(H74/G74,"")</x:f>
+      </x:c>
+      <x:c r="K74" s="34" t="str">
+        <x:f>IFERROR(I74/G74,"")</x:f>
+      </x:c>
+      <x:c r="L74" s="28"/>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" s="22" t="str">
+        <x:v>Prefill S=136</x:v>
+      </x:c>
+      <x:c r="B75" s="22" t="str">
+        <x:v>Q / Attention Out</x:v>
+      </x:c>
+      <x:c r="C75" s="22" t="n">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="D75" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="E75" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F75" s="27"/>
+      <x:c r="G75" s="31"/>
+      <x:c r="H75" s="32"/>
+      <x:c r="I75" s="33"/>
+      <x:c r="J75" s="34" t="str">
+        <x:f>IFERROR(H75/G75,"")</x:f>
+      </x:c>
+      <x:c r="K75" s="34" t="str">
+        <x:f>IFERROR(I75/G75,"")</x:f>
+      </x:c>
+      <x:c r="L75" s="28"/>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" s="22" t="str">
+        <x:v>Prefill S=136</x:v>
+      </x:c>
+      <x:c r="B76" s="22" t="str">
+        <x:v>K / V</x:v>
+      </x:c>
+      <x:c r="C76" s="22" t="n">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="D76" s="22" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="E76" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F76" s="27"/>
+      <x:c r="G76" s="31"/>
+      <x:c r="H76" s="32"/>
+      <x:c r="I76" s="33"/>
+      <x:c r="J76" s="34" t="str">
+        <x:f>IFERROR(H76/G76,"")</x:f>
+      </x:c>
+      <x:c r="K76" s="34" t="str">
+        <x:f>IFERROR(I76/G76,"")</x:f>
+      </x:c>
+      <x:c r="L76" s="28"/>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" s="22" t="str">
+        <x:v>Prefill S=136</x:v>
+      </x:c>
+      <x:c r="B77" s="22" t="str">
+        <x:v>MLP Up/Gate</x:v>
+      </x:c>
+      <x:c r="C77" s="22" t="n">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="D77" s="22" t="n">
+        <x:v>37888</x:v>
+      </x:c>
+      <x:c r="E77" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F77" s="27"/>
+      <x:c r="G77" s="31"/>
+      <x:c r="H77" s="32"/>
+      <x:c r="I77" s="33"/>
+      <x:c r="J77" s="34" t="str">
+        <x:f>IFERROR(H77/G77,"")</x:f>
+      </x:c>
+      <x:c r="K77" s="34" t="str">
+        <x:f>IFERROR(I77/G77,"")</x:f>
+      </x:c>
+      <x:c r="L77" s="28"/>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" s="22" t="str">
+        <x:v>Prefill S=136</x:v>
+      </x:c>
+      <x:c r="B78" s="22" t="str">
+        <x:v>MLP Down</x:v>
+      </x:c>
+      <x:c r="C78" s="22" t="n">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="D78" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="E78" s="22" t="n">
+        <x:v>18944</x:v>
+      </x:c>
+      <x:c r="F78" s="27"/>
+      <x:c r="G78" s="31"/>
+      <x:c r="H78" s="32"/>
+      <x:c r="I78" s="33"/>
+      <x:c r="J78" s="34" t="str">
+        <x:f>IFERROR(H78/G78,"")</x:f>
+      </x:c>
+      <x:c r="K78" s="34" t="str">
+        <x:f>IFERROR(I78/G78,"")</x:f>
+      </x:c>
+      <x:c r="L78" s="28"/>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" s="22" t="str">
+        <x:v>Prefill S=136</x:v>
+      </x:c>
+      <x:c r="B79" s="22" t="str">
+        <x:v>LM Head</x:v>
+      </x:c>
+      <x:c r="C79" s="22" t="n">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="D79" s="22" t="n">
+        <x:v>152064</x:v>
+      </x:c>
+      <x:c r="E79" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F79" s="27"/>
+      <x:c r="G79" s="31"/>
+      <x:c r="H79" s="32"/>
+      <x:c r="I79" s="33"/>
+      <x:c r="J79" s="34" t="str">
+        <x:f>IFERROR(H79/G79,"")</x:f>
+      </x:c>
+      <x:c r="K79" s="34" t="str">
+        <x:f>IFERROR(I79/G79,"")</x:f>
+      </x:c>
+      <x:c r="L79" s="28"/>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" s="22" t="str">
+        <x:v>Prefill S=136</x:v>
+      </x:c>
+      <x:c r="B80" s="22" t="str">
+        <x:v>Attention QK^T</x:v>
+      </x:c>
+      <x:c r="C80" s="22" t="n">
+        <x:v>3808</x:v>
+      </x:c>
+      <x:c r="D80" s="22" t="n">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="E80" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="F80" s="27"/>
+      <x:c r="G80" s="31"/>
+      <x:c r="H80" s="32"/>
+      <x:c r="I80" s="33"/>
+      <x:c r="J80" s="34" t="str">
+        <x:f>IFERROR(H80/G80,"")</x:f>
+      </x:c>
+      <x:c r="K80" s="34" t="str">
+        <x:f>IFERROR(I80/G80,"")</x:f>
+      </x:c>
+      <x:c r="L80" s="28"/>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" s="22" t="str">
+        <x:v>Prefill S=136</x:v>
+      </x:c>
+      <x:c r="B81" s="22" t="str">
+        <x:v>Attention AV</x:v>
+      </x:c>
+      <x:c r="C81" s="22" t="n">
+        <x:v>3808</x:v>
+      </x:c>
+      <x:c r="D81" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="E81" s="22" t="n">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="F81" s="27"/>
+      <x:c r="G81" s="31"/>
+      <x:c r="H81" s="32"/>
+      <x:c r="I81" s="33"/>
+      <x:c r="J81" s="34" t="str">
+        <x:f>IFERROR(H81/G81,"")</x:f>
+      </x:c>
+      <x:c r="K81" s="34" t="str">
+        <x:f>IFERROR(I81/G81,"")</x:f>
+      </x:c>
+      <x:c r="L81" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -933,7 +2669,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4f106c0dbb74a11"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R313380b3e67c4bb4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Standardize GEMM configuration names
</commit_message>
<xml_diff>
--- a/gemm_performance_comparison.xlsx
+++ b/gemm_performance_comparison.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="环境对比" sheetId="1" r:id="Ra25625ebaeb74763"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="环境对比" sheetId="1" r:id="R0ae2b948cc494272"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -679,7 +679,7 @@
         <x:v>Decode L=128</x:v>
       </x:c>
       <x:c r="B11" s="22" t="str">
-        <x:v>Attention QK^T / Attention AV</x:v>
+        <x:v>Attention QK^T / Attention PV</x:v>
       </x:c>
       <x:c r="C11" s="22" t="n">
         <x:v>28</x:v>
@@ -735,7 +735,7 @@
         <x:v>Decode L=256</x:v>
       </x:c>
       <x:c r="B13" s="22" t="str">
-        <x:v>Attention AV</x:v>
+        <x:v>Attention PV</x:v>
       </x:c>
       <x:c r="C13" s="22" t="n">
         <x:v>28</x:v>
@@ -791,7 +791,7 @@
         <x:v>Decode L=512</x:v>
       </x:c>
       <x:c r="B15" s="22" t="str">
-        <x:v>Attention AV</x:v>
+        <x:v>Attention PV</x:v>
       </x:c>
       <x:c r="C15" s="22" t="n">
         <x:v>28</x:v>
@@ -847,7 +847,7 @@
         <x:v>Decode L=1024</x:v>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>Attention AV</x:v>
+        <x:v>Attention PV</x:v>
       </x:c>
       <x:c r="C17" s="22" t="n">
         <x:v>28</x:v>
@@ -903,7 +903,7 @@
         <x:v>Decode L=2048</x:v>
       </x:c>
       <x:c r="B19" s="22" t="str">
-        <x:v>Attention AV</x:v>
+        <x:v>Attention PV</x:v>
       </x:c>
       <x:c r="C19" s="22" t="n">
         <x:v>28</x:v>
@@ -1071,7 +1071,7 @@
         <x:v>Prefill S=128</x:v>
       </x:c>
       <x:c r="B25" s="22" t="str">
-        <x:v>Attention QK^T / Attention AV</x:v>
+        <x:v>Attention QK^T / Attention PV</x:v>
       </x:c>
       <x:c r="C25" s="22" t="n">
         <x:v>3584</x:v>
@@ -1267,7 +1267,7 @@
         <x:v>Prefill S=256</x:v>
       </x:c>
       <x:c r="B32" s="22" t="str">
-        <x:v>Attention AV</x:v>
+        <x:v>Attention PV</x:v>
       </x:c>
       <x:c r="C32" s="22" t="n">
         <x:v>7168</x:v>
@@ -1463,7 +1463,7 @@
         <x:v>Prefill S=512</x:v>
       </x:c>
       <x:c r="B39" s="22" t="str">
-        <x:v>Attention AV</x:v>
+        <x:v>Attention PV</x:v>
       </x:c>
       <x:c r="C39" s="22" t="n">
         <x:v>14336</x:v>
@@ -1659,7 +1659,7 @@
         <x:v>Prefill S=1024</x:v>
       </x:c>
       <x:c r="B46" s="22" t="str">
-        <x:v>Attention AV</x:v>
+        <x:v>Attention PV</x:v>
       </x:c>
       <x:c r="C46" s="22" t="n">
         <x:v>28672</x:v>
@@ -1855,7 +1855,7 @@
         <x:v>Prefill S=2048</x:v>
       </x:c>
       <x:c r="B53" s="22" t="str">
-        <x:v>Attention AV</x:v>
+        <x:v>Attention PV</x:v>
       </x:c>
       <x:c r="C53" s="22" t="n">
         <x:v>57344</x:v>
@@ -2051,7 +2051,7 @@
         <x:v>Prefill S=129</x:v>
       </x:c>
       <x:c r="B60" s="22" t="str">
-        <x:v>Attention AV</x:v>
+        <x:v>Attention PV</x:v>
       </x:c>
       <x:c r="C60" s="22" t="n">
         <x:v>3612</x:v>
@@ -2247,7 +2247,7 @@
         <x:v>Prefill S=130</x:v>
       </x:c>
       <x:c r="B67" s="22" t="str">
-        <x:v>Attention AV</x:v>
+        <x:v>Attention PV</x:v>
       </x:c>
       <x:c r="C67" s="22" t="n">
         <x:v>3640</x:v>
@@ -2443,7 +2443,7 @@
         <x:v>Prefill S=132</x:v>
       </x:c>
       <x:c r="B74" s="22" t="str">
-        <x:v>Attention AV</x:v>
+        <x:v>Attention PV</x:v>
       </x:c>
       <x:c r="C74" s="22" t="n">
         <x:v>3696</x:v>
@@ -2639,7 +2639,7 @@
         <x:v>Prefill S=136</x:v>
       </x:c>
       <x:c r="B81" s="22" t="str">
-        <x:v>Attention AV</x:v>
+        <x:v>Attention PV</x:v>
       </x:c>
       <x:c r="C81" s="22" t="n">
         <x:v>3808</x:v>
@@ -2669,7 +2669,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R313380b3e67c4bb4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7b240889db74ebb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Split MLP up and gate GEMM cases
</commit_message>
<xml_diff>
--- a/gemm_performance_comparison.xlsx
+++ b/gemm_performance_comparison.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="环境对比" sheetId="1" r:id="R0ae2b948cc494272"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="环境对比" sheetId="1" r:id="Reccbd279ce0f4dcd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -197,7 +197,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="GemmComparison" displayName="GemmComparison" ref="A5:L81" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="GemmComparison" displayName="GemmComparison" ref="A5:L91" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="阶段/相关长度"/>
     <x:tableColumn id="2" name="来源算子"/>
@@ -481,7 +481,7 @@
     </x:row>
     <x:row r="3" ht="42" customHeight="1">
       <x:c r="A3" s="35" t="str">
-        <x:v>使用方法：Decode 与 Prefill GEMM 严格按 M/N/K 去重；L/S=- 表示与长度无关。运行 run_gemm.sh 保存 CUTLASS 日志，再用 collect_gemm_results.py 回填；两类 HGEMM 请按相同 M/N/K 人工筛选。</x:v>
+        <x:v>使用方法：Decode 与 Prefill GEMM 通常按 M/N/K 去重；MLP Up 与 MLP Gate 均使用 N=I 并分别执行。L/S=- 表示与长度无关。运行 run_gemm.sh 保存 CUTLASS 日志，再用 collect_gemm_results.py 回填；两类 HGEMM 请按相同 M/N/K 人工筛选。</x:v>
       </x:c>
       <x:c r="B3" s="35"/>
       <x:c r="C3" s="35"/>
@@ -595,13 +595,13 @@
         <x:v>Decode L=-</x:v>
       </x:c>
       <x:c r="B8" s="22" t="str">
-        <x:v>MLP Up/Gate</x:v>
+        <x:v>MLP Up</x:v>
       </x:c>
       <x:c r="C8" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D8" s="22" t="n">
-        <x:v>37888</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="E8" s="22" t="n">
         <x:v>3584</x:v>
@@ -623,16 +623,16 @@
         <x:v>Decode L=-</x:v>
       </x:c>
       <x:c r="B9" s="22" t="str">
-        <x:v>MLP Down</x:v>
+        <x:v>MLP Gate</x:v>
       </x:c>
       <x:c r="C9" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D9" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="E9" s="22" t="n">
-        <x:v>18944</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F9" s="27"/>
       <x:c r="G9" s="31"/>
@@ -651,16 +651,16 @@
         <x:v>Decode L=-</x:v>
       </x:c>
       <x:c r="B10" s="22" t="str">
-        <x:v>LM Head</x:v>
+        <x:v>MLP Down</x:v>
       </x:c>
       <x:c r="C10" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D10" s="22" t="n">
-        <x:v>152064</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="E10" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="F10" s="27"/>
       <x:c r="G10" s="31"/>
@@ -676,19 +676,19 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="22" t="str">
-        <x:v>Decode L=128</x:v>
+        <x:v>Decode L=-</x:v>
       </x:c>
       <x:c r="B11" s="22" t="str">
-        <x:v>Attention QK^T / Attention PV</x:v>
+        <x:v>LM Head</x:v>
       </x:c>
       <x:c r="C11" s="22" t="n">
-        <x:v>28</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D11" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>152064</x:v>
       </x:c>
       <x:c r="E11" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F11" s="27"/>
       <x:c r="G11" s="31"/>
@@ -704,16 +704,16 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="22" t="str">
-        <x:v>Decode L=256</x:v>
+        <x:v>Decode L=128</x:v>
       </x:c>
       <x:c r="B12" s="22" t="str">
-        <x:v>Attention QK^T</x:v>
+        <x:v>Attention QK^T / Attention AV</x:v>
       </x:c>
       <x:c r="C12" s="22" t="n">
         <x:v>28</x:v>
       </x:c>
       <x:c r="D12" s="22" t="n">
-        <x:v>256</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="E12" s="22" t="n">
         <x:v>128</x:v>
@@ -735,16 +735,16 @@
         <x:v>Decode L=256</x:v>
       </x:c>
       <x:c r="B13" s="22" t="str">
-        <x:v>Attention PV</x:v>
+        <x:v>Attention QK^T</x:v>
       </x:c>
       <x:c r="C13" s="22" t="n">
         <x:v>28</x:v>
       </x:c>
       <x:c r="D13" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="E13" s="22" t="n">
-        <x:v>256</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="F13" s="27"/>
       <x:c r="G13" s="31"/>
@@ -760,19 +760,19 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="22" t="str">
-        <x:v>Decode L=512</x:v>
+        <x:v>Decode L=256</x:v>
       </x:c>
       <x:c r="B14" s="22" t="str">
-        <x:v>Attention QK^T</x:v>
+        <x:v>Attention AV</x:v>
       </x:c>
       <x:c r="C14" s="22" t="n">
         <x:v>28</x:v>
       </x:c>
       <x:c r="D14" s="22" t="n">
-        <x:v>512</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="E14" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="F14" s="27"/>
       <x:c r="G14" s="31"/>
@@ -791,16 +791,16 @@
         <x:v>Decode L=512</x:v>
       </x:c>
       <x:c r="B15" s="22" t="str">
-        <x:v>Attention PV</x:v>
+        <x:v>Attention QK^T</x:v>
       </x:c>
       <x:c r="C15" s="22" t="n">
         <x:v>28</x:v>
       </x:c>
       <x:c r="D15" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="E15" s="22" t="n">
-        <x:v>512</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="F15" s="27"/>
       <x:c r="G15" s="31"/>
@@ -816,19 +816,19 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="22" t="str">
-        <x:v>Decode L=1024</x:v>
+        <x:v>Decode L=512</x:v>
       </x:c>
       <x:c r="B16" s="22" t="str">
-        <x:v>Attention QK^T</x:v>
+        <x:v>Attention AV</x:v>
       </x:c>
       <x:c r="C16" s="22" t="n">
         <x:v>28</x:v>
       </x:c>
       <x:c r="D16" s="22" t="n">
-        <x:v>1024</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="E16" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="F16" s="27"/>
       <x:c r="G16" s="31"/>
@@ -847,16 +847,16 @@
         <x:v>Decode L=1024</x:v>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>Attention PV</x:v>
+        <x:v>Attention QK^T</x:v>
       </x:c>
       <x:c r="C17" s="22" t="n">
         <x:v>28</x:v>
       </x:c>
       <x:c r="D17" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>1024</x:v>
       </x:c>
       <x:c r="E17" s="22" t="n">
-        <x:v>1024</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="F17" s="27"/>
       <x:c r="G17" s="31"/>
@@ -872,19 +872,19 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="22" t="str">
-        <x:v>Decode L=2048</x:v>
+        <x:v>Decode L=1024</x:v>
       </x:c>
       <x:c r="B18" s="22" t="str">
-        <x:v>Attention QK^T</x:v>
+        <x:v>Attention AV</x:v>
       </x:c>
       <x:c r="C18" s="22" t="n">
         <x:v>28</x:v>
       </x:c>
       <x:c r="D18" s="22" t="n">
-        <x:v>2048</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="E18" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>1024</x:v>
       </x:c>
       <x:c r="F18" s="27"/>
       <x:c r="G18" s="31"/>
@@ -903,16 +903,16 @@
         <x:v>Decode L=2048</x:v>
       </x:c>
       <x:c r="B19" s="22" t="str">
-        <x:v>Attention PV</x:v>
+        <x:v>Attention QK^T</x:v>
       </x:c>
       <x:c r="C19" s="22" t="n">
         <x:v>28</x:v>
       </x:c>
       <x:c r="D19" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>2048</x:v>
       </x:c>
       <x:c r="E19" s="22" t="n">
-        <x:v>2048</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="F19" s="27"/>
       <x:c r="G19" s="31"/>
@@ -928,19 +928,19 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="22" t="str">
-        <x:v>Prefill S=128</x:v>
+        <x:v>Decode L=2048</x:v>
       </x:c>
       <x:c r="B20" s="22" t="str">
-        <x:v>Q / Attention Out</x:v>
+        <x:v>Attention AV</x:v>
       </x:c>
       <x:c r="C20" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="D20" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="E20" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>2048</x:v>
       </x:c>
       <x:c r="F20" s="27"/>
       <x:c r="G20" s="31"/>
@@ -959,13 +959,13 @@
         <x:v>Prefill S=128</x:v>
       </x:c>
       <x:c r="B21" s="22" t="str">
-        <x:v>K / V</x:v>
+        <x:v>Q / Attention Out</x:v>
       </x:c>
       <x:c r="C21" s="22" t="n">
         <x:v>128</x:v>
       </x:c>
       <x:c r="D21" s="22" t="n">
-        <x:v>512</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="E21" s="22" t="n">
         <x:v>3584</x:v>
@@ -987,13 +987,13 @@
         <x:v>Prefill S=128</x:v>
       </x:c>
       <x:c r="B22" s="22" t="str">
-        <x:v>MLP Up/Gate</x:v>
+        <x:v>K / V</x:v>
       </x:c>
       <x:c r="C22" s="22" t="n">
         <x:v>128</x:v>
       </x:c>
       <x:c r="D22" s="22" t="n">
-        <x:v>37888</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="E22" s="22" t="n">
         <x:v>3584</x:v>
@@ -1015,16 +1015,16 @@
         <x:v>Prefill S=128</x:v>
       </x:c>
       <x:c r="B23" s="22" t="str">
-        <x:v>MLP Down</x:v>
+        <x:v>MLP Up</x:v>
       </x:c>
       <x:c r="C23" s="22" t="n">
         <x:v>128</x:v>
       </x:c>
       <x:c r="D23" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="E23" s="22" t="n">
-        <x:v>18944</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F23" s="27"/>
       <x:c r="G23" s="31"/>
@@ -1043,13 +1043,13 @@
         <x:v>Prefill S=128</x:v>
       </x:c>
       <x:c r="B24" s="22" t="str">
-        <x:v>LM Head</x:v>
+        <x:v>MLP Gate</x:v>
       </x:c>
       <x:c r="C24" s="22" t="n">
         <x:v>128</x:v>
       </x:c>
       <x:c r="D24" s="22" t="n">
-        <x:v>152064</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="E24" s="22" t="n">
         <x:v>3584</x:v>
@@ -1071,16 +1071,16 @@
         <x:v>Prefill S=128</x:v>
       </x:c>
       <x:c r="B25" s="22" t="str">
-        <x:v>Attention QK^T / Attention PV</x:v>
+        <x:v>MLP Down</x:v>
       </x:c>
       <x:c r="C25" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="D25" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="E25" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="F25" s="27"/>
       <x:c r="G25" s="31"/>
@@ -1096,16 +1096,16 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="22" t="str">
-        <x:v>Prefill S=256</x:v>
+        <x:v>Prefill S=128</x:v>
       </x:c>
       <x:c r="B26" s="22" t="str">
-        <x:v>Q / Attention Out</x:v>
+        <x:v>LM Head</x:v>
       </x:c>
       <x:c r="C26" s="22" t="n">
-        <x:v>256</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="D26" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>152064</x:v>
       </x:c>
       <x:c r="E26" s="22" t="n">
         <x:v>3584</x:v>
@@ -1124,19 +1124,19 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="22" t="str">
-        <x:v>Prefill S=256</x:v>
+        <x:v>Prefill S=128</x:v>
       </x:c>
       <x:c r="B27" s="22" t="str">
-        <x:v>K / V</x:v>
+        <x:v>Attention QK^T / Attention AV</x:v>
       </x:c>
       <x:c r="C27" s="22" t="n">
-        <x:v>256</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="D27" s="22" t="n">
-        <x:v>512</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="E27" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="F27" s="27"/>
       <x:c r="G27" s="31"/>
@@ -1155,13 +1155,13 @@
         <x:v>Prefill S=256</x:v>
       </x:c>
       <x:c r="B28" s="22" t="str">
-        <x:v>MLP Up/Gate</x:v>
+        <x:v>Q / Attention Out</x:v>
       </x:c>
       <x:c r="C28" s="22" t="n">
         <x:v>256</x:v>
       </x:c>
       <x:c r="D28" s="22" t="n">
-        <x:v>37888</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="E28" s="22" t="n">
         <x:v>3584</x:v>
@@ -1183,16 +1183,16 @@
         <x:v>Prefill S=256</x:v>
       </x:c>
       <x:c r="B29" s="22" t="str">
-        <x:v>MLP Down</x:v>
+        <x:v>K / V</x:v>
       </x:c>
       <x:c r="C29" s="22" t="n">
         <x:v>256</x:v>
       </x:c>
       <x:c r="D29" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="E29" s="22" t="n">
-        <x:v>18944</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F29" s="27"/>
       <x:c r="G29" s="31"/>
@@ -1211,13 +1211,13 @@
         <x:v>Prefill S=256</x:v>
       </x:c>
       <x:c r="B30" s="22" t="str">
-        <x:v>LM Head</x:v>
+        <x:v>MLP Up</x:v>
       </x:c>
       <x:c r="C30" s="22" t="n">
         <x:v>256</x:v>
       </x:c>
       <x:c r="D30" s="22" t="n">
-        <x:v>152064</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="E30" s="22" t="n">
         <x:v>3584</x:v>
@@ -1239,16 +1239,16 @@
         <x:v>Prefill S=256</x:v>
       </x:c>
       <x:c r="B31" s="22" t="str">
-        <x:v>Attention QK^T</x:v>
+        <x:v>MLP Gate</x:v>
       </x:c>
       <x:c r="C31" s="22" t="n">
-        <x:v>7168</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="D31" s="22" t="n">
-        <x:v>256</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="E31" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F31" s="27"/>
       <x:c r="G31" s="31"/>
@@ -1267,16 +1267,16 @@
         <x:v>Prefill S=256</x:v>
       </x:c>
       <x:c r="B32" s="22" t="str">
-        <x:v>Attention PV</x:v>
+        <x:v>MLP Down</x:v>
       </x:c>
       <x:c r="C32" s="22" t="n">
-        <x:v>7168</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="D32" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="E32" s="22" t="n">
-        <x:v>256</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="F32" s="27"/>
       <x:c r="G32" s="31"/>
@@ -1292,16 +1292,16 @@
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="22" t="str">
-        <x:v>Prefill S=512</x:v>
+        <x:v>Prefill S=256</x:v>
       </x:c>
       <x:c r="B33" s="22" t="str">
-        <x:v>Q / Attention Out</x:v>
+        <x:v>LM Head</x:v>
       </x:c>
       <x:c r="C33" s="22" t="n">
-        <x:v>512</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="D33" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>152064</x:v>
       </x:c>
       <x:c r="E33" s="22" t="n">
         <x:v>3584</x:v>
@@ -1320,19 +1320,19 @@
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="22" t="str">
-        <x:v>Prefill S=512</x:v>
+        <x:v>Prefill S=256</x:v>
       </x:c>
       <x:c r="B34" s="22" t="str">
-        <x:v>K / V</x:v>
+        <x:v>Attention QK^T</x:v>
       </x:c>
       <x:c r="C34" s="22" t="n">
-        <x:v>512</x:v>
+        <x:v>7168</x:v>
       </x:c>
       <x:c r="D34" s="22" t="n">
-        <x:v>512</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="E34" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="F34" s="27"/>
       <x:c r="G34" s="31"/>
@@ -1348,19 +1348,19 @@
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="22" t="str">
-        <x:v>Prefill S=512</x:v>
+        <x:v>Prefill S=256</x:v>
       </x:c>
       <x:c r="B35" s="22" t="str">
-        <x:v>MLP Up/Gate</x:v>
+        <x:v>Attention AV</x:v>
       </x:c>
       <x:c r="C35" s="22" t="n">
-        <x:v>512</x:v>
+        <x:v>7168</x:v>
       </x:c>
       <x:c r="D35" s="22" t="n">
-        <x:v>37888</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="E35" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="F35" s="27"/>
       <x:c r="G35" s="31"/>
@@ -1379,7 +1379,7 @@
         <x:v>Prefill S=512</x:v>
       </x:c>
       <x:c r="B36" s="22" t="str">
-        <x:v>MLP Down</x:v>
+        <x:v>Q / Attention Out</x:v>
       </x:c>
       <x:c r="C36" s="22" t="n">
         <x:v>512</x:v>
@@ -1388,7 +1388,7 @@
         <x:v>3584</x:v>
       </x:c>
       <x:c r="E36" s="22" t="n">
-        <x:v>18944</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F36" s="27"/>
       <x:c r="G36" s="31"/>
@@ -1407,13 +1407,13 @@
         <x:v>Prefill S=512</x:v>
       </x:c>
       <x:c r="B37" s="22" t="str">
-        <x:v>LM Head</x:v>
+        <x:v>K / V</x:v>
       </x:c>
       <x:c r="C37" s="22" t="n">
         <x:v>512</x:v>
       </x:c>
       <x:c r="D37" s="22" t="n">
-        <x:v>152064</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="E37" s="22" t="n">
         <x:v>3584</x:v>
@@ -1435,16 +1435,16 @@
         <x:v>Prefill S=512</x:v>
       </x:c>
       <x:c r="B38" s="22" t="str">
-        <x:v>Attention QK^T</x:v>
+        <x:v>MLP Up</x:v>
       </x:c>
       <x:c r="C38" s="22" t="n">
-        <x:v>14336</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="D38" s="22" t="n">
-        <x:v>512</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="E38" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F38" s="27"/>
       <x:c r="G38" s="31"/>
@@ -1463,16 +1463,16 @@
         <x:v>Prefill S=512</x:v>
       </x:c>
       <x:c r="B39" s="22" t="str">
-        <x:v>Attention PV</x:v>
+        <x:v>MLP Gate</x:v>
       </x:c>
       <x:c r="C39" s="22" t="n">
-        <x:v>14336</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="D39" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="E39" s="22" t="n">
-        <x:v>512</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F39" s="27"/>
       <x:c r="G39" s="31"/>
@@ -1488,19 +1488,19 @@
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="22" t="str">
-        <x:v>Prefill S=1024</x:v>
+        <x:v>Prefill S=512</x:v>
       </x:c>
       <x:c r="B40" s="22" t="str">
-        <x:v>Q / Attention Out</x:v>
+        <x:v>MLP Down</x:v>
       </x:c>
       <x:c r="C40" s="22" t="n">
-        <x:v>1024</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="D40" s="22" t="n">
         <x:v>3584</x:v>
       </x:c>
       <x:c r="E40" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="F40" s="27"/>
       <x:c r="G40" s="31"/>
@@ -1516,16 +1516,16 @@
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="22" t="str">
-        <x:v>Prefill S=1024</x:v>
+        <x:v>Prefill S=512</x:v>
       </x:c>
       <x:c r="B41" s="22" t="str">
-        <x:v>K / V</x:v>
+        <x:v>LM Head</x:v>
       </x:c>
       <x:c r="C41" s="22" t="n">
-        <x:v>1024</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="D41" s="22" t="n">
-        <x:v>512</x:v>
+        <x:v>152064</x:v>
       </x:c>
       <x:c r="E41" s="22" t="n">
         <x:v>3584</x:v>
@@ -1544,19 +1544,19 @@
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="22" t="str">
-        <x:v>Prefill S=1024</x:v>
+        <x:v>Prefill S=512</x:v>
       </x:c>
       <x:c r="B42" s="22" t="str">
-        <x:v>MLP Up/Gate</x:v>
+        <x:v>Attention QK^T</x:v>
       </x:c>
       <x:c r="C42" s="22" t="n">
-        <x:v>1024</x:v>
+        <x:v>14336</x:v>
       </x:c>
       <x:c r="D42" s="22" t="n">
-        <x:v>37888</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="E42" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="F42" s="27"/>
       <x:c r="G42" s="31"/>
@@ -1572,19 +1572,19 @@
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="22" t="str">
-        <x:v>Prefill S=1024</x:v>
+        <x:v>Prefill S=512</x:v>
       </x:c>
       <x:c r="B43" s="22" t="str">
-        <x:v>MLP Down</x:v>
+        <x:v>Attention AV</x:v>
       </x:c>
       <x:c r="C43" s="22" t="n">
-        <x:v>1024</x:v>
+        <x:v>14336</x:v>
       </x:c>
       <x:c r="D43" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="E43" s="22" t="n">
-        <x:v>18944</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="F43" s="27"/>
       <x:c r="G43" s="31"/>
@@ -1603,13 +1603,13 @@
         <x:v>Prefill S=1024</x:v>
       </x:c>
       <x:c r="B44" s="22" t="str">
-        <x:v>LM Head</x:v>
+        <x:v>Q / Attention Out</x:v>
       </x:c>
       <x:c r="C44" s="22" t="n">
         <x:v>1024</x:v>
       </x:c>
       <x:c r="D44" s="22" t="n">
-        <x:v>152064</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="E44" s="22" t="n">
         <x:v>3584</x:v>
@@ -1631,16 +1631,16 @@
         <x:v>Prefill S=1024</x:v>
       </x:c>
       <x:c r="B45" s="22" t="str">
-        <x:v>Attention QK^T</x:v>
+        <x:v>K / V</x:v>
       </x:c>
       <x:c r="C45" s="22" t="n">
-        <x:v>28672</x:v>
+        <x:v>1024</x:v>
       </x:c>
       <x:c r="D45" s="22" t="n">
-        <x:v>1024</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="E45" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F45" s="27"/>
       <x:c r="G45" s="31"/>
@@ -1659,16 +1659,16 @@
         <x:v>Prefill S=1024</x:v>
       </x:c>
       <x:c r="B46" s="22" t="str">
-        <x:v>Attention PV</x:v>
+        <x:v>MLP Up</x:v>
       </x:c>
       <x:c r="C46" s="22" t="n">
-        <x:v>28672</x:v>
+        <x:v>1024</x:v>
       </x:c>
       <x:c r="D46" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="E46" s="22" t="n">
-        <x:v>1024</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F46" s="27"/>
       <x:c r="G46" s="31"/>
@@ -1684,16 +1684,16 @@
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="22" t="str">
-        <x:v>Prefill S=2048</x:v>
+        <x:v>Prefill S=1024</x:v>
       </x:c>
       <x:c r="B47" s="22" t="str">
-        <x:v>Q / Attention Out</x:v>
+        <x:v>MLP Gate</x:v>
       </x:c>
       <x:c r="C47" s="22" t="n">
-        <x:v>2048</x:v>
+        <x:v>1024</x:v>
       </x:c>
       <x:c r="D47" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="E47" s="22" t="n">
         <x:v>3584</x:v>
@@ -1712,19 +1712,19 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="22" t="str">
-        <x:v>Prefill S=2048</x:v>
+        <x:v>Prefill S=1024</x:v>
       </x:c>
       <x:c r="B48" s="22" t="str">
-        <x:v>K / V</x:v>
+        <x:v>MLP Down</x:v>
       </x:c>
       <x:c r="C48" s="22" t="n">
-        <x:v>2048</x:v>
+        <x:v>1024</x:v>
       </x:c>
       <x:c r="D48" s="22" t="n">
-        <x:v>512</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="E48" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="F48" s="27"/>
       <x:c r="G48" s="31"/>
@@ -1740,16 +1740,16 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="22" t="str">
-        <x:v>Prefill S=2048</x:v>
+        <x:v>Prefill S=1024</x:v>
       </x:c>
       <x:c r="B49" s="22" t="str">
-        <x:v>MLP Up/Gate</x:v>
+        <x:v>LM Head</x:v>
       </x:c>
       <x:c r="C49" s="22" t="n">
-        <x:v>2048</x:v>
+        <x:v>1024</x:v>
       </x:c>
       <x:c r="D49" s="22" t="n">
-        <x:v>37888</x:v>
+        <x:v>152064</x:v>
       </x:c>
       <x:c r="E49" s="22" t="n">
         <x:v>3584</x:v>
@@ -1768,19 +1768,19 @@
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="22" t="str">
-        <x:v>Prefill S=2048</x:v>
+        <x:v>Prefill S=1024</x:v>
       </x:c>
       <x:c r="B50" s="22" t="str">
-        <x:v>MLP Down</x:v>
+        <x:v>Attention QK^T</x:v>
       </x:c>
       <x:c r="C50" s="22" t="n">
-        <x:v>2048</x:v>
+        <x:v>28672</x:v>
       </x:c>
       <x:c r="D50" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>1024</x:v>
       </x:c>
       <x:c r="E50" s="22" t="n">
-        <x:v>18944</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="F50" s="27"/>
       <x:c r="G50" s="31"/>
@@ -1796,19 +1796,19 @@
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="22" t="str">
-        <x:v>Prefill S=2048</x:v>
+        <x:v>Prefill S=1024</x:v>
       </x:c>
       <x:c r="B51" s="22" t="str">
-        <x:v>LM Head</x:v>
+        <x:v>Attention AV</x:v>
       </x:c>
       <x:c r="C51" s="22" t="n">
-        <x:v>2048</x:v>
+        <x:v>28672</x:v>
       </x:c>
       <x:c r="D51" s="22" t="n">
-        <x:v>152064</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="E51" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>1024</x:v>
       </x:c>
       <x:c r="F51" s="27"/>
       <x:c r="G51" s="31"/>
@@ -1827,16 +1827,16 @@
         <x:v>Prefill S=2048</x:v>
       </x:c>
       <x:c r="B52" s="22" t="str">
-        <x:v>Attention QK^T</x:v>
+        <x:v>Q / Attention Out</x:v>
       </x:c>
       <x:c r="C52" s="22" t="n">
-        <x:v>57344</x:v>
+        <x:v>2048</x:v>
       </x:c>
       <x:c r="D52" s="22" t="n">
-        <x:v>2048</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="E52" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F52" s="27"/>
       <x:c r="G52" s="31"/>
@@ -1855,16 +1855,16 @@
         <x:v>Prefill S=2048</x:v>
       </x:c>
       <x:c r="B53" s="22" t="str">
-        <x:v>Attention PV</x:v>
+        <x:v>K / V</x:v>
       </x:c>
       <x:c r="C53" s="22" t="n">
-        <x:v>57344</x:v>
+        <x:v>2048</x:v>
       </x:c>
       <x:c r="D53" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="E53" s="22" t="n">
-        <x:v>2048</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F53" s="27"/>
       <x:c r="G53" s="31"/>
@@ -1880,16 +1880,16 @@
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="22" t="str">
-        <x:v>Prefill S=129</x:v>
+        <x:v>Prefill S=2048</x:v>
       </x:c>
       <x:c r="B54" s="22" t="str">
-        <x:v>Q / Attention Out</x:v>
+        <x:v>MLP Up</x:v>
       </x:c>
       <x:c r="C54" s="22" t="n">
-        <x:v>129</x:v>
+        <x:v>2048</x:v>
       </x:c>
       <x:c r="D54" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="E54" s="22" t="n">
         <x:v>3584</x:v>
@@ -1908,16 +1908,16 @@
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="22" t="str">
-        <x:v>Prefill S=129</x:v>
+        <x:v>Prefill S=2048</x:v>
       </x:c>
       <x:c r="B55" s="22" t="str">
-        <x:v>K / V</x:v>
+        <x:v>MLP Gate</x:v>
       </x:c>
       <x:c r="C55" s="22" t="n">
-        <x:v>129</x:v>
+        <x:v>2048</x:v>
       </x:c>
       <x:c r="D55" s="22" t="n">
-        <x:v>512</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="E55" s="22" t="n">
         <x:v>3584</x:v>
@@ -1936,19 +1936,19 @@
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="22" t="str">
-        <x:v>Prefill S=129</x:v>
+        <x:v>Prefill S=2048</x:v>
       </x:c>
       <x:c r="B56" s="22" t="str">
-        <x:v>MLP Up/Gate</x:v>
+        <x:v>MLP Down</x:v>
       </x:c>
       <x:c r="C56" s="22" t="n">
-        <x:v>129</x:v>
+        <x:v>2048</x:v>
       </x:c>
       <x:c r="D56" s="22" t="n">
-        <x:v>37888</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="E56" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="F56" s="27"/>
       <x:c r="G56" s="31"/>
@@ -1964,19 +1964,19 @@
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="22" t="str">
-        <x:v>Prefill S=129</x:v>
+        <x:v>Prefill S=2048</x:v>
       </x:c>
       <x:c r="B57" s="22" t="str">
-        <x:v>MLP Down</x:v>
+        <x:v>LM Head</x:v>
       </x:c>
       <x:c r="C57" s="22" t="n">
-        <x:v>129</x:v>
+        <x:v>2048</x:v>
       </x:c>
       <x:c r="D57" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>152064</x:v>
       </x:c>
       <x:c r="E57" s="22" t="n">
-        <x:v>18944</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F57" s="27"/>
       <x:c r="G57" s="31"/>
@@ -1992,19 +1992,19 @@
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="22" t="str">
-        <x:v>Prefill S=129</x:v>
+        <x:v>Prefill S=2048</x:v>
       </x:c>
       <x:c r="B58" s="22" t="str">
-        <x:v>LM Head</x:v>
+        <x:v>Attention QK^T</x:v>
       </x:c>
       <x:c r="C58" s="22" t="n">
-        <x:v>129</x:v>
+        <x:v>57344</x:v>
       </x:c>
       <x:c r="D58" s="22" t="n">
-        <x:v>152064</x:v>
+        <x:v>2048</x:v>
       </x:c>
       <x:c r="E58" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="F58" s="27"/>
       <x:c r="G58" s="31"/>
@@ -2020,19 +2020,19 @@
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="22" t="str">
-        <x:v>Prefill S=129</x:v>
+        <x:v>Prefill S=2048</x:v>
       </x:c>
       <x:c r="B59" s="22" t="str">
-        <x:v>Attention QK^T</x:v>
+        <x:v>Attention AV</x:v>
       </x:c>
       <x:c r="C59" s="22" t="n">
-        <x:v>3612</x:v>
+        <x:v>57344</x:v>
       </x:c>
       <x:c r="D59" s="22" t="n">
-        <x:v>129</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="E59" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>2048</x:v>
       </x:c>
       <x:c r="F59" s="27"/>
       <x:c r="G59" s="31"/>
@@ -2051,16 +2051,16 @@
         <x:v>Prefill S=129</x:v>
       </x:c>
       <x:c r="B60" s="22" t="str">
-        <x:v>Attention PV</x:v>
+        <x:v>Q / Attention Out</x:v>
       </x:c>
       <x:c r="C60" s="22" t="n">
-        <x:v>3612</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="D60" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="E60" s="22" t="n">
-        <x:v>129</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F60" s="27"/>
       <x:c r="G60" s="31"/>
@@ -2076,16 +2076,16 @@
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="22" t="str">
-        <x:v>Prefill S=130</x:v>
+        <x:v>Prefill S=129</x:v>
       </x:c>
       <x:c r="B61" s="22" t="str">
-        <x:v>Q / Attention Out</x:v>
+        <x:v>K / V</x:v>
       </x:c>
       <x:c r="C61" s="22" t="n">
-        <x:v>130</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="D61" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="E61" s="22" t="n">
         <x:v>3584</x:v>
@@ -2104,16 +2104,16 @@
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="22" t="str">
-        <x:v>Prefill S=130</x:v>
+        <x:v>Prefill S=129</x:v>
       </x:c>
       <x:c r="B62" s="22" t="str">
-        <x:v>K / V</x:v>
+        <x:v>MLP Up</x:v>
       </x:c>
       <x:c r="C62" s="22" t="n">
-        <x:v>130</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="D62" s="22" t="n">
-        <x:v>512</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="E62" s="22" t="n">
         <x:v>3584</x:v>
@@ -2132,16 +2132,16 @@
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="22" t="str">
-        <x:v>Prefill S=130</x:v>
+        <x:v>Prefill S=129</x:v>
       </x:c>
       <x:c r="B63" s="22" t="str">
-        <x:v>MLP Up/Gate</x:v>
+        <x:v>MLP Gate</x:v>
       </x:c>
       <x:c r="C63" s="22" t="n">
-        <x:v>130</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="D63" s="22" t="n">
-        <x:v>37888</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="E63" s="22" t="n">
         <x:v>3584</x:v>
@@ -2160,13 +2160,13 @@
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="22" t="str">
-        <x:v>Prefill S=130</x:v>
+        <x:v>Prefill S=129</x:v>
       </x:c>
       <x:c r="B64" s="22" t="str">
         <x:v>MLP Down</x:v>
       </x:c>
       <x:c r="C64" s="22" t="n">
-        <x:v>130</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="D64" s="22" t="n">
         <x:v>3584</x:v>
@@ -2188,13 +2188,13 @@
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="22" t="str">
-        <x:v>Prefill S=130</x:v>
+        <x:v>Prefill S=129</x:v>
       </x:c>
       <x:c r="B65" s="22" t="str">
         <x:v>LM Head</x:v>
       </x:c>
       <x:c r="C65" s="22" t="n">
-        <x:v>130</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="D65" s="22" t="n">
         <x:v>152064</x:v>
@@ -2216,16 +2216,16 @@
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="22" t="str">
-        <x:v>Prefill S=130</x:v>
+        <x:v>Prefill S=129</x:v>
       </x:c>
       <x:c r="B66" s="22" t="str">
         <x:v>Attention QK^T</x:v>
       </x:c>
       <x:c r="C66" s="22" t="n">
-        <x:v>3640</x:v>
+        <x:v>3612</x:v>
       </x:c>
       <x:c r="D66" s="22" t="n">
-        <x:v>130</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="E66" s="22" t="n">
         <x:v>128</x:v>
@@ -2244,19 +2244,19 @@
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="22" t="str">
-        <x:v>Prefill S=130</x:v>
+        <x:v>Prefill S=129</x:v>
       </x:c>
       <x:c r="B67" s="22" t="str">
-        <x:v>Attention PV</x:v>
+        <x:v>Attention AV</x:v>
       </x:c>
       <x:c r="C67" s="22" t="n">
-        <x:v>3640</x:v>
+        <x:v>3612</x:v>
       </x:c>
       <x:c r="D67" s="22" t="n">
         <x:v>128</x:v>
       </x:c>
       <x:c r="E67" s="22" t="n">
-        <x:v>130</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="F67" s="27"/>
       <x:c r="G67" s="31"/>
@@ -2272,13 +2272,13 @@
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="22" t="str">
-        <x:v>Prefill S=132</x:v>
+        <x:v>Prefill S=130</x:v>
       </x:c>
       <x:c r="B68" s="22" t="str">
         <x:v>Q / Attention Out</x:v>
       </x:c>
       <x:c r="C68" s="22" t="n">
-        <x:v>132</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="D68" s="22" t="n">
         <x:v>3584</x:v>
@@ -2300,13 +2300,13 @@
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="22" t="str">
-        <x:v>Prefill S=132</x:v>
+        <x:v>Prefill S=130</x:v>
       </x:c>
       <x:c r="B69" s="22" t="str">
         <x:v>K / V</x:v>
       </x:c>
       <x:c r="C69" s="22" t="n">
-        <x:v>132</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="D69" s="22" t="n">
         <x:v>512</x:v>
@@ -2328,16 +2328,16 @@
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="22" t="str">
-        <x:v>Prefill S=132</x:v>
+        <x:v>Prefill S=130</x:v>
       </x:c>
       <x:c r="B70" s="22" t="str">
-        <x:v>MLP Up/Gate</x:v>
+        <x:v>MLP Up</x:v>
       </x:c>
       <x:c r="C70" s="22" t="n">
-        <x:v>132</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="D70" s="22" t="n">
-        <x:v>37888</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="E70" s="22" t="n">
         <x:v>3584</x:v>
@@ -2356,19 +2356,19 @@
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="22" t="str">
-        <x:v>Prefill S=132</x:v>
+        <x:v>Prefill S=130</x:v>
       </x:c>
       <x:c r="B71" s="22" t="str">
-        <x:v>MLP Down</x:v>
+        <x:v>MLP Gate</x:v>
       </x:c>
       <x:c r="C71" s="22" t="n">
-        <x:v>132</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="D71" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="E71" s="22" t="n">
-        <x:v>18944</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F71" s="27"/>
       <x:c r="G71" s="31"/>
@@ -2384,19 +2384,19 @@
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="22" t="str">
-        <x:v>Prefill S=132</x:v>
+        <x:v>Prefill S=130</x:v>
       </x:c>
       <x:c r="B72" s="22" t="str">
-        <x:v>LM Head</x:v>
+        <x:v>MLP Down</x:v>
       </x:c>
       <x:c r="C72" s="22" t="n">
-        <x:v>132</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="D72" s="22" t="n">
-        <x:v>152064</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="E72" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="F72" s="27"/>
       <x:c r="G72" s="31"/>
@@ -2412,19 +2412,19 @@
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="22" t="str">
-        <x:v>Prefill S=132</x:v>
+        <x:v>Prefill S=130</x:v>
       </x:c>
       <x:c r="B73" s="22" t="str">
-        <x:v>Attention QK^T</x:v>
+        <x:v>LM Head</x:v>
       </x:c>
       <x:c r="C73" s="22" t="n">
-        <x:v>3696</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="D73" s="22" t="n">
-        <x:v>132</x:v>
+        <x:v>152064</x:v>
       </x:c>
       <x:c r="E73" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F73" s="27"/>
       <x:c r="G73" s="31"/>
@@ -2440,19 +2440,19 @@
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="22" t="str">
-        <x:v>Prefill S=132</x:v>
+        <x:v>Prefill S=130</x:v>
       </x:c>
       <x:c r="B74" s="22" t="str">
-        <x:v>Attention PV</x:v>
+        <x:v>Attention QK^T</x:v>
       </x:c>
       <x:c r="C74" s="22" t="n">
-        <x:v>3696</x:v>
+        <x:v>3640</x:v>
       </x:c>
       <x:c r="D74" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="E74" s="22" t="n">
-        <x:v>132</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="F74" s="27"/>
       <x:c r="G74" s="31"/>
@@ -2468,19 +2468,19 @@
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="22" t="str">
-        <x:v>Prefill S=136</x:v>
+        <x:v>Prefill S=130</x:v>
       </x:c>
       <x:c r="B75" s="22" t="str">
-        <x:v>Q / Attention Out</x:v>
+        <x:v>Attention AV</x:v>
       </x:c>
       <x:c r="C75" s="22" t="n">
-        <x:v>136</x:v>
+        <x:v>3640</x:v>
       </x:c>
       <x:c r="D75" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="E75" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="F75" s="27"/>
       <x:c r="G75" s="31"/>
@@ -2496,16 +2496,16 @@
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="22" t="str">
-        <x:v>Prefill S=136</x:v>
+        <x:v>Prefill S=132</x:v>
       </x:c>
       <x:c r="B76" s="22" t="str">
-        <x:v>K / V</x:v>
+        <x:v>Q / Attention Out</x:v>
       </x:c>
       <x:c r="C76" s="22" t="n">
-        <x:v>136</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="D76" s="22" t="n">
-        <x:v>512</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="E76" s="22" t="n">
         <x:v>3584</x:v>
@@ -2524,16 +2524,16 @@
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="22" t="str">
-        <x:v>Prefill S=136</x:v>
+        <x:v>Prefill S=132</x:v>
       </x:c>
       <x:c r="B77" s="22" t="str">
-        <x:v>MLP Up/Gate</x:v>
+        <x:v>K / V</x:v>
       </x:c>
       <x:c r="C77" s="22" t="n">
-        <x:v>136</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="D77" s="22" t="n">
-        <x:v>37888</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="E77" s="22" t="n">
         <x:v>3584</x:v>
@@ -2552,19 +2552,19 @@
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="22" t="str">
-        <x:v>Prefill S=136</x:v>
+        <x:v>Prefill S=132</x:v>
       </x:c>
       <x:c r="B78" s="22" t="str">
-        <x:v>MLP Down</x:v>
+        <x:v>MLP Up</x:v>
       </x:c>
       <x:c r="C78" s="22" t="n">
-        <x:v>136</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="D78" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="E78" s="22" t="n">
-        <x:v>18944</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F78" s="27"/>
       <x:c r="G78" s="31"/>
@@ -2580,16 +2580,16 @@
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="22" t="str">
-        <x:v>Prefill S=136</x:v>
+        <x:v>Prefill S=132</x:v>
       </x:c>
       <x:c r="B79" s="22" t="str">
-        <x:v>LM Head</x:v>
+        <x:v>MLP Gate</x:v>
       </x:c>
       <x:c r="C79" s="22" t="n">
-        <x:v>136</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="D79" s="22" t="n">
-        <x:v>152064</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="E79" s="22" t="n">
         <x:v>3584</x:v>
@@ -2608,19 +2608,19 @@
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="22" t="str">
-        <x:v>Prefill S=136</x:v>
+        <x:v>Prefill S=132</x:v>
       </x:c>
       <x:c r="B80" s="22" t="str">
-        <x:v>Attention QK^T</x:v>
+        <x:v>MLP Down</x:v>
       </x:c>
       <x:c r="C80" s="22" t="n">
-        <x:v>3808</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="D80" s="22" t="n">
-        <x:v>136</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="E80" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="F80" s="27"/>
       <x:c r="G80" s="31"/>
@@ -2636,19 +2636,19 @@
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="22" t="str">
-        <x:v>Prefill S=136</x:v>
+        <x:v>Prefill S=132</x:v>
       </x:c>
       <x:c r="B81" s="22" t="str">
-        <x:v>Attention PV</x:v>
+        <x:v>LM Head</x:v>
       </x:c>
       <x:c r="C81" s="22" t="n">
-        <x:v>3808</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="D81" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>152064</x:v>
       </x:c>
       <x:c r="E81" s="22" t="n">
-        <x:v>136</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F81" s="27"/>
       <x:c r="G81" s="31"/>
@@ -2661,6 +2661,286 @@
         <x:f>IFERROR(I81/G81,"")</x:f>
       </x:c>
       <x:c r="L81" s="28"/>
+    </x:row>
+    <x:row r="82">
+      <x:c r="A82" s="22" t="str">
+        <x:v>Prefill S=132</x:v>
+      </x:c>
+      <x:c r="B82" s="22" t="str">
+        <x:v>Attention QK^T</x:v>
+      </x:c>
+      <x:c r="C82" s="22" t="n">
+        <x:v>3696</x:v>
+      </x:c>
+      <x:c r="D82" s="22" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="E82" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="F82" s="27"/>
+      <x:c r="G82" s="31"/>
+      <x:c r="H82" s="32"/>
+      <x:c r="I82" s="33"/>
+      <x:c r="J82" s="34" t="str">
+        <x:f>IFERROR(H82/G82,"")</x:f>
+      </x:c>
+      <x:c r="K82" s="34" t="str">
+        <x:f>IFERROR(I82/G82,"")</x:f>
+      </x:c>
+      <x:c r="L82" s="28"/>
+    </x:row>
+    <x:row r="83">
+      <x:c r="A83" s="22" t="str">
+        <x:v>Prefill S=132</x:v>
+      </x:c>
+      <x:c r="B83" s="22" t="str">
+        <x:v>Attention AV</x:v>
+      </x:c>
+      <x:c r="C83" s="22" t="n">
+        <x:v>3696</x:v>
+      </x:c>
+      <x:c r="D83" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="E83" s="22" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="F83" s="27"/>
+      <x:c r="G83" s="31"/>
+      <x:c r="H83" s="32"/>
+      <x:c r="I83" s="33"/>
+      <x:c r="J83" s="34" t="str">
+        <x:f>IFERROR(H83/G83,"")</x:f>
+      </x:c>
+      <x:c r="K83" s="34" t="str">
+        <x:f>IFERROR(I83/G83,"")</x:f>
+      </x:c>
+      <x:c r="L83" s="28"/>
+    </x:row>
+    <x:row r="84">
+      <x:c r="A84" s="22" t="str">
+        <x:v>Prefill S=136</x:v>
+      </x:c>
+      <x:c r="B84" s="22" t="str">
+        <x:v>Q / Attention Out</x:v>
+      </x:c>
+      <x:c r="C84" s="22" t="n">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="D84" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="E84" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F84" s="27"/>
+      <x:c r="G84" s="31"/>
+      <x:c r="H84" s="32"/>
+      <x:c r="I84" s="33"/>
+      <x:c r="J84" s="34" t="str">
+        <x:f>IFERROR(H84/G84,"")</x:f>
+      </x:c>
+      <x:c r="K84" s="34" t="str">
+        <x:f>IFERROR(I84/G84,"")</x:f>
+      </x:c>
+      <x:c r="L84" s="28"/>
+    </x:row>
+    <x:row r="85">
+      <x:c r="A85" s="22" t="str">
+        <x:v>Prefill S=136</x:v>
+      </x:c>
+      <x:c r="B85" s="22" t="str">
+        <x:v>K / V</x:v>
+      </x:c>
+      <x:c r="C85" s="22" t="n">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="D85" s="22" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="E85" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F85" s="27"/>
+      <x:c r="G85" s="31"/>
+      <x:c r="H85" s="32"/>
+      <x:c r="I85" s="33"/>
+      <x:c r="J85" s="34" t="str">
+        <x:f>IFERROR(H85/G85,"")</x:f>
+      </x:c>
+      <x:c r="K85" s="34" t="str">
+        <x:f>IFERROR(I85/G85,"")</x:f>
+      </x:c>
+      <x:c r="L85" s="28"/>
+    </x:row>
+    <x:row r="86">
+      <x:c r="A86" s="22" t="str">
+        <x:v>Prefill S=136</x:v>
+      </x:c>
+      <x:c r="B86" s="22" t="str">
+        <x:v>MLP Up</x:v>
+      </x:c>
+      <x:c r="C86" s="22" t="n">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="D86" s="22" t="n">
+        <x:v>18944</x:v>
+      </x:c>
+      <x:c r="E86" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F86" s="27"/>
+      <x:c r="G86" s="31"/>
+      <x:c r="H86" s="32"/>
+      <x:c r="I86" s="33"/>
+      <x:c r="J86" s="34" t="str">
+        <x:f>IFERROR(H86/G86,"")</x:f>
+      </x:c>
+      <x:c r="K86" s="34" t="str">
+        <x:f>IFERROR(I86/G86,"")</x:f>
+      </x:c>
+      <x:c r="L86" s="28"/>
+    </x:row>
+    <x:row r="87">
+      <x:c r="A87" s="22" t="str">
+        <x:v>Prefill S=136</x:v>
+      </x:c>
+      <x:c r="B87" s="22" t="str">
+        <x:v>MLP Gate</x:v>
+      </x:c>
+      <x:c r="C87" s="22" t="n">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="D87" s="22" t="n">
+        <x:v>18944</x:v>
+      </x:c>
+      <x:c r="E87" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F87" s="27"/>
+      <x:c r="G87" s="31"/>
+      <x:c r="H87" s="32"/>
+      <x:c r="I87" s="33"/>
+      <x:c r="J87" s="34" t="str">
+        <x:f>IFERROR(H87/G87,"")</x:f>
+      </x:c>
+      <x:c r="K87" s="34" t="str">
+        <x:f>IFERROR(I87/G87,"")</x:f>
+      </x:c>
+      <x:c r="L87" s="28"/>
+    </x:row>
+    <x:row r="88">
+      <x:c r="A88" s="22" t="str">
+        <x:v>Prefill S=136</x:v>
+      </x:c>
+      <x:c r="B88" s="22" t="str">
+        <x:v>MLP Down</x:v>
+      </x:c>
+      <x:c r="C88" s="22" t="n">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="D88" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="E88" s="22" t="n">
+        <x:v>18944</x:v>
+      </x:c>
+      <x:c r="F88" s="27"/>
+      <x:c r="G88" s="31"/>
+      <x:c r="H88" s="32"/>
+      <x:c r="I88" s="33"/>
+      <x:c r="J88" s="34" t="str">
+        <x:f>IFERROR(H88/G88,"")</x:f>
+      </x:c>
+      <x:c r="K88" s="34" t="str">
+        <x:f>IFERROR(I88/G88,"")</x:f>
+      </x:c>
+      <x:c r="L88" s="28"/>
+    </x:row>
+    <x:row r="89">
+      <x:c r="A89" s="22" t="str">
+        <x:v>Prefill S=136</x:v>
+      </x:c>
+      <x:c r="B89" s="22" t="str">
+        <x:v>LM Head</x:v>
+      </x:c>
+      <x:c r="C89" s="22" t="n">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="D89" s="22" t="n">
+        <x:v>152064</x:v>
+      </x:c>
+      <x:c r="E89" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="F89" s="27"/>
+      <x:c r="G89" s="31"/>
+      <x:c r="H89" s="32"/>
+      <x:c r="I89" s="33"/>
+      <x:c r="J89" s="34" t="str">
+        <x:f>IFERROR(H89/G89,"")</x:f>
+      </x:c>
+      <x:c r="K89" s="34" t="str">
+        <x:f>IFERROR(I89/G89,"")</x:f>
+      </x:c>
+      <x:c r="L89" s="28"/>
+    </x:row>
+    <x:row r="90">
+      <x:c r="A90" s="22" t="str">
+        <x:v>Prefill S=136</x:v>
+      </x:c>
+      <x:c r="B90" s="22" t="str">
+        <x:v>Attention QK^T</x:v>
+      </x:c>
+      <x:c r="C90" s="22" t="n">
+        <x:v>3808</x:v>
+      </x:c>
+      <x:c r="D90" s="22" t="n">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="E90" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="F90" s="27"/>
+      <x:c r="G90" s="31"/>
+      <x:c r="H90" s="32"/>
+      <x:c r="I90" s="33"/>
+      <x:c r="J90" s="34" t="str">
+        <x:f>IFERROR(H90/G90,"")</x:f>
+      </x:c>
+      <x:c r="K90" s="34" t="str">
+        <x:f>IFERROR(I90/G90,"")</x:f>
+      </x:c>
+      <x:c r="L90" s="28"/>
+    </x:row>
+    <x:row r="91">
+      <x:c r="A91" s="22" t="str">
+        <x:v>Prefill S=136</x:v>
+      </x:c>
+      <x:c r="B91" s="22" t="str">
+        <x:v>Attention AV</x:v>
+      </x:c>
+      <x:c r="C91" s="22" t="n">
+        <x:v>3808</x:v>
+      </x:c>
+      <x:c r="D91" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="E91" s="22" t="n">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="F91" s="27"/>
+      <x:c r="G91" s="31"/>
+      <x:c r="H91" s="32"/>
+      <x:c r="I91" s="33"/>
+      <x:c r="J91" s="34" t="str">
+        <x:f>IFERROR(H91/G91,"")</x:f>
+      </x:c>
+      <x:c r="K91" s="34" t="str">
+        <x:f>IFERROR(I91/G91,"")</x:f>
+      </x:c>
+      <x:c r="L91" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2669,7 +2949,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7b240889db74ebb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42113330be7e42ad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Deduplicate MLP up and gate benchmark shape
</commit_message>
<xml_diff>
--- a/gemm_performance_comparison.xlsx
+++ b/gemm_performance_comparison.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="环境对比" sheetId="1" r:id="Reccbd279ce0f4dcd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="环境对比" sheetId="1" r:id="Rf8d0c7913aac4c8b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -197,7 +197,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="GemmComparison" displayName="GemmComparison" ref="A5:L91" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="GemmComparison" displayName="GemmComparison" ref="A5:L81" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="阶段/相关长度"/>
     <x:tableColumn id="2" name="来源算子"/>
@@ -481,7 +481,7 @@
     </x:row>
     <x:row r="3" ht="42" customHeight="1">
       <x:c r="A3" s="35" t="str">
-        <x:v>使用方法：Decode 与 Prefill GEMM 通常按 M/N/K 去重；MLP Up 与 MLP Gate 均使用 N=I 并分别执行。L/S=- 表示与长度无关。运行 run_gemm.sh 保存 CUTLASS 日志，再用 collect_gemm_results.py 回填；两类 HGEMM 请按相同 M/N/K 人工筛选。</x:v>
+        <x:v>使用方法：Decode 与 Prefill GEMM 严格按 M/N/K 去重；MLP Up 与 MLP Gate 均使用 N=I，并作为相同 shape 合并统计。L/S=- 表示与长度无关。运行 run_gemm.sh 保存 CUTLASS 日志，再用 collect_gemm_results.py 回填；两类 HGEMM 请按相同 M/N/K 人工筛选。</x:v>
       </x:c>
       <x:c r="B3" s="35"/>
       <x:c r="C3" s="35"/>
@@ -595,7 +595,7 @@
         <x:v>Decode L=-</x:v>
       </x:c>
       <x:c r="B8" s="22" t="str">
-        <x:v>MLP Up</x:v>
+        <x:v>MLP Up / MLP Gate</x:v>
       </x:c>
       <x:c r="C8" s="22" t="n">
         <x:v>1</x:v>
@@ -623,16 +623,16 @@
         <x:v>Decode L=-</x:v>
       </x:c>
       <x:c r="B9" s="22" t="str">
-        <x:v>MLP Gate</x:v>
+        <x:v>MLP Down</x:v>
       </x:c>
       <x:c r="C9" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D9" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="E9" s="22" t="n">
         <x:v>18944</x:v>
-      </x:c>
-      <x:c r="E9" s="22" t="n">
-        <x:v>3584</x:v>
       </x:c>
       <x:c r="F9" s="27"/>
       <x:c r="G9" s="31"/>
@@ -651,16 +651,16 @@
         <x:v>Decode L=-</x:v>
       </x:c>
       <x:c r="B10" s="22" t="str">
-        <x:v>MLP Down</x:v>
+        <x:v>LM Head</x:v>
       </x:c>
       <x:c r="C10" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D10" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>152064</x:v>
       </x:c>
       <x:c r="E10" s="22" t="n">
-        <x:v>18944</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F10" s="27"/>
       <x:c r="G10" s="31"/>
@@ -676,19 +676,19 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="22" t="str">
-        <x:v>Decode L=-</x:v>
+        <x:v>Decode L=128</x:v>
       </x:c>
       <x:c r="B11" s="22" t="str">
-        <x:v>LM Head</x:v>
+        <x:v>Attention QK^T / Attention AV</x:v>
       </x:c>
       <x:c r="C11" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="D11" s="22" t="n">
-        <x:v>152064</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="E11" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="F11" s="27"/>
       <x:c r="G11" s="31"/>
@@ -704,16 +704,16 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="22" t="str">
-        <x:v>Decode L=128</x:v>
+        <x:v>Decode L=256</x:v>
       </x:c>
       <x:c r="B12" s="22" t="str">
-        <x:v>Attention QK^T / Attention AV</x:v>
+        <x:v>Attention QK^T</x:v>
       </x:c>
       <x:c r="C12" s="22" t="n">
         <x:v>28</x:v>
       </x:c>
       <x:c r="D12" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="E12" s="22" t="n">
         <x:v>128</x:v>
@@ -735,16 +735,16 @@
         <x:v>Decode L=256</x:v>
       </x:c>
       <x:c r="B13" s="22" t="str">
-        <x:v>Attention QK^T</x:v>
+        <x:v>Attention AV</x:v>
       </x:c>
       <x:c r="C13" s="22" t="n">
         <x:v>28</x:v>
       </x:c>
       <x:c r="D13" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="E13" s="22" t="n">
         <x:v>256</x:v>
-      </x:c>
-      <x:c r="E13" s="22" t="n">
-        <x:v>128</x:v>
       </x:c>
       <x:c r="F13" s="27"/>
       <x:c r="G13" s="31"/>
@@ -760,19 +760,19 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="22" t="str">
-        <x:v>Decode L=256</x:v>
+        <x:v>Decode L=512</x:v>
       </x:c>
       <x:c r="B14" s="22" t="str">
-        <x:v>Attention AV</x:v>
+        <x:v>Attention QK^T</x:v>
       </x:c>
       <x:c r="C14" s="22" t="n">
         <x:v>28</x:v>
       </x:c>
       <x:c r="D14" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="E14" s="22" t="n">
-        <x:v>256</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="F14" s="27"/>
       <x:c r="G14" s="31"/>
@@ -791,16 +791,16 @@
         <x:v>Decode L=512</x:v>
       </x:c>
       <x:c r="B15" s="22" t="str">
-        <x:v>Attention QK^T</x:v>
+        <x:v>Attention AV</x:v>
       </x:c>
       <x:c r="C15" s="22" t="n">
         <x:v>28</x:v>
       </x:c>
       <x:c r="D15" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="E15" s="22" t="n">
         <x:v>512</x:v>
-      </x:c>
-      <x:c r="E15" s="22" t="n">
-        <x:v>128</x:v>
       </x:c>
       <x:c r="F15" s="27"/>
       <x:c r="G15" s="31"/>
@@ -816,19 +816,19 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="22" t="str">
-        <x:v>Decode L=512</x:v>
+        <x:v>Decode L=1024</x:v>
       </x:c>
       <x:c r="B16" s="22" t="str">
-        <x:v>Attention AV</x:v>
+        <x:v>Attention QK^T</x:v>
       </x:c>
       <x:c r="C16" s="22" t="n">
         <x:v>28</x:v>
       </x:c>
       <x:c r="D16" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>1024</x:v>
       </x:c>
       <x:c r="E16" s="22" t="n">
-        <x:v>512</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="F16" s="27"/>
       <x:c r="G16" s="31"/>
@@ -847,16 +847,16 @@
         <x:v>Decode L=1024</x:v>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>Attention QK^T</x:v>
+        <x:v>Attention AV</x:v>
       </x:c>
       <x:c r="C17" s="22" t="n">
         <x:v>28</x:v>
       </x:c>
       <x:c r="D17" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="E17" s="22" t="n">
         <x:v>1024</x:v>
-      </x:c>
-      <x:c r="E17" s="22" t="n">
-        <x:v>128</x:v>
       </x:c>
       <x:c r="F17" s="27"/>
       <x:c r="G17" s="31"/>
@@ -872,19 +872,19 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="22" t="str">
-        <x:v>Decode L=1024</x:v>
+        <x:v>Decode L=2048</x:v>
       </x:c>
       <x:c r="B18" s="22" t="str">
-        <x:v>Attention AV</x:v>
+        <x:v>Attention QK^T</x:v>
       </x:c>
       <x:c r="C18" s="22" t="n">
         <x:v>28</x:v>
       </x:c>
       <x:c r="D18" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>2048</x:v>
       </x:c>
       <x:c r="E18" s="22" t="n">
-        <x:v>1024</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="F18" s="27"/>
       <x:c r="G18" s="31"/>
@@ -903,16 +903,16 @@
         <x:v>Decode L=2048</x:v>
       </x:c>
       <x:c r="B19" s="22" t="str">
-        <x:v>Attention QK^T</x:v>
+        <x:v>Attention AV</x:v>
       </x:c>
       <x:c r="C19" s="22" t="n">
         <x:v>28</x:v>
       </x:c>
       <x:c r="D19" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="E19" s="22" t="n">
         <x:v>2048</x:v>
-      </x:c>
-      <x:c r="E19" s="22" t="n">
-        <x:v>128</x:v>
       </x:c>
       <x:c r="F19" s="27"/>
       <x:c r="G19" s="31"/>
@@ -928,19 +928,19 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="22" t="str">
-        <x:v>Decode L=2048</x:v>
+        <x:v>Prefill S=128</x:v>
       </x:c>
       <x:c r="B20" s="22" t="str">
-        <x:v>Attention AV</x:v>
+        <x:v>Q / Attention Out</x:v>
       </x:c>
       <x:c r="C20" s="22" t="n">
-        <x:v>28</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="D20" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="E20" s="22" t="n">
-        <x:v>2048</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F20" s="27"/>
       <x:c r="G20" s="31"/>
@@ -959,13 +959,13 @@
         <x:v>Prefill S=128</x:v>
       </x:c>
       <x:c r="B21" s="22" t="str">
-        <x:v>Q / Attention Out</x:v>
+        <x:v>K / V</x:v>
       </x:c>
       <x:c r="C21" s="22" t="n">
         <x:v>128</x:v>
       </x:c>
       <x:c r="D21" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="E21" s="22" t="n">
         <x:v>3584</x:v>
@@ -987,13 +987,13 @@
         <x:v>Prefill S=128</x:v>
       </x:c>
       <x:c r="B22" s="22" t="str">
-        <x:v>K / V</x:v>
+        <x:v>MLP Up / MLP Gate</x:v>
       </x:c>
       <x:c r="C22" s="22" t="n">
         <x:v>128</x:v>
       </x:c>
       <x:c r="D22" s="22" t="n">
-        <x:v>512</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="E22" s="22" t="n">
         <x:v>3584</x:v>
@@ -1015,16 +1015,16 @@
         <x:v>Prefill S=128</x:v>
       </x:c>
       <x:c r="B23" s="22" t="str">
-        <x:v>MLP Up</x:v>
+        <x:v>MLP Down</x:v>
       </x:c>
       <x:c r="C23" s="22" t="n">
         <x:v>128</x:v>
       </x:c>
       <x:c r="D23" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="E23" s="22" t="n">
         <x:v>18944</x:v>
-      </x:c>
-      <x:c r="E23" s="22" t="n">
-        <x:v>3584</x:v>
       </x:c>
       <x:c r="F23" s="27"/>
       <x:c r="G23" s="31"/>
@@ -1043,13 +1043,13 @@
         <x:v>Prefill S=128</x:v>
       </x:c>
       <x:c r="B24" s="22" t="str">
-        <x:v>MLP Gate</x:v>
+        <x:v>LM Head</x:v>
       </x:c>
       <x:c r="C24" s="22" t="n">
         <x:v>128</x:v>
       </x:c>
       <x:c r="D24" s="22" t="n">
-        <x:v>18944</x:v>
+        <x:v>152064</x:v>
       </x:c>
       <x:c r="E24" s="22" t="n">
         <x:v>3584</x:v>
@@ -1071,16 +1071,16 @@
         <x:v>Prefill S=128</x:v>
       </x:c>
       <x:c r="B25" s="22" t="str">
-        <x:v>MLP Down</x:v>
+        <x:v>Attention QK^T / Attention AV</x:v>
       </x:c>
       <x:c r="C25" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="D25" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="E25" s="22" t="n">
-        <x:v>18944</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="F25" s="27"/>
       <x:c r="G25" s="31"/>
@@ -1096,16 +1096,16 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="22" t="str">
-        <x:v>Prefill S=128</x:v>
+        <x:v>Prefill S=256</x:v>
       </x:c>
       <x:c r="B26" s="22" t="str">
-        <x:v>LM Head</x:v>
+        <x:v>Q / Attention Out</x:v>
       </x:c>
       <x:c r="C26" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="D26" s="22" t="n">
-        <x:v>152064</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="E26" s="22" t="n">
         <x:v>3584</x:v>
@@ -1124,19 +1124,19 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="22" t="str">
-        <x:v>Prefill S=128</x:v>
+        <x:v>Prefill S=256</x:v>
       </x:c>
       <x:c r="B27" s="22" t="str">
-        <x:v>Attention QK^T / Attention AV</x:v>
+        <x:v>K / V</x:v>
       </x:c>
       <x:c r="C27" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="D27" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="E27" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F27" s="27"/>
       <x:c r="G27" s="31"/>
@@ -1155,13 +1155,13 @@
         <x:v>Prefill S=256</x:v>
       </x:c>
       <x:c r="B28" s="22" t="str">
-        <x:v>Q / Attention Out</x:v>
+        <x:v>MLP Up / MLP Gate</x:v>
       </x:c>
       <x:c r="C28" s="22" t="n">
         <x:v>256</x:v>
       </x:c>
       <x:c r="D28" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="E28" s="22" t="n">
         <x:v>3584</x:v>
@@ -1183,16 +1183,16 @@
         <x:v>Prefill S=256</x:v>
       </x:c>
       <x:c r="B29" s="22" t="str">
-        <x:v>K / V</x:v>
+        <x:v>MLP Down</x:v>
       </x:c>
       <x:c r="C29" s="22" t="n">
         <x:v>256</x:v>
       </x:c>
       <x:c r="D29" s="22" t="n">
-        <x:v>512</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="E29" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="F29" s="27"/>
       <x:c r="G29" s="31"/>
@@ -1211,13 +1211,13 @@
         <x:v>Prefill S=256</x:v>
       </x:c>
       <x:c r="B30" s="22" t="str">
-        <x:v>MLP Up</x:v>
+        <x:v>LM Head</x:v>
       </x:c>
       <x:c r="C30" s="22" t="n">
         <x:v>256</x:v>
       </x:c>
       <x:c r="D30" s="22" t="n">
-        <x:v>18944</x:v>
+        <x:v>152064</x:v>
       </x:c>
       <x:c r="E30" s="22" t="n">
         <x:v>3584</x:v>
@@ -1239,16 +1239,16 @@
         <x:v>Prefill S=256</x:v>
       </x:c>
       <x:c r="B31" s="22" t="str">
-        <x:v>MLP Gate</x:v>
+        <x:v>Attention QK^T</x:v>
       </x:c>
       <x:c r="C31" s="22" t="n">
+        <x:v>7168</x:v>
+      </x:c>
+      <x:c r="D31" s="22" t="n">
         <x:v>256</x:v>
       </x:c>
-      <x:c r="D31" s="22" t="n">
-        <x:v>18944</x:v>
-      </x:c>
       <x:c r="E31" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="F31" s="27"/>
       <x:c r="G31" s="31"/>
@@ -1267,16 +1267,16 @@
         <x:v>Prefill S=256</x:v>
       </x:c>
       <x:c r="B32" s="22" t="str">
-        <x:v>MLP Down</x:v>
+        <x:v>Attention AV</x:v>
       </x:c>
       <x:c r="C32" s="22" t="n">
+        <x:v>7168</x:v>
+      </x:c>
+      <x:c r="D32" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="E32" s="22" t="n">
         <x:v>256</x:v>
-      </x:c>
-      <x:c r="D32" s="22" t="n">
-        <x:v>3584</x:v>
-      </x:c>
-      <x:c r="E32" s="22" t="n">
-        <x:v>18944</x:v>
       </x:c>
       <x:c r="F32" s="27"/>
       <x:c r="G32" s="31"/>
@@ -1292,16 +1292,16 @@
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="22" t="str">
-        <x:v>Prefill S=256</x:v>
+        <x:v>Prefill S=512</x:v>
       </x:c>
       <x:c r="B33" s="22" t="str">
-        <x:v>LM Head</x:v>
+        <x:v>Q / Attention Out</x:v>
       </x:c>
       <x:c r="C33" s="22" t="n">
-        <x:v>256</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="D33" s="22" t="n">
-        <x:v>152064</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="E33" s="22" t="n">
         <x:v>3584</x:v>
@@ -1320,19 +1320,19 @@
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="22" t="str">
-        <x:v>Prefill S=256</x:v>
+        <x:v>Prefill S=512</x:v>
       </x:c>
       <x:c r="B34" s="22" t="str">
-        <x:v>Attention QK^T</x:v>
+        <x:v>K / V</x:v>
       </x:c>
       <x:c r="C34" s="22" t="n">
-        <x:v>7168</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="D34" s="22" t="n">
-        <x:v>256</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="E34" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F34" s="27"/>
       <x:c r="G34" s="31"/>
@@ -1348,19 +1348,19 @@
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="22" t="str">
-        <x:v>Prefill S=256</x:v>
+        <x:v>Prefill S=512</x:v>
       </x:c>
       <x:c r="B35" s="22" t="str">
-        <x:v>Attention AV</x:v>
+        <x:v>MLP Up / MLP Gate</x:v>
       </x:c>
       <x:c r="C35" s="22" t="n">
-        <x:v>7168</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="D35" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="E35" s="22" t="n">
-        <x:v>256</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F35" s="27"/>
       <x:c r="G35" s="31"/>
@@ -1379,7 +1379,7 @@
         <x:v>Prefill S=512</x:v>
       </x:c>
       <x:c r="B36" s="22" t="str">
-        <x:v>Q / Attention Out</x:v>
+        <x:v>MLP Down</x:v>
       </x:c>
       <x:c r="C36" s="22" t="n">
         <x:v>512</x:v>
@@ -1388,7 +1388,7 @@
         <x:v>3584</x:v>
       </x:c>
       <x:c r="E36" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="F36" s="27"/>
       <x:c r="G36" s="31"/>
@@ -1407,13 +1407,13 @@
         <x:v>Prefill S=512</x:v>
       </x:c>
       <x:c r="B37" s="22" t="str">
-        <x:v>K / V</x:v>
+        <x:v>LM Head</x:v>
       </x:c>
       <x:c r="C37" s="22" t="n">
         <x:v>512</x:v>
       </x:c>
       <x:c r="D37" s="22" t="n">
-        <x:v>512</x:v>
+        <x:v>152064</x:v>
       </x:c>
       <x:c r="E37" s="22" t="n">
         <x:v>3584</x:v>
@@ -1435,16 +1435,16 @@
         <x:v>Prefill S=512</x:v>
       </x:c>
       <x:c r="B38" s="22" t="str">
-        <x:v>MLP Up</x:v>
+        <x:v>Attention QK^T</x:v>
       </x:c>
       <x:c r="C38" s="22" t="n">
+        <x:v>14336</x:v>
+      </x:c>
+      <x:c r="D38" s="22" t="n">
         <x:v>512</x:v>
       </x:c>
-      <x:c r="D38" s="22" t="n">
-        <x:v>18944</x:v>
-      </x:c>
       <x:c r="E38" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="F38" s="27"/>
       <x:c r="G38" s="31"/>
@@ -1463,16 +1463,16 @@
         <x:v>Prefill S=512</x:v>
       </x:c>
       <x:c r="B39" s="22" t="str">
-        <x:v>MLP Gate</x:v>
+        <x:v>Attention AV</x:v>
       </x:c>
       <x:c r="C39" s="22" t="n">
+        <x:v>14336</x:v>
+      </x:c>
+      <x:c r="D39" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="E39" s="22" t="n">
         <x:v>512</x:v>
-      </x:c>
-      <x:c r="D39" s="22" t="n">
-        <x:v>18944</x:v>
-      </x:c>
-      <x:c r="E39" s="22" t="n">
-        <x:v>3584</x:v>
       </x:c>
       <x:c r="F39" s="27"/>
       <x:c r="G39" s="31"/>
@@ -1488,19 +1488,19 @@
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="22" t="str">
-        <x:v>Prefill S=512</x:v>
+        <x:v>Prefill S=1024</x:v>
       </x:c>
       <x:c r="B40" s="22" t="str">
-        <x:v>MLP Down</x:v>
+        <x:v>Q / Attention Out</x:v>
       </x:c>
       <x:c r="C40" s="22" t="n">
-        <x:v>512</x:v>
+        <x:v>1024</x:v>
       </x:c>
       <x:c r="D40" s="22" t="n">
         <x:v>3584</x:v>
       </x:c>
       <x:c r="E40" s="22" t="n">
-        <x:v>18944</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F40" s="27"/>
       <x:c r="G40" s="31"/>
@@ -1516,16 +1516,16 @@
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="22" t="str">
-        <x:v>Prefill S=512</x:v>
+        <x:v>Prefill S=1024</x:v>
       </x:c>
       <x:c r="B41" s="22" t="str">
-        <x:v>LM Head</x:v>
+        <x:v>K / V</x:v>
       </x:c>
       <x:c r="C41" s="22" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="D41" s="22" t="n">
         <x:v>512</x:v>
-      </x:c>
-      <x:c r="D41" s="22" t="n">
-        <x:v>152064</x:v>
       </x:c>
       <x:c r="E41" s="22" t="n">
         <x:v>3584</x:v>
@@ -1544,19 +1544,19 @@
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="22" t="str">
-        <x:v>Prefill S=512</x:v>
+        <x:v>Prefill S=1024</x:v>
       </x:c>
       <x:c r="B42" s="22" t="str">
-        <x:v>Attention QK^T</x:v>
+        <x:v>MLP Up / MLP Gate</x:v>
       </x:c>
       <x:c r="C42" s="22" t="n">
-        <x:v>14336</x:v>
+        <x:v>1024</x:v>
       </x:c>
       <x:c r="D42" s="22" t="n">
-        <x:v>512</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="E42" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F42" s="27"/>
       <x:c r="G42" s="31"/>
@@ -1572,19 +1572,19 @@
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="22" t="str">
-        <x:v>Prefill S=512</x:v>
+        <x:v>Prefill S=1024</x:v>
       </x:c>
       <x:c r="B43" s="22" t="str">
-        <x:v>Attention AV</x:v>
+        <x:v>MLP Down</x:v>
       </x:c>
       <x:c r="C43" s="22" t="n">
-        <x:v>14336</x:v>
+        <x:v>1024</x:v>
       </x:c>
       <x:c r="D43" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="E43" s="22" t="n">
-        <x:v>512</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="F43" s="27"/>
       <x:c r="G43" s="31"/>
@@ -1603,13 +1603,13 @@
         <x:v>Prefill S=1024</x:v>
       </x:c>
       <x:c r="B44" s="22" t="str">
-        <x:v>Q / Attention Out</x:v>
+        <x:v>LM Head</x:v>
       </x:c>
       <x:c r="C44" s="22" t="n">
         <x:v>1024</x:v>
       </x:c>
       <x:c r="D44" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>152064</x:v>
       </x:c>
       <x:c r="E44" s="22" t="n">
         <x:v>3584</x:v>
@@ -1631,16 +1631,16 @@
         <x:v>Prefill S=1024</x:v>
       </x:c>
       <x:c r="B45" s="22" t="str">
-        <x:v>K / V</x:v>
+        <x:v>Attention QK^T</x:v>
       </x:c>
       <x:c r="C45" s="22" t="n">
+        <x:v>28672</x:v>
+      </x:c>
+      <x:c r="D45" s="22" t="n">
         <x:v>1024</x:v>
       </x:c>
-      <x:c r="D45" s="22" t="n">
-        <x:v>512</x:v>
-      </x:c>
       <x:c r="E45" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="F45" s="27"/>
       <x:c r="G45" s="31"/>
@@ -1659,16 +1659,16 @@
         <x:v>Prefill S=1024</x:v>
       </x:c>
       <x:c r="B46" s="22" t="str">
-        <x:v>MLP Up</x:v>
+        <x:v>Attention AV</x:v>
       </x:c>
       <x:c r="C46" s="22" t="n">
+        <x:v>28672</x:v>
+      </x:c>
+      <x:c r="D46" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="E46" s="22" t="n">
         <x:v>1024</x:v>
-      </x:c>
-      <x:c r="D46" s="22" t="n">
-        <x:v>18944</x:v>
-      </x:c>
-      <x:c r="E46" s="22" t="n">
-        <x:v>3584</x:v>
       </x:c>
       <x:c r="F46" s="27"/>
       <x:c r="G46" s="31"/>
@@ -1684,16 +1684,16 @@
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="22" t="str">
-        <x:v>Prefill S=1024</x:v>
+        <x:v>Prefill S=2048</x:v>
       </x:c>
       <x:c r="B47" s="22" t="str">
-        <x:v>MLP Gate</x:v>
+        <x:v>Q / Attention Out</x:v>
       </x:c>
       <x:c r="C47" s="22" t="n">
-        <x:v>1024</x:v>
+        <x:v>2048</x:v>
       </x:c>
       <x:c r="D47" s="22" t="n">
-        <x:v>18944</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="E47" s="22" t="n">
         <x:v>3584</x:v>
@@ -1712,19 +1712,19 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="22" t="str">
-        <x:v>Prefill S=1024</x:v>
+        <x:v>Prefill S=2048</x:v>
       </x:c>
       <x:c r="B48" s="22" t="str">
-        <x:v>MLP Down</x:v>
+        <x:v>K / V</x:v>
       </x:c>
       <x:c r="C48" s="22" t="n">
-        <x:v>1024</x:v>
+        <x:v>2048</x:v>
       </x:c>
       <x:c r="D48" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="E48" s="22" t="n">
-        <x:v>18944</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F48" s="27"/>
       <x:c r="G48" s="31"/>
@@ -1740,16 +1740,16 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="22" t="str">
-        <x:v>Prefill S=1024</x:v>
+        <x:v>Prefill S=2048</x:v>
       </x:c>
       <x:c r="B49" s="22" t="str">
-        <x:v>LM Head</x:v>
+        <x:v>MLP Up / MLP Gate</x:v>
       </x:c>
       <x:c r="C49" s="22" t="n">
-        <x:v>1024</x:v>
+        <x:v>2048</x:v>
       </x:c>
       <x:c r="D49" s="22" t="n">
-        <x:v>152064</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="E49" s="22" t="n">
         <x:v>3584</x:v>
@@ -1768,19 +1768,19 @@
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="22" t="str">
-        <x:v>Prefill S=1024</x:v>
+        <x:v>Prefill S=2048</x:v>
       </x:c>
       <x:c r="B50" s="22" t="str">
-        <x:v>Attention QK^T</x:v>
+        <x:v>MLP Down</x:v>
       </x:c>
       <x:c r="C50" s="22" t="n">
-        <x:v>28672</x:v>
+        <x:v>2048</x:v>
       </x:c>
       <x:c r="D50" s="22" t="n">
-        <x:v>1024</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="E50" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="F50" s="27"/>
       <x:c r="G50" s="31"/>
@@ -1796,19 +1796,19 @@
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="22" t="str">
-        <x:v>Prefill S=1024</x:v>
+        <x:v>Prefill S=2048</x:v>
       </x:c>
       <x:c r="B51" s="22" t="str">
-        <x:v>Attention AV</x:v>
+        <x:v>LM Head</x:v>
       </x:c>
       <x:c r="C51" s="22" t="n">
-        <x:v>28672</x:v>
+        <x:v>2048</x:v>
       </x:c>
       <x:c r="D51" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>152064</x:v>
       </x:c>
       <x:c r="E51" s="22" t="n">
-        <x:v>1024</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F51" s="27"/>
       <x:c r="G51" s="31"/>
@@ -1827,16 +1827,16 @@
         <x:v>Prefill S=2048</x:v>
       </x:c>
       <x:c r="B52" s="22" t="str">
-        <x:v>Q / Attention Out</x:v>
+        <x:v>Attention QK^T</x:v>
       </x:c>
       <x:c r="C52" s="22" t="n">
+        <x:v>57344</x:v>
+      </x:c>
+      <x:c r="D52" s="22" t="n">
         <x:v>2048</x:v>
       </x:c>
-      <x:c r="D52" s="22" t="n">
-        <x:v>3584</x:v>
-      </x:c>
       <x:c r="E52" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="F52" s="27"/>
       <x:c r="G52" s="31"/>
@@ -1855,16 +1855,16 @@
         <x:v>Prefill S=2048</x:v>
       </x:c>
       <x:c r="B53" s="22" t="str">
-        <x:v>K / V</x:v>
+        <x:v>Attention AV</x:v>
       </x:c>
       <x:c r="C53" s="22" t="n">
+        <x:v>57344</x:v>
+      </x:c>
+      <x:c r="D53" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="E53" s="22" t="n">
         <x:v>2048</x:v>
-      </x:c>
-      <x:c r="D53" s="22" t="n">
-        <x:v>512</x:v>
-      </x:c>
-      <x:c r="E53" s="22" t="n">
-        <x:v>3584</x:v>
       </x:c>
       <x:c r="F53" s="27"/>
       <x:c r="G53" s="31"/>
@@ -1880,16 +1880,16 @@
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="22" t="str">
-        <x:v>Prefill S=2048</x:v>
+        <x:v>Prefill S=129</x:v>
       </x:c>
       <x:c r="B54" s="22" t="str">
-        <x:v>MLP Up</x:v>
+        <x:v>Q / Attention Out</x:v>
       </x:c>
       <x:c r="C54" s="22" t="n">
-        <x:v>2048</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="D54" s="22" t="n">
-        <x:v>18944</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="E54" s="22" t="n">
         <x:v>3584</x:v>
@@ -1908,16 +1908,16 @@
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="22" t="str">
-        <x:v>Prefill S=2048</x:v>
+        <x:v>Prefill S=129</x:v>
       </x:c>
       <x:c r="B55" s="22" t="str">
-        <x:v>MLP Gate</x:v>
+        <x:v>K / V</x:v>
       </x:c>
       <x:c r="C55" s="22" t="n">
-        <x:v>2048</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="D55" s="22" t="n">
-        <x:v>18944</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="E55" s="22" t="n">
         <x:v>3584</x:v>
@@ -1936,19 +1936,19 @@
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="22" t="str">
-        <x:v>Prefill S=2048</x:v>
+        <x:v>Prefill S=129</x:v>
       </x:c>
       <x:c r="B56" s="22" t="str">
-        <x:v>MLP Down</x:v>
+        <x:v>MLP Up / MLP Gate</x:v>
       </x:c>
       <x:c r="C56" s="22" t="n">
-        <x:v>2048</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="D56" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="E56" s="22" t="n">
-        <x:v>18944</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F56" s="27"/>
       <x:c r="G56" s="31"/>
@@ -1964,19 +1964,19 @@
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="22" t="str">
-        <x:v>Prefill S=2048</x:v>
+        <x:v>Prefill S=129</x:v>
       </x:c>
       <x:c r="B57" s="22" t="str">
-        <x:v>LM Head</x:v>
+        <x:v>MLP Down</x:v>
       </x:c>
       <x:c r="C57" s="22" t="n">
-        <x:v>2048</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="D57" s="22" t="n">
-        <x:v>152064</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="E57" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="F57" s="27"/>
       <x:c r="G57" s="31"/>
@@ -1992,19 +1992,19 @@
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="22" t="str">
-        <x:v>Prefill S=2048</x:v>
+        <x:v>Prefill S=129</x:v>
       </x:c>
       <x:c r="B58" s="22" t="str">
-        <x:v>Attention QK^T</x:v>
+        <x:v>LM Head</x:v>
       </x:c>
       <x:c r="C58" s="22" t="n">
-        <x:v>57344</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="D58" s="22" t="n">
-        <x:v>2048</x:v>
+        <x:v>152064</x:v>
       </x:c>
       <x:c r="E58" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F58" s="27"/>
       <x:c r="G58" s="31"/>
@@ -2020,19 +2020,19 @@
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="22" t="str">
-        <x:v>Prefill S=2048</x:v>
+        <x:v>Prefill S=129</x:v>
       </x:c>
       <x:c r="B59" s="22" t="str">
-        <x:v>Attention AV</x:v>
+        <x:v>Attention QK^T</x:v>
       </x:c>
       <x:c r="C59" s="22" t="n">
-        <x:v>57344</x:v>
+        <x:v>3612</x:v>
       </x:c>
       <x:c r="D59" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="E59" s="22" t="n">
-        <x:v>2048</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="F59" s="27"/>
       <x:c r="G59" s="31"/>
@@ -2051,16 +2051,16 @@
         <x:v>Prefill S=129</x:v>
       </x:c>
       <x:c r="B60" s="22" t="str">
-        <x:v>Q / Attention Out</x:v>
+        <x:v>Attention AV</x:v>
       </x:c>
       <x:c r="C60" s="22" t="n">
+        <x:v>3612</x:v>
+      </x:c>
+      <x:c r="D60" s="22" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="E60" s="22" t="n">
         <x:v>129</x:v>
-      </x:c>
-      <x:c r="D60" s="22" t="n">
-        <x:v>3584</x:v>
-      </x:c>
-      <x:c r="E60" s="22" t="n">
-        <x:v>3584</x:v>
       </x:c>
       <x:c r="F60" s="27"/>
       <x:c r="G60" s="31"/>
@@ -2076,16 +2076,16 @@
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="22" t="str">
-        <x:v>Prefill S=129</x:v>
+        <x:v>Prefill S=130</x:v>
       </x:c>
       <x:c r="B61" s="22" t="str">
-        <x:v>K / V</x:v>
+        <x:v>Q / Attention Out</x:v>
       </x:c>
       <x:c r="C61" s="22" t="n">
-        <x:v>129</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="D61" s="22" t="n">
-        <x:v>512</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="E61" s="22" t="n">
         <x:v>3584</x:v>
@@ -2104,16 +2104,16 @@
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="22" t="str">
-        <x:v>Prefill S=129</x:v>
+        <x:v>Prefill S=130</x:v>
       </x:c>
       <x:c r="B62" s="22" t="str">
-        <x:v>MLP Up</x:v>
+        <x:v>K / V</x:v>
       </x:c>
       <x:c r="C62" s="22" t="n">
-        <x:v>129</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="D62" s="22" t="n">
-        <x:v>18944</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="E62" s="22" t="n">
         <x:v>3584</x:v>
@@ -2132,13 +2132,13 @@
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="22" t="str">
-        <x:v>Prefill S=129</x:v>
+        <x:v>Prefill S=130</x:v>
       </x:c>
       <x:c r="B63" s="22" t="str">
-        <x:v>MLP Gate</x:v>
+        <x:v>MLP Up / MLP Gate</x:v>
       </x:c>
       <x:c r="C63" s="22" t="n">
-        <x:v>129</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="D63" s="22" t="n">
         <x:v>18944</x:v>
@@ -2160,13 +2160,13 @@
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="22" t="str">
-        <x:v>Prefill S=129</x:v>
+        <x:v>Prefill S=130</x:v>
       </x:c>
       <x:c r="B64" s="22" t="str">
         <x:v>MLP Down</x:v>
       </x:c>
       <x:c r="C64" s="22" t="n">
-        <x:v>129</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="D64" s="22" t="n">
         <x:v>3584</x:v>
@@ -2188,13 +2188,13 @@
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="22" t="str">
-        <x:v>Prefill S=129</x:v>
+        <x:v>Prefill S=130</x:v>
       </x:c>
       <x:c r="B65" s="22" t="str">
         <x:v>LM Head</x:v>
       </x:c>
       <x:c r="C65" s="22" t="n">
-        <x:v>129</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="D65" s="22" t="n">
         <x:v>152064</x:v>
@@ -2216,16 +2216,16 @@
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="22" t="str">
-        <x:v>Prefill S=129</x:v>
+        <x:v>Prefill S=130</x:v>
       </x:c>
       <x:c r="B66" s="22" t="str">
         <x:v>Attention QK^T</x:v>
       </x:c>
       <x:c r="C66" s="22" t="n">
-        <x:v>3612</x:v>
+        <x:v>3640</x:v>
       </x:c>
       <x:c r="D66" s="22" t="n">
-        <x:v>129</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="E66" s="22" t="n">
         <x:v>128</x:v>
@@ -2244,19 +2244,19 @@
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="22" t="str">
-        <x:v>Prefill S=129</x:v>
+        <x:v>Prefill S=130</x:v>
       </x:c>
       <x:c r="B67" s="22" t="str">
         <x:v>Attention AV</x:v>
       </x:c>
       <x:c r="C67" s="22" t="n">
-        <x:v>3612</x:v>
+        <x:v>3640</x:v>
       </x:c>
       <x:c r="D67" s="22" t="n">
         <x:v>128</x:v>
       </x:c>
       <x:c r="E67" s="22" t="n">
-        <x:v>129</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="F67" s="27"/>
       <x:c r="G67" s="31"/>
@@ -2272,13 +2272,13 @@
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="22" t="str">
-        <x:v>Prefill S=130</x:v>
+        <x:v>Prefill S=132</x:v>
       </x:c>
       <x:c r="B68" s="22" t="str">
         <x:v>Q / Attention Out</x:v>
       </x:c>
       <x:c r="C68" s="22" t="n">
-        <x:v>130</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="D68" s="22" t="n">
         <x:v>3584</x:v>
@@ -2300,13 +2300,13 @@
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="22" t="str">
-        <x:v>Prefill S=130</x:v>
+        <x:v>Prefill S=132</x:v>
       </x:c>
       <x:c r="B69" s="22" t="str">
         <x:v>K / V</x:v>
       </x:c>
       <x:c r="C69" s="22" t="n">
-        <x:v>130</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="D69" s="22" t="n">
         <x:v>512</x:v>
@@ -2328,13 +2328,13 @@
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="22" t="str">
-        <x:v>Prefill S=130</x:v>
+        <x:v>Prefill S=132</x:v>
       </x:c>
       <x:c r="B70" s="22" t="str">
-        <x:v>MLP Up</x:v>
+        <x:v>MLP Up / MLP Gate</x:v>
       </x:c>
       <x:c r="C70" s="22" t="n">
-        <x:v>130</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="D70" s="22" t="n">
         <x:v>18944</x:v>
@@ -2356,19 +2356,19 @@
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="22" t="str">
-        <x:v>Prefill S=130</x:v>
+        <x:v>Prefill S=132</x:v>
       </x:c>
       <x:c r="B71" s="22" t="str">
-        <x:v>MLP Gate</x:v>
+        <x:v>MLP Down</x:v>
       </x:c>
       <x:c r="C71" s="22" t="n">
-        <x:v>130</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="D71" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="E71" s="22" t="n">
         <x:v>18944</x:v>
-      </x:c>
-      <x:c r="E71" s="22" t="n">
-        <x:v>3584</x:v>
       </x:c>
       <x:c r="F71" s="27"/>
       <x:c r="G71" s="31"/>
@@ -2384,19 +2384,19 @@
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="22" t="str">
-        <x:v>Prefill S=130</x:v>
+        <x:v>Prefill S=132</x:v>
       </x:c>
       <x:c r="B72" s="22" t="str">
-        <x:v>MLP Down</x:v>
+        <x:v>LM Head</x:v>
       </x:c>
       <x:c r="C72" s="22" t="n">
-        <x:v>130</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="D72" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>152064</x:v>
       </x:c>
       <x:c r="E72" s="22" t="n">
-        <x:v>18944</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F72" s="27"/>
       <x:c r="G72" s="31"/>
@@ -2412,19 +2412,19 @@
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="22" t="str">
-        <x:v>Prefill S=130</x:v>
+        <x:v>Prefill S=132</x:v>
       </x:c>
       <x:c r="B73" s="22" t="str">
-        <x:v>LM Head</x:v>
+        <x:v>Attention QK^T</x:v>
       </x:c>
       <x:c r="C73" s="22" t="n">
-        <x:v>130</x:v>
+        <x:v>3696</x:v>
       </x:c>
       <x:c r="D73" s="22" t="n">
-        <x:v>152064</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="E73" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="F73" s="27"/>
       <x:c r="G73" s="31"/>
@@ -2440,19 +2440,19 @@
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="22" t="str">
-        <x:v>Prefill S=130</x:v>
+        <x:v>Prefill S=132</x:v>
       </x:c>
       <x:c r="B74" s="22" t="str">
-        <x:v>Attention QK^T</x:v>
+        <x:v>Attention AV</x:v>
       </x:c>
       <x:c r="C74" s="22" t="n">
-        <x:v>3640</x:v>
+        <x:v>3696</x:v>
       </x:c>
       <x:c r="D74" s="22" t="n">
-        <x:v>130</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="E74" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="F74" s="27"/>
       <x:c r="G74" s="31"/>
@@ -2468,19 +2468,19 @@
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="22" t="str">
-        <x:v>Prefill S=130</x:v>
+        <x:v>Prefill S=136</x:v>
       </x:c>
       <x:c r="B75" s="22" t="str">
-        <x:v>Attention AV</x:v>
+        <x:v>Q / Attention Out</x:v>
       </x:c>
       <x:c r="C75" s="22" t="n">
-        <x:v>3640</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="D75" s="22" t="n">
-        <x:v>128</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="E75" s="22" t="n">
-        <x:v>130</x:v>
+        <x:v>3584</x:v>
       </x:c>
       <x:c r="F75" s="27"/>
       <x:c r="G75" s="31"/>
@@ -2496,16 +2496,16 @@
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="22" t="str">
-        <x:v>Prefill S=132</x:v>
+        <x:v>Prefill S=136</x:v>
       </x:c>
       <x:c r="B76" s="22" t="str">
-        <x:v>Q / Attention Out</x:v>
+        <x:v>K / V</x:v>
       </x:c>
       <x:c r="C76" s="22" t="n">
-        <x:v>132</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="D76" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="E76" s="22" t="n">
         <x:v>3584</x:v>
@@ -2524,16 +2524,16 @@
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="22" t="str">
-        <x:v>Prefill S=132</x:v>
+        <x:v>Prefill S=136</x:v>
       </x:c>
       <x:c r="B77" s="22" t="str">
-        <x:v>K / V</x:v>
+        <x:v>MLP Up / MLP Gate</x:v>
       </x:c>
       <x:c r="C77" s="22" t="n">
-        <x:v>132</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="D77" s="22" t="n">
-        <x:v>512</x:v>
+        <x:v>18944</x:v>
       </x:c>
       <x:c r="E77" s="22" t="n">
         <x:v>3584</x:v>
@@ -2552,19 +2552,19 @@
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="22" t="str">
-        <x:v>Prefill S=132</x:v>
+        <x:v>Prefill S=136</x:v>
       </x:c>
       <x:c r="B78" s="22" t="str">
-        <x:v>MLP Up</x:v>
+        <x:v>MLP Down</x:v>
       </x:c>
       <x:c r="C78" s="22" t="n">
-        <x:v>132</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="D78" s="22" t="n">
+        <x:v>3584</x:v>
+      </x:c>
+      <x:c r="E78" s="22" t="n">
         <x:v>18944</x:v>
-      </x:c>
-      <x:c r="E78" s="22" t="n">
-        <x:v>3584</x:v>
       </x:c>
       <x:c r="F78" s="27"/>
       <x:c r="G78" s="31"/>
@@ -2580,16 +2580,16 @@
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="22" t="str">
-        <x:v>Prefill S=132</x:v>
+        <x:v>Prefill S=136</x:v>
       </x:c>
       <x:c r="B79" s="22" t="str">
-        <x:v>MLP Gate</x:v>
+        <x:v>LM Head</x:v>
       </x:c>
       <x:c r="C79" s="22" t="n">
-        <x:v>132</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="D79" s="22" t="n">
-        <x:v>18944</x:v>
+        <x:v>152064</x:v>
       </x:c>
       <x:c r="E79" s="22" t="n">
         <x:v>3584</x:v>
@@ -2608,19 +2608,19 @@
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="22" t="str">
-        <x:v>Prefill S=132</x:v>
+        <x:v>Prefill S=136</x:v>
       </x:c>
       <x:c r="B80" s="22" t="str">
-        <x:v>MLP Down</x:v>
+        <x:v>Attention QK^T</x:v>
       </x:c>
       <x:c r="C80" s="22" t="n">
-        <x:v>132</x:v>
+        <x:v>3808</x:v>
       </x:c>
       <x:c r="D80" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="E80" s="22" t="n">
-        <x:v>18944</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="F80" s="27"/>
       <x:c r="G80" s="31"/>
@@ -2636,19 +2636,19 @@
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="22" t="str">
-        <x:v>Prefill S=132</x:v>
+        <x:v>Prefill S=136</x:v>
       </x:c>
       <x:c r="B81" s="22" t="str">
-        <x:v>LM Head</x:v>
+        <x:v>Attention AV</x:v>
       </x:c>
       <x:c r="C81" s="22" t="n">
-        <x:v>132</x:v>
+        <x:v>3808</x:v>
       </x:c>
       <x:c r="D81" s="22" t="n">
-        <x:v>152064</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="E81" s="22" t="n">
-        <x:v>3584</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="F81" s="27"/>
       <x:c r="G81" s="31"/>
@@ -2661,286 +2661,6 @@
         <x:f>IFERROR(I81/G81,"")</x:f>
       </x:c>
       <x:c r="L81" s="28"/>
-    </x:row>
-    <x:row r="82">
-      <x:c r="A82" s="22" t="str">
-        <x:v>Prefill S=132</x:v>
-      </x:c>
-      <x:c r="B82" s="22" t="str">
-        <x:v>Attention QK^T</x:v>
-      </x:c>
-      <x:c r="C82" s="22" t="n">
-        <x:v>3696</x:v>
-      </x:c>
-      <x:c r="D82" s="22" t="n">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="E82" s="22" t="n">
-        <x:v>128</x:v>
-      </x:c>
-      <x:c r="F82" s="27"/>
-      <x:c r="G82" s="31"/>
-      <x:c r="H82" s="32"/>
-      <x:c r="I82" s="33"/>
-      <x:c r="J82" s="34" t="str">
-        <x:f>IFERROR(H82/G82,"")</x:f>
-      </x:c>
-      <x:c r="K82" s="34" t="str">
-        <x:f>IFERROR(I82/G82,"")</x:f>
-      </x:c>
-      <x:c r="L82" s="28"/>
-    </x:row>
-    <x:row r="83">
-      <x:c r="A83" s="22" t="str">
-        <x:v>Prefill S=132</x:v>
-      </x:c>
-      <x:c r="B83" s="22" t="str">
-        <x:v>Attention AV</x:v>
-      </x:c>
-      <x:c r="C83" s="22" t="n">
-        <x:v>3696</x:v>
-      </x:c>
-      <x:c r="D83" s="22" t="n">
-        <x:v>128</x:v>
-      </x:c>
-      <x:c r="E83" s="22" t="n">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="F83" s="27"/>
-      <x:c r="G83" s="31"/>
-      <x:c r="H83" s="32"/>
-      <x:c r="I83" s="33"/>
-      <x:c r="J83" s="34" t="str">
-        <x:f>IFERROR(H83/G83,"")</x:f>
-      </x:c>
-      <x:c r="K83" s="34" t="str">
-        <x:f>IFERROR(I83/G83,"")</x:f>
-      </x:c>
-      <x:c r="L83" s="28"/>
-    </x:row>
-    <x:row r="84">
-      <x:c r="A84" s="22" t="str">
-        <x:v>Prefill S=136</x:v>
-      </x:c>
-      <x:c r="B84" s="22" t="str">
-        <x:v>Q / Attention Out</x:v>
-      </x:c>
-      <x:c r="C84" s="22" t="n">
-        <x:v>136</x:v>
-      </x:c>
-      <x:c r="D84" s="22" t="n">
-        <x:v>3584</x:v>
-      </x:c>
-      <x:c r="E84" s="22" t="n">
-        <x:v>3584</x:v>
-      </x:c>
-      <x:c r="F84" s="27"/>
-      <x:c r="G84" s="31"/>
-      <x:c r="H84" s="32"/>
-      <x:c r="I84" s="33"/>
-      <x:c r="J84" s="34" t="str">
-        <x:f>IFERROR(H84/G84,"")</x:f>
-      </x:c>
-      <x:c r="K84" s="34" t="str">
-        <x:f>IFERROR(I84/G84,"")</x:f>
-      </x:c>
-      <x:c r="L84" s="28"/>
-    </x:row>
-    <x:row r="85">
-      <x:c r="A85" s="22" t="str">
-        <x:v>Prefill S=136</x:v>
-      </x:c>
-      <x:c r="B85" s="22" t="str">
-        <x:v>K / V</x:v>
-      </x:c>
-      <x:c r="C85" s="22" t="n">
-        <x:v>136</x:v>
-      </x:c>
-      <x:c r="D85" s="22" t="n">
-        <x:v>512</x:v>
-      </x:c>
-      <x:c r="E85" s="22" t="n">
-        <x:v>3584</x:v>
-      </x:c>
-      <x:c r="F85" s="27"/>
-      <x:c r="G85" s="31"/>
-      <x:c r="H85" s="32"/>
-      <x:c r="I85" s="33"/>
-      <x:c r="J85" s="34" t="str">
-        <x:f>IFERROR(H85/G85,"")</x:f>
-      </x:c>
-      <x:c r="K85" s="34" t="str">
-        <x:f>IFERROR(I85/G85,"")</x:f>
-      </x:c>
-      <x:c r="L85" s="28"/>
-    </x:row>
-    <x:row r="86">
-      <x:c r="A86" s="22" t="str">
-        <x:v>Prefill S=136</x:v>
-      </x:c>
-      <x:c r="B86" s="22" t="str">
-        <x:v>MLP Up</x:v>
-      </x:c>
-      <x:c r="C86" s="22" t="n">
-        <x:v>136</x:v>
-      </x:c>
-      <x:c r="D86" s="22" t="n">
-        <x:v>18944</x:v>
-      </x:c>
-      <x:c r="E86" s="22" t="n">
-        <x:v>3584</x:v>
-      </x:c>
-      <x:c r="F86" s="27"/>
-      <x:c r="G86" s="31"/>
-      <x:c r="H86" s="32"/>
-      <x:c r="I86" s="33"/>
-      <x:c r="J86" s="34" t="str">
-        <x:f>IFERROR(H86/G86,"")</x:f>
-      </x:c>
-      <x:c r="K86" s="34" t="str">
-        <x:f>IFERROR(I86/G86,"")</x:f>
-      </x:c>
-      <x:c r="L86" s="28"/>
-    </x:row>
-    <x:row r="87">
-      <x:c r="A87" s="22" t="str">
-        <x:v>Prefill S=136</x:v>
-      </x:c>
-      <x:c r="B87" s="22" t="str">
-        <x:v>MLP Gate</x:v>
-      </x:c>
-      <x:c r="C87" s="22" t="n">
-        <x:v>136</x:v>
-      </x:c>
-      <x:c r="D87" s="22" t="n">
-        <x:v>18944</x:v>
-      </x:c>
-      <x:c r="E87" s="22" t="n">
-        <x:v>3584</x:v>
-      </x:c>
-      <x:c r="F87" s="27"/>
-      <x:c r="G87" s="31"/>
-      <x:c r="H87" s="32"/>
-      <x:c r="I87" s="33"/>
-      <x:c r="J87" s="34" t="str">
-        <x:f>IFERROR(H87/G87,"")</x:f>
-      </x:c>
-      <x:c r="K87" s="34" t="str">
-        <x:f>IFERROR(I87/G87,"")</x:f>
-      </x:c>
-      <x:c r="L87" s="28"/>
-    </x:row>
-    <x:row r="88">
-      <x:c r="A88" s="22" t="str">
-        <x:v>Prefill S=136</x:v>
-      </x:c>
-      <x:c r="B88" s="22" t="str">
-        <x:v>MLP Down</x:v>
-      </x:c>
-      <x:c r="C88" s="22" t="n">
-        <x:v>136</x:v>
-      </x:c>
-      <x:c r="D88" s="22" t="n">
-        <x:v>3584</x:v>
-      </x:c>
-      <x:c r="E88" s="22" t="n">
-        <x:v>18944</x:v>
-      </x:c>
-      <x:c r="F88" s="27"/>
-      <x:c r="G88" s="31"/>
-      <x:c r="H88" s="32"/>
-      <x:c r="I88" s="33"/>
-      <x:c r="J88" s="34" t="str">
-        <x:f>IFERROR(H88/G88,"")</x:f>
-      </x:c>
-      <x:c r="K88" s="34" t="str">
-        <x:f>IFERROR(I88/G88,"")</x:f>
-      </x:c>
-      <x:c r="L88" s="28"/>
-    </x:row>
-    <x:row r="89">
-      <x:c r="A89" s="22" t="str">
-        <x:v>Prefill S=136</x:v>
-      </x:c>
-      <x:c r="B89" s="22" t="str">
-        <x:v>LM Head</x:v>
-      </x:c>
-      <x:c r="C89" s="22" t="n">
-        <x:v>136</x:v>
-      </x:c>
-      <x:c r="D89" s="22" t="n">
-        <x:v>152064</x:v>
-      </x:c>
-      <x:c r="E89" s="22" t="n">
-        <x:v>3584</x:v>
-      </x:c>
-      <x:c r="F89" s="27"/>
-      <x:c r="G89" s="31"/>
-      <x:c r="H89" s="32"/>
-      <x:c r="I89" s="33"/>
-      <x:c r="J89" s="34" t="str">
-        <x:f>IFERROR(H89/G89,"")</x:f>
-      </x:c>
-      <x:c r="K89" s="34" t="str">
-        <x:f>IFERROR(I89/G89,"")</x:f>
-      </x:c>
-      <x:c r="L89" s="28"/>
-    </x:row>
-    <x:row r="90">
-      <x:c r="A90" s="22" t="str">
-        <x:v>Prefill S=136</x:v>
-      </x:c>
-      <x:c r="B90" s="22" t="str">
-        <x:v>Attention QK^T</x:v>
-      </x:c>
-      <x:c r="C90" s="22" t="n">
-        <x:v>3808</x:v>
-      </x:c>
-      <x:c r="D90" s="22" t="n">
-        <x:v>136</x:v>
-      </x:c>
-      <x:c r="E90" s="22" t="n">
-        <x:v>128</x:v>
-      </x:c>
-      <x:c r="F90" s="27"/>
-      <x:c r="G90" s="31"/>
-      <x:c r="H90" s="32"/>
-      <x:c r="I90" s="33"/>
-      <x:c r="J90" s="34" t="str">
-        <x:f>IFERROR(H90/G90,"")</x:f>
-      </x:c>
-      <x:c r="K90" s="34" t="str">
-        <x:f>IFERROR(I90/G90,"")</x:f>
-      </x:c>
-      <x:c r="L90" s="28"/>
-    </x:row>
-    <x:row r="91">
-      <x:c r="A91" s="22" t="str">
-        <x:v>Prefill S=136</x:v>
-      </x:c>
-      <x:c r="B91" s="22" t="str">
-        <x:v>Attention AV</x:v>
-      </x:c>
-      <x:c r="C91" s="22" t="n">
-        <x:v>3808</x:v>
-      </x:c>
-      <x:c r="D91" s="22" t="n">
-        <x:v>128</x:v>
-      </x:c>
-      <x:c r="E91" s="22" t="n">
-        <x:v>136</x:v>
-      </x:c>
-      <x:c r="F91" s="27"/>
-      <x:c r="G91" s="31"/>
-      <x:c r="H91" s="32"/>
-      <x:c r="I91" s="33"/>
-      <x:c r="J91" s="34" t="str">
-        <x:f>IFERROR(H91/G91,"")</x:f>
-      </x:c>
-      <x:c r="K91" s="34" t="str">
-        <x:f>IFERROR(I91/G91,"")</x:f>
-      </x:c>
-      <x:c r="L91" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2949,7 +2669,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42113330be7e42ad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf1b2893244a4563"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>